<commit_message>
Atualizando os preços 24/04
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodos.xlsx
+++ b/data/ProdutosFomatodos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\listaDeProdutosB\lista-de-produtos-b\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF26B1DA-46EA-43C1-8D54-6FE737EB8526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F14D8423-DC7B-45B1-ACFC-2A1656BD6568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="630" yWindow="1500" windowWidth="24240" windowHeight="13920" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="promoçoes" sheetId="18" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3530" uniqueCount="1089">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3526" uniqueCount="1089">
   <si>
     <t>produto_grupo</t>
   </si>
@@ -5114,7 +5114,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:G117"/>
+  <dimension ref="A1:G116"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -5766,7 +5766,7 @@
         <v>32</v>
       </c>
       <c r="G28">
-        <v>540</v>
+        <v>595</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -5777,10 +5777,10 @@
         <v>667</v>
       </c>
       <c r="C29">
-        <v>3487</v>
+        <v>4488</v>
       </c>
       <c r="D29">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E29" t="s">
         <v>8</v>
@@ -5789,18 +5789,18 @@
         <v>13</v>
       </c>
       <c r="G29">
-        <v>163</v>
+        <v>299.5</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="B30" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="C30">
-        <v>4488</v>
+        <v>4333</v>
       </c>
       <c r="D30">
         <v>5</v>
@@ -5812,18 +5812,18 @@
         <v>13</v>
       </c>
       <c r="G30">
-        <v>272</v>
+        <v>259.5</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="B31" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="C31">
-        <v>4333</v>
+        <v>4388</v>
       </c>
       <c r="D31">
         <v>5</v>
@@ -5835,18 +5835,18 @@
         <v>13</v>
       </c>
       <c r="G31">
-        <v>259.5</v>
+        <v>145</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="B32" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="C32">
-        <v>4388</v>
+        <v>4389</v>
       </c>
       <c r="D32">
         <v>5</v>
@@ -5858,30 +5858,30 @@
         <v>13</v>
       </c>
       <c r="G32">
-        <v>145</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="B33" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="C33">
-        <v>4389</v>
+        <v>3488</v>
       </c>
       <c r="D33">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E33" t="s">
         <v>8</v>
       </c>
       <c r="F33" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G33">
-        <v>102</v>
+        <v>220</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -5892,33 +5892,33 @@
         <v>675</v>
       </c>
       <c r="C34">
-        <v>3488</v>
+        <v>3400</v>
       </c>
       <c r="D34">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E34" t="s">
         <v>8</v>
       </c>
       <c r="F34" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G34">
-        <v>220</v>
+        <v>57</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="B35" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="C35">
-        <v>3400</v>
+        <v>2257</v>
       </c>
       <c r="D35">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E35" t="s">
         <v>8</v>
@@ -5927,7 +5927,7 @@
         <v>13</v>
       </c>
       <c r="G35">
-        <v>57</v>
+        <v>16</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -5938,53 +5938,53 @@
         <v>677</v>
       </c>
       <c r="C36">
-        <v>2257</v>
+        <v>565</v>
       </c>
       <c r="D36">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="E36" t="s">
         <v>8</v>
       </c>
       <c r="F36" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G36">
-        <v>16</v>
+        <v>123</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="B37" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="C37">
-        <v>565</v>
+        <v>4474</v>
       </c>
       <c r="D37">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="E37" t="s">
         <v>8</v>
       </c>
       <c r="F37" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G37">
-        <v>123</v>
+        <v>39</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="B38" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="C38">
-        <v>4474</v>
+        <v>4473</v>
       </c>
       <c r="D38">
         <v>3</v>
@@ -6001,13 +6001,13 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="B39" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="C39">
-        <v>4473</v>
+        <v>2658</v>
       </c>
       <c r="D39">
         <v>3</v>
@@ -6024,13 +6024,13 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="B40" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="C40">
-        <v>2658</v>
+        <v>2657</v>
       </c>
       <c r="D40">
         <v>3</v>
@@ -6047,16 +6047,16 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="B41" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="C41">
         <v>2657</v>
       </c>
       <c r="D41">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E41" t="s">
         <v>8</v>
@@ -6065,18 +6065,18 @@
         <v>13</v>
       </c>
       <c r="G41">
-        <v>39</v>
+        <v>65</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>686</v>
+        <v>682</v>
       </c>
       <c r="B42" t="s">
-        <v>687</v>
+        <v>683</v>
       </c>
       <c r="C42">
-        <v>2657</v>
+        <v>2658</v>
       </c>
       <c r="D42">
         <v>5</v>
@@ -6093,48 +6093,48 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="B43" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="C43">
-        <v>2658</v>
+        <v>3537</v>
       </c>
       <c r="D43">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>8</v>
+        <v>1057</v>
       </c>
       <c r="F43" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G43">
-        <v>65</v>
+        <v>162</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="B44" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="C44">
-        <v>3537</v>
+        <v>2732</v>
       </c>
       <c r="D44">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E44" t="s">
-        <v>1057</v>
+        <v>8</v>
       </c>
       <c r="F44" t="s">
         <v>9</v>
       </c>
       <c r="G44">
-        <v>162</v>
+        <v>189</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
@@ -6145,42 +6145,42 @@
         <v>691</v>
       </c>
       <c r="C45">
-        <v>2732</v>
+        <v>2733</v>
       </c>
       <c r="D45">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E45" t="s">
         <v>8</v>
       </c>
       <c r="F45" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G45">
-        <v>175</v>
+        <v>96.5</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="B46" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="C46">
-        <v>2733</v>
+        <v>2584</v>
       </c>
       <c r="D46">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E46" t="s">
         <v>8</v>
       </c>
       <c r="F46" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G46">
-        <v>87.5</v>
+        <v>223</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
@@ -6191,42 +6191,42 @@
         <v>693</v>
       </c>
       <c r="C47">
-        <v>2584</v>
+        <v>2677</v>
       </c>
       <c r="D47">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E47" t="s">
         <v>8</v>
       </c>
       <c r="F47" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G47">
-        <v>205</v>
+        <v>113.5</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="B48" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="C48">
-        <v>2677</v>
+        <v>2495</v>
       </c>
       <c r="D48">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E48" t="s">
         <v>8</v>
       </c>
       <c r="F48" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G48">
-        <v>104.5</v>
+        <v>220</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -6237,65 +6237,65 @@
         <v>695</v>
       </c>
       <c r="C49">
-        <v>2495</v>
+        <v>2678</v>
       </c>
       <c r="D49">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E49" t="s">
         <v>8</v>
       </c>
       <c r="F49" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G49">
-        <v>197</v>
+        <v>112</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="B50" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="C50">
-        <v>2678</v>
+        <v>4498</v>
       </c>
       <c r="D50">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E50" t="s">
-        <v>8</v>
+        <v>1057</v>
       </c>
       <c r="F50" t="s">
-        <v>13</v>
+        <v>233</v>
       </c>
       <c r="G50">
-        <v>100.5</v>
+        <v>240</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="B51" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="C51">
-        <v>4498</v>
+        <v>4253</v>
       </c>
       <c r="D51">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E51" t="s">
-        <v>1057</v>
+        <v>8</v>
       </c>
       <c r="F51" t="s">
         <v>233</v>
       </c>
       <c r="G51">
-        <v>240</v>
+        <v>112</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
@@ -6306,10 +6306,10 @@
         <v>699</v>
       </c>
       <c r="C52">
-        <v>4253</v>
+        <v>4500</v>
       </c>
       <c r="D52">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E52" t="s">
         <v>8</v>
@@ -6318,7 +6318,7 @@
         <v>233</v>
       </c>
       <c r="G52">
-        <v>112</v>
+        <v>224</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
@@ -6329,19 +6329,19 @@
         <v>699</v>
       </c>
       <c r="C53">
-        <v>4500</v>
+        <v>4249</v>
       </c>
       <c r="D53">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E53" t="s">
-        <v>8</v>
+        <v>1057</v>
       </c>
       <c r="F53" t="s">
         <v>233</v>
       </c>
       <c r="G53">
-        <v>224</v>
+        <v>230</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
@@ -6352,10 +6352,10 @@
         <v>699</v>
       </c>
       <c r="C54">
-        <v>4249</v>
+        <v>3724</v>
       </c>
       <c r="D54">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E54" t="s">
         <v>1057</v>
@@ -6364,99 +6364,99 @@
         <v>233</v>
       </c>
       <c r="G54">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="B55" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="C55">
-        <v>3724</v>
+        <v>3736</v>
       </c>
       <c r="D55">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E55" t="s">
         <v>1057</v>
       </c>
       <c r="F55" t="s">
-        <v>233</v>
+        <v>9</v>
       </c>
       <c r="G55">
-        <v>224</v>
+        <v>162</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B56" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="C56">
-        <v>3736</v>
+        <v>4499</v>
       </c>
       <c r="D56">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E56" t="s">
         <v>1057</v>
       </c>
       <c r="F56" t="s">
-        <v>9</v>
+        <v>233</v>
       </c>
       <c r="G56">
-        <v>162</v>
+        <v>240</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B57" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="C57">
-        <v>4499</v>
+        <v>3536</v>
       </c>
       <c r="D57">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E57" t="s">
         <v>1057</v>
       </c>
       <c r="F57" t="s">
-        <v>233</v>
+        <v>9</v>
       </c>
       <c r="G57">
-        <v>240</v>
+        <v>162</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B58" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="C58">
-        <v>3536</v>
+        <v>2494</v>
       </c>
       <c r="D58">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E58" t="s">
-        <v>1057</v>
+        <v>8</v>
       </c>
       <c r="F58" t="s">
         <v>9</v>
       </c>
       <c r="G58">
-        <v>162</v>
+        <v>188.5</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
@@ -6467,134 +6467,134 @@
         <v>707</v>
       </c>
       <c r="C59">
-        <v>2494</v>
+        <v>2679</v>
       </c>
       <c r="D59">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E59" t="s">
         <v>8</v>
       </c>
       <c r="F59" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G59">
-        <v>170</v>
+        <v>96</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="B60" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="C60">
-        <v>2679</v>
+        <v>4497</v>
       </c>
       <c r="D60">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E60" t="s">
-        <v>8</v>
+        <v>1057</v>
       </c>
       <c r="F60" t="s">
-        <v>13</v>
+        <v>233</v>
       </c>
       <c r="G60">
-        <v>87</v>
+        <v>240</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="B61" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="C61">
-        <v>4497</v>
+        <v>2493</v>
       </c>
       <c r="D61">
         <v>10</v>
       </c>
       <c r="E61" t="s">
-        <v>1057</v>
+        <v>8</v>
       </c>
       <c r="F61" t="s">
-        <v>233</v>
+        <v>9</v>
       </c>
       <c r="G61">
-        <v>240</v>
+        <v>180</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B62" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="C62">
-        <v>2493</v>
+        <v>3535</v>
       </c>
       <c r="D62">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E62" t="s">
-        <v>8</v>
+        <v>1057</v>
       </c>
       <c r="F62" t="s">
         <v>9</v>
       </c>
       <c r="G62">
-        <v>170</v>
+        <v>162</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="B63" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="C63">
-        <v>3535</v>
+        <v>2498</v>
       </c>
       <c r="D63">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E63" t="s">
-        <v>1057</v>
+        <v>8</v>
       </c>
       <c r="F63" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G63">
-        <v>162</v>
+        <v>92</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="B64" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="C64">
-        <v>2498</v>
+        <v>2806</v>
       </c>
       <c r="D64">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E64" t="s">
         <v>8</v>
       </c>
       <c r="F64" t="s">
-        <v>13</v>
+        <v>233</v>
       </c>
       <c r="G64">
-        <v>87</v>
+        <v>472.5</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
@@ -6605,42 +6605,42 @@
         <v>715</v>
       </c>
       <c r="C65">
-        <v>2806</v>
+        <v>2807</v>
       </c>
       <c r="D65">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E65" t="s">
         <v>8</v>
       </c>
       <c r="F65" t="s">
-        <v>233</v>
+        <v>9</v>
       </c>
       <c r="G65">
-        <v>472.5</v>
+        <v>159.5</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="B66" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="C66">
-        <v>2807</v>
+        <v>4556</v>
       </c>
       <c r="D66">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E66" t="s">
         <v>8</v>
       </c>
       <c r="F66" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="G66">
-        <v>159.5</v>
+        <v>900</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
@@ -6651,33 +6651,33 @@
         <v>717</v>
       </c>
       <c r="C67">
-        <v>4556</v>
+        <v>4557</v>
       </c>
       <c r="D67">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E67" t="s">
         <v>8</v>
       </c>
       <c r="F67" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G67">
-        <v>900</v>
+        <v>182</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="B68" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="C68">
-        <v>4557</v>
+        <v>4018</v>
       </c>
       <c r="D68">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E68" t="s">
         <v>8</v>
@@ -6686,7 +6686,7 @@
         <v>13</v>
       </c>
       <c r="G68">
-        <v>182</v>
+        <v>230</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
@@ -6697,10 +6697,10 @@
         <v>719</v>
       </c>
       <c r="C69">
-        <v>4018</v>
+        <v>2652</v>
       </c>
       <c r="D69">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E69" t="s">
         <v>8</v>
@@ -6709,21 +6709,21 @@
         <v>13</v>
       </c>
       <c r="G69">
-        <v>230</v>
+        <v>117</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="B70" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="C70">
-        <v>2652</v>
+        <v>4049</v>
       </c>
       <c r="D70">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E70" t="s">
         <v>8</v>
@@ -6732,7 +6732,7 @@
         <v>13</v>
       </c>
       <c r="G70">
-        <v>117</v>
+        <v>210</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
@@ -6743,10 +6743,10 @@
         <v>721</v>
       </c>
       <c r="C71">
-        <v>4049</v>
+        <v>3737</v>
       </c>
       <c r="D71">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E71" t="s">
         <v>8</v>
@@ -6755,21 +6755,21 @@
         <v>13</v>
       </c>
       <c r="G71">
-        <v>210</v>
+        <v>107</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="B72" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="C72">
-        <v>3737</v>
+        <v>4301</v>
       </c>
       <c r="D72">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E72" t="s">
         <v>8</v>
@@ -6778,21 +6778,21 @@
         <v>13</v>
       </c>
       <c r="G72">
-        <v>107</v>
+        <v>235</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="B73" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="C73">
-        <v>4301</v>
+        <v>4334</v>
       </c>
       <c r="D73">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E73" t="s">
         <v>8</v>
@@ -6801,30 +6801,30 @@
         <v>13</v>
       </c>
       <c r="G73">
-        <v>235</v>
+        <v>376.5</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="B74" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="C74">
-        <v>4334</v>
+        <v>195</v>
       </c>
       <c r="D74">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E74" t="s">
         <v>8</v>
       </c>
       <c r="F74" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G74">
-        <v>376.5</v>
+        <v>255</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
@@ -6835,42 +6835,42 @@
         <v>727</v>
       </c>
       <c r="C75">
-        <v>195</v>
+        <v>54</v>
       </c>
       <c r="D75">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E75" t="s">
         <v>8</v>
       </c>
       <c r="F75" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G75">
-        <v>255</v>
+        <v>53</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="B76" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="C76">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D76">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E76" t="s">
         <v>8</v>
       </c>
       <c r="F76" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G76">
-        <v>53</v>
+        <v>237.5</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
@@ -6881,42 +6881,42 @@
         <v>729</v>
       </c>
       <c r="C77">
-        <v>63</v>
+        <v>2483</v>
       </c>
       <c r="D77">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E77" t="s">
         <v>8</v>
       </c>
       <c r="F77" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G77">
-        <v>237.5</v>
+        <v>49.5</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="B78" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="C78">
-        <v>2483</v>
+        <v>2974</v>
       </c>
       <c r="D78">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E78" t="s">
         <v>8</v>
       </c>
       <c r="F78" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G78">
-        <v>49.5</v>
+        <v>250</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
@@ -6927,33 +6927,33 @@
         <v>731</v>
       </c>
       <c r="C79">
-        <v>2974</v>
+        <v>2831</v>
       </c>
       <c r="D79">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E79" t="s">
         <v>8</v>
       </c>
       <c r="F79" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G79">
-        <v>250</v>
+        <v>127</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B80" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="C80">
-        <v>2831</v>
+        <v>4137</v>
       </c>
       <c r="D80">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E80" t="s">
         <v>8</v>
@@ -6962,18 +6962,18 @@
         <v>13</v>
       </c>
       <c r="G80">
-        <v>127</v>
+        <v>270</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="B81" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="C81">
-        <v>4137</v>
+        <v>4380</v>
       </c>
       <c r="D81">
         <v>3</v>
@@ -6990,16 +6990,16 @@
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="B82" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="C82">
-        <v>4380</v>
+        <v>4566</v>
       </c>
       <c r="D82">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E82" t="s">
         <v>8</v>
@@ -7008,18 +7008,18 @@
         <v>13</v>
       </c>
       <c r="G82">
-        <v>270</v>
+        <v>240</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="B83" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="C83">
-        <v>4566</v>
+        <v>4567</v>
       </c>
       <c r="D83">
         <v>5</v>
@@ -7036,16 +7036,16 @@
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="B84" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="C84">
-        <v>4567</v>
+        <v>4204</v>
       </c>
       <c r="D84">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E84" t="s">
         <v>8</v>
@@ -7054,7 +7054,7 @@
         <v>13</v>
       </c>
       <c r="G84">
-        <v>240</v>
+        <v>145.5</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
@@ -7065,19 +7065,19 @@
         <v>741</v>
       </c>
       <c r="C85">
-        <v>4204</v>
+        <v>4205</v>
       </c>
       <c r="D85">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E85" t="s">
         <v>8</v>
       </c>
       <c r="F85" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G85">
-        <v>145.5</v>
+        <v>360</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
@@ -7088,42 +7088,42 @@
         <v>741</v>
       </c>
       <c r="C86">
-        <v>4205</v>
+        <v>4225</v>
       </c>
       <c r="D86">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E86" t="s">
         <v>8</v>
       </c>
       <c r="F86" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G86">
-        <v>360</v>
+        <v>900</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="B87" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="C87">
-        <v>4225</v>
+        <v>4378</v>
       </c>
       <c r="D87">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E87" t="s">
         <v>8</v>
       </c>
       <c r="F87" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G87">
-        <v>900</v>
+        <v>430</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
@@ -7134,10 +7134,10 @@
         <v>743</v>
       </c>
       <c r="C88">
-        <v>4378</v>
+        <v>4379</v>
       </c>
       <c r="D88">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E88" t="s">
         <v>8</v>
@@ -7146,30 +7146,30 @@
         <v>32</v>
       </c>
       <c r="G88">
-        <v>430</v>
+        <v>43</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="B89" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="C89">
-        <v>4379</v>
+        <v>3524</v>
       </c>
       <c r="D89">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="E89" t="s">
         <v>8</v>
       </c>
       <c r="F89" t="s">
-        <v>32</v>
+        <v>746</v>
       </c>
       <c r="G89">
-        <v>43</v>
+        <v>350</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
@@ -7180,10 +7180,10 @@
         <v>745</v>
       </c>
       <c r="C90">
-        <v>3524</v>
+        <v>3523</v>
       </c>
       <c r="D90">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="E90" t="s">
         <v>8</v>
@@ -7192,30 +7192,30 @@
         <v>746</v>
       </c>
       <c r="G90">
-        <v>350</v>
+        <v>72</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="B91" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
       <c r="C91">
-        <v>3523</v>
+        <v>3521</v>
       </c>
       <c r="D91">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="E91" t="s">
-        <v>8</v>
+        <v>1084</v>
       </c>
       <c r="F91" t="s">
-        <v>746</v>
+        <v>9</v>
       </c>
       <c r="G91">
-        <v>72</v>
+        <v>158</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
@@ -7226,53 +7226,53 @@
         <v>748</v>
       </c>
       <c r="C92">
-        <v>3521</v>
+        <v>3522</v>
       </c>
       <c r="D92">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E92" t="s">
-        <v>1084</v>
+        <v>1075</v>
       </c>
       <c r="F92" t="s">
         <v>9</v>
       </c>
       <c r="G92">
-        <v>158</v>
+        <v>216.5</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="B93" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="C93">
-        <v>3522</v>
+        <v>64</v>
       </c>
       <c r="D93">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E93" t="s">
-        <v>1075</v>
+        <v>1057</v>
       </c>
       <c r="F93" t="s">
         <v>9</v>
       </c>
       <c r="G93">
-        <v>216.5</v>
+        <v>132</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="B94" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="C94">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="D94">
         <v>8</v>
@@ -7289,25 +7289,25 @@
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="B95" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="C95">
-        <v>90</v>
+        <v>3637</v>
       </c>
       <c r="D95">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E95" t="s">
-        <v>1057</v>
+        <v>8</v>
       </c>
       <c r="F95" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="G95">
-        <v>132</v>
+        <v>375</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
@@ -7318,10 +7318,10 @@
         <v>754</v>
       </c>
       <c r="C96">
-        <v>3637</v>
+        <v>2805</v>
       </c>
       <c r="D96">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E96" t="s">
         <v>8</v>
@@ -7330,7 +7330,7 @@
         <v>32</v>
       </c>
       <c r="G96">
-        <v>375</v>
+        <v>150</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
@@ -7341,42 +7341,42 @@
         <v>754</v>
       </c>
       <c r="C97">
-        <v>2805</v>
+        <v>2427</v>
       </c>
       <c r="D97">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E97" t="s">
         <v>8</v>
       </c>
       <c r="F97" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G97">
-        <v>150</v>
+        <v>46</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="B98" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="C98">
-        <v>2427</v>
+        <v>3437</v>
       </c>
       <c r="D98">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E98" t="s">
         <v>8</v>
       </c>
       <c r="F98" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G98">
-        <v>46</v>
+        <v>390</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
@@ -7387,53 +7387,53 @@
         <v>756</v>
       </c>
       <c r="C99">
-        <v>3437</v>
+        <v>3396</v>
       </c>
       <c r="D99">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E99" t="s">
         <v>8</v>
       </c>
       <c r="F99" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G99">
-        <v>390</v>
+        <v>197</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="B100" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="C100">
-        <v>3396</v>
+        <v>3395</v>
       </c>
       <c r="D100">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E100" t="s">
-        <v>8</v>
+        <v>1060</v>
       </c>
       <c r="F100" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G100">
-        <v>197</v>
+        <v>54</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="B101" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="C101">
-        <v>3395</v>
+        <v>3490</v>
       </c>
       <c r="D101">
         <v>12</v>
@@ -7445,41 +7445,41 @@
         <v>9</v>
       </c>
       <c r="G101">
-        <v>54</v>
+        <v>169</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="B102" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C102">
-        <v>3490</v>
+        <v>458</v>
       </c>
       <c r="D102">
         <v>12</v>
       </c>
       <c r="E102" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="F102" t="s">
         <v>9</v>
       </c>
       <c r="G102">
-        <v>169</v>
+        <v>269.5</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="B103" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="C103">
-        <v>458</v>
+        <v>2641</v>
       </c>
       <c r="D103">
         <v>12</v>
@@ -7491,18 +7491,18 @@
         <v>9</v>
       </c>
       <c r="G103">
-        <v>269.5</v>
+        <v>222</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="B104" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="C104">
-        <v>2641</v>
+        <v>4293</v>
       </c>
       <c r="D104">
         <v>12</v>
@@ -7514,30 +7514,30 @@
         <v>9</v>
       </c>
       <c r="G104">
-        <v>222</v>
+        <v>210</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="B105" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="C105">
-        <v>4293</v>
+        <v>2396</v>
       </c>
       <c r="D105">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E105" t="s">
-        <v>1061</v>
+        <v>8</v>
       </c>
       <c r="F105" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="G105">
-        <v>210</v>
+        <v>675</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
@@ -7548,33 +7548,33 @@
         <v>768</v>
       </c>
       <c r="C106">
-        <v>2396</v>
+        <v>2426</v>
       </c>
       <c r="D106">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E106" t="s">
         <v>8</v>
       </c>
       <c r="F106" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G106">
-        <v>675</v>
+        <v>137</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="B107" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="C107">
-        <v>2426</v>
+        <v>4335</v>
       </c>
       <c r="D107">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E107" t="s">
         <v>8</v>
@@ -7583,21 +7583,21 @@
         <v>13</v>
       </c>
       <c r="G107">
-        <v>137</v>
+        <v>424.5</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="B108" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="C108">
-        <v>4335</v>
+        <v>4477</v>
       </c>
       <c r="D108">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E108" t="s">
         <v>8</v>
@@ -7606,18 +7606,18 @@
         <v>13</v>
       </c>
       <c r="G108">
-        <v>424.5</v>
+        <v>244.5</v>
       </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="B109" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="C109">
-        <v>4477</v>
+        <v>4479</v>
       </c>
       <c r="D109">
         <v>5</v>
@@ -7634,13 +7634,13 @@
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="B110" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="C110">
-        <v>4479</v>
+        <v>4478</v>
       </c>
       <c r="D110">
         <v>5</v>
@@ -7657,25 +7657,25 @@
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="B111" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="C111">
-        <v>4478</v>
+        <v>2646</v>
       </c>
       <c r="D111">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E111" t="s">
-        <v>8</v>
+        <v>1062</v>
       </c>
       <c r="F111" t="s">
-        <v>13</v>
+        <v>233</v>
       </c>
       <c r="G111">
-        <v>244.5</v>
+        <v>50.5</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
@@ -7686,19 +7686,19 @@
         <v>778</v>
       </c>
       <c r="C112">
-        <v>2646</v>
+        <v>2645</v>
       </c>
       <c r="D112">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E112" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="F112" t="s">
         <v>233</v>
       </c>
       <c r="G112">
-        <v>50.5</v>
+        <v>78</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
@@ -7709,110 +7709,87 @@
         <v>778</v>
       </c>
       <c r="C113">
-        <v>2645</v>
+        <v>2638</v>
       </c>
       <c r="D113">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E113" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="F113" t="s">
         <v>233</v>
       </c>
       <c r="G113">
-        <v>78</v>
+        <v>65</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
       <c r="B114" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="C114">
-        <v>2638</v>
+        <v>4294</v>
       </c>
       <c r="D114">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E114" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="F114" t="s">
         <v>233</v>
       </c>
       <c r="G114">
-        <v>65</v>
+        <v>150</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="B115" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="C115">
-        <v>4294</v>
+        <v>4314</v>
       </c>
       <c r="D115">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E115" t="s">
-        <v>1065</v>
+        <v>1075</v>
       </c>
       <c r="F115" t="s">
-        <v>233</v>
+        <v>9</v>
       </c>
       <c r="G115">
-        <v>150</v>
+        <v>252</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="B116" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="C116">
-        <v>4314</v>
+        <v>4315</v>
       </c>
       <c r="D116">
         <v>15</v>
       </c>
       <c r="E116" t="s">
-        <v>1075</v>
+        <v>1066</v>
       </c>
       <c r="F116" t="s">
         <v>9</v>
       </c>
       <c r="G116">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>783</v>
-      </c>
-      <c r="B117" t="s">
-        <v>784</v>
-      </c>
-      <c r="C117">
-        <v>4315</v>
-      </c>
-      <c r="D117">
-        <v>15</v>
-      </c>
-      <c r="E117" t="s">
-        <v>1066</v>
-      </c>
-      <c r="F117" t="s">
-        <v>9</v>
-      </c>
-      <c r="G117">
         <v>450</v>
       </c>
     </row>
@@ -20904,7 +20881,7 @@
         <v>32</v>
       </c>
       <c r="G20">
-        <v>500</v>
+        <v>530</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -20927,7 +20904,7 @@
         <v>13</v>
       </c>
       <c r="G21">
-        <v>252</v>
+        <v>267</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Acresentando novos produtos 06/05
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodos.xlsx
+++ b/data/ProdutosFomatodos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\listaDeProdutosB\lista-de-produtos-b\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{327C41BC-5FE6-4316-8AA1-428E209C121D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F46D7A7E-755E-4141-964D-418547CDBC0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="promoçoes" sheetId="18" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3562" uniqueCount="1089">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3590" uniqueCount="1107">
   <si>
     <t>produto_grupo</t>
   </si>
@@ -3304,6 +3304,60 @@
   </si>
   <si>
     <t>CHÁ DE HORTELÃ</t>
+  </si>
+  <si>
+    <t>doce-brigadeiro</t>
+  </si>
+  <si>
+    <t>doce-geleia-de-mocoto</t>
+  </si>
+  <si>
+    <t>doce-palha-italiana</t>
+  </si>
+  <si>
+    <t>doce-pingo-bel</t>
+  </si>
+  <si>
+    <t>doce-de-leite-souvenir</t>
+  </si>
+  <si>
+    <t>doce-de-leite-c-cocosouvenir</t>
+  </si>
+  <si>
+    <t>DOCE DE BRIGADEIRO</t>
+  </si>
+  <si>
+    <t>DOCE GELEIA DE MOCOTO</t>
+  </si>
+  <si>
+    <t>DOCE PALHA ITALIANA</t>
+  </si>
+  <si>
+    <t>DOCE PINGO BEL</t>
+  </si>
+  <si>
+    <t>DOCE DE LEITE SOUVENIR</t>
+  </si>
+  <si>
+    <t>DOCE DE LEITE C/COCOSUVENIR</t>
+  </si>
+  <si>
+    <t>X50G</t>
+  </si>
+  <si>
+    <t>X55G</t>
+  </si>
+  <si>
+    <t>X37,5G</t>
+  </si>
+  <si>
+    <t>X400g</t>
+  </si>
+  <si>
+    <t>doce-de-leite-docura-fazenda</t>
+  </si>
+  <si>
+    <t>DOCE DE LEITE DOÇURA FAZENDA</t>
   </si>
 </sst>
 </file>
@@ -9229,7 +9283,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
-  <dimension ref="A1:G115"/>
+  <dimension ref="A1:G122"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -11220,128 +11274,128 @@
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>987</v>
+        <v>1089</v>
       </c>
       <c r="B87" t="s">
-        <v>988</v>
+        <v>1095</v>
       </c>
       <c r="C87">
-        <v>4104</v>
+        <v>4624</v>
       </c>
       <c r="D87">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E87" t="s">
-        <v>1078</v>
+        <v>1101</v>
       </c>
       <c r="F87" t="s">
-        <v>233</v>
+        <v>13</v>
       </c>
       <c r="G87">
-        <v>77</v>
+        <v>48</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>989</v>
+        <v>1105</v>
       </c>
       <c r="B88" t="s">
-        <v>990</v>
+        <v>1106</v>
       </c>
       <c r="C88">
-        <v>4101</v>
+        <v>4627</v>
       </c>
       <c r="D88">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E88" t="s">
-        <v>1078</v>
+        <v>1102</v>
       </c>
       <c r="F88" t="s">
-        <v>233</v>
+        <v>13</v>
       </c>
       <c r="G88">
-        <v>77</v>
+        <v>60</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>991</v>
+        <v>1090</v>
       </c>
       <c r="B89" t="s">
-        <v>992</v>
+        <v>1096</v>
       </c>
       <c r="C89">
-        <v>4105</v>
+        <v>4628</v>
       </c>
       <c r="D89">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E89" t="s">
-        <v>1078</v>
+        <v>1103</v>
       </c>
       <c r="F89" t="s">
-        <v>233</v>
+        <v>13</v>
       </c>
       <c r="G89">
-        <v>77</v>
+        <v>28</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>993</v>
+        <v>1091</v>
       </c>
       <c r="B90" t="s">
-        <v>994</v>
+        <v>1097</v>
       </c>
       <c r="C90">
-        <v>3705</v>
+        <v>4625</v>
       </c>
       <c r="D90">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E90" t="s">
-        <v>1076</v>
+        <v>1101</v>
       </c>
       <c r="F90" t="s">
-        <v>233</v>
+        <v>13</v>
       </c>
       <c r="G90">
-        <v>123.5</v>
+        <v>48</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>995</v>
+        <v>1092</v>
       </c>
       <c r="B91" t="s">
-        <v>996</v>
+        <v>1098</v>
       </c>
       <c r="C91">
-        <v>3823</v>
+        <v>4626</v>
       </c>
       <c r="D91">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E91" t="s">
-        <v>1078</v>
+        <v>1101</v>
       </c>
       <c r="F91" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G91">
-        <v>77</v>
+        <v>48</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>997</v>
+        <v>1093</v>
       </c>
       <c r="B92" t="s">
-        <v>998</v>
+        <v>1099</v>
       </c>
       <c r="C92">
-        <v>4583</v>
+        <v>4629</v>
       </c>
       <c r="D92">
         <v>12</v>
@@ -11350,366 +11404,366 @@
         <v>1078</v>
       </c>
       <c r="F92" t="s">
-        <v>233</v>
+        <v>9</v>
       </c>
       <c r="G92">
-        <v>144</v>
+        <v>195</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>999</v>
+        <v>1094</v>
       </c>
       <c r="B93" t="s">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="C93">
-        <v>4308</v>
+        <v>4630</v>
       </c>
       <c r="D93">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E93" t="s">
-        <v>1077</v>
+        <v>1104</v>
       </c>
       <c r="F93" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G93">
-        <v>68.5</v>
+        <v>127.5</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>1001</v>
+        <v>987</v>
       </c>
       <c r="B94" t="s">
-        <v>1002</v>
+        <v>988</v>
       </c>
       <c r="C94">
-        <v>4309</v>
+        <v>4104</v>
       </c>
       <c r="D94">
         <v>10</v>
       </c>
       <c r="E94" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="F94" t="s">
-        <v>968</v>
+        <v>233</v>
       </c>
       <c r="G94">
-        <v>68.5</v>
+        <v>77</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>1003</v>
+        <v>989</v>
       </c>
       <c r="B95" t="s">
-        <v>1004</v>
+        <v>990</v>
       </c>
       <c r="C95">
-        <v>4412</v>
+        <v>4101</v>
       </c>
       <c r="D95">
-        <v>2.5</v>
+        <v>10</v>
       </c>
       <c r="E95" t="s">
-        <v>8</v>
+        <v>1078</v>
       </c>
       <c r="F95" t="s">
-        <v>968</v>
+        <v>233</v>
       </c>
       <c r="G95">
-        <v>71.5</v>
+        <v>77</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>1005</v>
+        <v>991</v>
       </c>
       <c r="B96" t="s">
-        <v>1006</v>
+        <v>992</v>
       </c>
       <c r="C96">
-        <v>4413</v>
+        <v>4105</v>
       </c>
       <c r="D96">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E96" t="s">
-        <v>8</v>
+        <v>1078</v>
       </c>
       <c r="F96" t="s">
-        <v>13</v>
+        <v>233</v>
       </c>
       <c r="G96">
-        <v>496</v>
+        <v>77</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>1005</v>
+        <v>993</v>
       </c>
       <c r="B97" t="s">
-        <v>1006</v>
+        <v>994</v>
       </c>
       <c r="C97">
-        <v>4414</v>
+        <v>3705</v>
       </c>
       <c r="D97">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E97" t="s">
-        <v>8</v>
+        <v>1076</v>
       </c>
       <c r="F97" t="s">
-        <v>13</v>
+        <v>233</v>
       </c>
       <c r="G97">
-        <v>101</v>
+        <v>123.5</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>1007</v>
+        <v>995</v>
       </c>
       <c r="B98" t="s">
-        <v>1008</v>
+        <v>996</v>
       </c>
       <c r="C98">
-        <v>4415</v>
+        <v>3823</v>
       </c>
       <c r="D98">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E98" t="s">
-        <v>8</v>
+        <v>1078</v>
       </c>
       <c r="F98" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G98">
-        <v>414</v>
+        <v>77</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>1007</v>
+        <v>997</v>
       </c>
       <c r="B99" t="s">
-        <v>1008</v>
+        <v>998</v>
       </c>
       <c r="C99">
-        <v>4416</v>
+        <v>4583</v>
       </c>
       <c r="D99">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E99" t="s">
-        <v>8</v>
+        <v>1078</v>
       </c>
       <c r="F99" t="s">
-        <v>13</v>
+        <v>233</v>
       </c>
       <c r="G99">
-        <v>85</v>
+        <v>144</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>1009</v>
+        <v>999</v>
       </c>
       <c r="B100" t="s">
-        <v>1010</v>
+        <v>1000</v>
       </c>
       <c r="C100">
-        <v>4475</v>
+        <v>4308</v>
       </c>
       <c r="D100">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E100" t="s">
-        <v>1083</v>
+        <v>1077</v>
       </c>
       <c r="F100" t="s">
         <v>13</v>
       </c>
       <c r="G100">
-        <v>9</v>
+        <v>68.5</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>1011</v>
+        <v>1001</v>
       </c>
       <c r="B101" t="s">
-        <v>1012</v>
+        <v>1002</v>
       </c>
       <c r="C101">
-        <v>4354</v>
+        <v>4309</v>
       </c>
       <c r="D101">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E101" t="s">
-        <v>1083</v>
+        <v>1077</v>
       </c>
       <c r="F101" t="s">
-        <v>744</v>
+        <v>968</v>
       </c>
       <c r="G101">
-        <v>79.5</v>
+        <v>68.5</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>1013</v>
+        <v>1003</v>
       </c>
       <c r="B102" t="s">
-        <v>1014</v>
+        <v>1004</v>
       </c>
       <c r="C102">
-        <v>4445</v>
+        <v>4412</v>
       </c>
       <c r="D102">
-        <v>12</v>
+        <v>2.5</v>
       </c>
       <c r="E102" t="s">
-        <v>1083</v>
+        <v>8</v>
       </c>
       <c r="F102" t="s">
-        <v>9</v>
+        <v>968</v>
       </c>
       <c r="G102">
-        <v>79.5</v>
+        <v>71.5</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>1015</v>
+        <v>1005</v>
       </c>
       <c r="B103" t="s">
-        <v>1016</v>
+        <v>1006</v>
       </c>
       <c r="C103">
-        <v>4353</v>
+        <v>4413</v>
       </c>
       <c r="D103">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E103" t="s">
-        <v>1083</v>
+        <v>8</v>
       </c>
       <c r="F103" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G103">
-        <v>79.5</v>
+        <v>496</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>1017</v>
+        <v>1005</v>
       </c>
       <c r="B104" t="s">
-        <v>1018</v>
+        <v>1006</v>
       </c>
       <c r="C104">
-        <v>4350</v>
+        <v>4414</v>
       </c>
       <c r="D104">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E104" t="s">
-        <v>1083</v>
+        <v>8</v>
       </c>
       <c r="F104" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G104">
-        <v>79.5</v>
+        <v>101</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>1019</v>
+        <v>1007</v>
       </c>
       <c r="B105" t="s">
-        <v>1020</v>
+        <v>1008</v>
       </c>
       <c r="C105">
-        <v>4352</v>
+        <v>4415</v>
       </c>
       <c r="D105">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E105" t="s">
-        <v>1083</v>
+        <v>8</v>
       </c>
       <c r="F105" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G105">
-        <v>79.5</v>
+        <v>414</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>1021</v>
+        <v>1007</v>
       </c>
       <c r="B106" t="s">
-        <v>1022</v>
+        <v>1008</v>
       </c>
       <c r="C106">
-        <v>4349</v>
+        <v>4416</v>
       </c>
       <c r="D106">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E106" t="s">
-        <v>1083</v>
+        <v>8</v>
       </c>
       <c r="F106" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G106">
-        <v>79.5</v>
+        <v>85</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>1023</v>
+        <v>1009</v>
       </c>
       <c r="B107" t="s">
-        <v>1024</v>
+        <v>1010</v>
       </c>
       <c r="C107">
-        <v>4351</v>
+        <v>4475</v>
       </c>
       <c r="D107">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E107" t="s">
         <v>1083</v>
       </c>
       <c r="F107" t="s">
+        <v>13</v>
+      </c>
+      <c r="G107">
         <v>9</v>
-      </c>
-      <c r="G107">
-        <v>79.5</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>1025</v>
+        <v>1011</v>
       </c>
       <c r="B108" t="s">
-        <v>1026</v>
+        <v>1012</v>
       </c>
       <c r="C108">
-        <v>4581</v>
+        <v>4354</v>
       </c>
       <c r="D108">
         <v>12</v>
@@ -11718,7 +11772,7 @@
         <v>1083</v>
       </c>
       <c r="F108" t="s">
-        <v>9</v>
+        <v>744</v>
       </c>
       <c r="G108">
         <v>79.5</v>
@@ -11726,162 +11780,323 @@
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>1027</v>
+        <v>1013</v>
       </c>
       <c r="B109" t="s">
-        <v>1028</v>
+        <v>1014</v>
       </c>
       <c r="C109">
-        <v>4096</v>
+        <v>4445</v>
       </c>
       <c r="D109">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E109" t="s">
-        <v>8</v>
+        <v>1083</v>
       </c>
       <c r="F109" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G109">
-        <v>79</v>
+        <v>79.5</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>1029</v>
+        <v>1015</v>
       </c>
       <c r="B110" t="s">
-        <v>1030</v>
+        <v>1016</v>
       </c>
       <c r="C110">
-        <v>4123</v>
+        <v>4353</v>
       </c>
       <c r="D110">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E110" t="s">
-        <v>1076</v>
+        <v>1083</v>
       </c>
       <c r="F110" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G110">
-        <v>60</v>
+        <v>79.5</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>1031</v>
+        <v>1017</v>
       </c>
       <c r="B111" t="s">
-        <v>1032</v>
+        <v>1018</v>
       </c>
       <c r="C111">
-        <v>4306</v>
+        <v>4350</v>
       </c>
       <c r="D111">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E111" t="s">
-        <v>1078</v>
+        <v>1083</v>
       </c>
       <c r="F111" t="s">
-        <v>968</v>
+        <v>9</v>
       </c>
       <c r="G111">
-        <v>81</v>
+        <v>79.5</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>1033</v>
+        <v>1019</v>
       </c>
       <c r="B112" t="s">
-        <v>1034</v>
+        <v>1020</v>
       </c>
       <c r="C112">
-        <v>4307</v>
+        <v>4352</v>
       </c>
       <c r="D112">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E112" t="s">
-        <v>1078</v>
+        <v>1083</v>
       </c>
       <c r="F112" t="s">
-        <v>968</v>
+        <v>9</v>
       </c>
       <c r="G112">
-        <v>81</v>
+        <v>79.5</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>1035</v>
+        <v>1021</v>
       </c>
       <c r="B113" t="s">
-        <v>1036</v>
+        <v>1022</v>
       </c>
       <c r="C113">
-        <v>2659</v>
+        <v>4349</v>
       </c>
       <c r="D113">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E113" t="s">
-        <v>1079</v>
+        <v>1083</v>
       </c>
       <c r="F113" t="s">
-        <v>233</v>
+        <v>9</v>
       </c>
       <c r="G113">
-        <v>27.5</v>
+        <v>79.5</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>1035</v>
+        <v>1023</v>
       </c>
       <c r="B114" t="s">
-        <v>1036</v>
+        <v>1024</v>
       </c>
       <c r="C114">
-        <v>2621</v>
+        <v>4351</v>
       </c>
       <c r="D114">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E114" t="s">
-        <v>1080</v>
+        <v>1083</v>
       </c>
       <c r="F114" t="s">
-        <v>233</v>
+        <v>9</v>
       </c>
       <c r="G114">
-        <v>24.5</v>
+        <v>79.5</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B115" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C115">
+        <v>4581</v>
+      </c>
+      <c r="D115">
+        <v>12</v>
+      </c>
+      <c r="E115" t="s">
+        <v>1083</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+      <c r="G115">
+        <v>79.5</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B116" t="s">
+        <v>1028</v>
+      </c>
+      <c r="C116">
+        <v>4096</v>
+      </c>
+      <c r="D116">
+        <v>5</v>
+      </c>
+      <c r="E116" t="s">
+        <v>8</v>
+      </c>
+      <c r="F116" t="s">
+        <v>13</v>
+      </c>
+      <c r="G116">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B117" t="s">
+        <v>1030</v>
+      </c>
+      <c r="C117">
+        <v>4123</v>
+      </c>
+      <c r="D117">
+        <v>10</v>
+      </c>
+      <c r="E117" t="s">
+        <v>1076</v>
+      </c>
+      <c r="F117" t="s">
+        <v>13</v>
+      </c>
+      <c r="G117">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>1031</v>
+      </c>
+      <c r="B118" t="s">
+        <v>1032</v>
+      </c>
+      <c r="C118">
+        <v>4306</v>
+      </c>
+      <c r="D118">
+        <v>10</v>
+      </c>
+      <c r="E118" t="s">
+        <v>1078</v>
+      </c>
+      <c r="F118" t="s">
+        <v>968</v>
+      </c>
+      <c r="G118">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B119" t="s">
+        <v>1034</v>
+      </c>
+      <c r="C119">
+        <v>4307</v>
+      </c>
+      <c r="D119">
+        <v>10</v>
+      </c>
+      <c r="E119" t="s">
+        <v>1078</v>
+      </c>
+      <c r="F119" t="s">
+        <v>968</v>
+      </c>
+      <c r="G119">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B120" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C120">
+        <v>2659</v>
+      </c>
+      <c r="D120">
+        <v>20</v>
+      </c>
+      <c r="E120" t="s">
+        <v>1079</v>
+      </c>
+      <c r="F120" t="s">
+        <v>233</v>
+      </c>
+      <c r="G120">
+        <v>27.5</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B121" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C121">
+        <v>2621</v>
+      </c>
+      <c r="D121">
+        <v>5</v>
+      </c>
+      <c r="E121" t="s">
+        <v>1080</v>
+      </c>
+      <c r="F121" t="s">
+        <v>233</v>
+      </c>
+      <c r="G121">
+        <v>24.5</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
         <v>1037</v>
       </c>
-      <c r="B115" t="s">
+      <c r="B122" t="s">
         <v>1038</v>
       </c>
-      <c r="C115">
+      <c r="C122">
         <v>3656</v>
       </c>
-      <c r="D115">
-        <v>5</v>
-      </c>
-      <c r="E115" t="s">
+      <c r="D122">
+        <v>5</v>
+      </c>
+      <c r="E122" t="s">
         <v>1078</v>
       </c>
-      <c r="F115" t="s">
+      <c r="F122" t="s">
         <v>233</v>
       </c>
-      <c r="G115">
+      <c r="G122">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizando imagens erradas 06/05
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodos.xlsx
+++ b/data/ProdutosFomatodos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\listaDeProdutosB\lista-de-produtos-b\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F46D7A7E-755E-4141-964D-418547CDBC0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF9C33E3-851A-44B5-9B12-F5FC2576BA13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2709,18 +2709,6 @@
     <t>BALA GELATINA BEIJO</t>
   </si>
   <si>
-    <t>bala-geatina-cobrinha-citrica</t>
-  </si>
-  <si>
-    <t>BALA GEATINA COBRINHA CITRICA</t>
-  </si>
-  <si>
-    <t>bala-geatina-diversas</t>
-  </si>
-  <si>
-    <t>BALA GEATINA DIVERSAS</t>
-  </si>
-  <si>
     <t>bala-gelatina-mix-formatos</t>
   </si>
   <si>
@@ -3358,6 +3346,18 @@
   </si>
   <si>
     <t>DOCE DE LEITE DOÇURA FAZENDA</t>
+  </si>
+  <si>
+    <t>bala-gelatina-cobrinha-citrica</t>
+  </si>
+  <si>
+    <t>bala-gelatina-diversas</t>
+  </si>
+  <si>
+    <t>BALA GELATINA DIVERSAS</t>
+  </si>
+  <si>
+    <t>BALA GELATINA COBRINHA CITRICA</t>
   </si>
 </sst>
 </file>
@@ -4260,7 +4260,7 @@
         <v>2</v>
       </c>
       <c r="E13" t="s">
-        <v>1057</v>
+        <v>1053</v>
       </c>
       <c r="F13" t="s">
         <v>9</v>
@@ -4306,7 +4306,7 @@
         <v>2</v>
       </c>
       <c r="E15" t="s">
-        <v>1057</v>
+        <v>1053</v>
       </c>
       <c r="F15" t="s">
         <v>13</v>
@@ -4352,7 +4352,7 @@
         <v>2</v>
       </c>
       <c r="E17" t="s">
-        <v>1057</v>
+        <v>1053</v>
       </c>
       <c r="F17" t="s">
         <v>9</v>
@@ -4968,7 +4968,7 @@
         <v>2</v>
       </c>
       <c r="E20" t="s">
-        <v>1057</v>
+        <v>1053</v>
       </c>
       <c r="F20" t="s">
         <v>9</v>
@@ -5469,7 +5469,7 @@
         <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F5" t="s">
         <v>233</v>
@@ -5515,7 +5515,7 @@
         <v>6</v>
       </c>
       <c r="E7" t="s">
-        <v>1056</v>
+        <v>1052</v>
       </c>
       <c r="F7" t="s">
         <v>233</v>
@@ -5538,7 +5538,7 @@
         <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F8" t="s">
         <v>233</v>
@@ -5561,7 +5561,7 @@
         <v>20</v>
       </c>
       <c r="E9" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
       <c r="F9" t="s">
         <v>233</v>
@@ -6343,7 +6343,7 @@
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F43" t="s">
         <v>9</v>
@@ -6504,7 +6504,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F50" t="s">
         <v>233</v>
@@ -6573,7 +6573,7 @@
         <v>20</v>
       </c>
       <c r="E53" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F53" t="s">
         <v>233</v>
@@ -6596,7 +6596,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F54" t="s">
         <v>233</v>
@@ -6619,7 +6619,7 @@
         <v>12</v>
       </c>
       <c r="E55" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F55" t="s">
         <v>9</v>
@@ -6642,7 +6642,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F56" t="s">
         <v>233</v>
@@ -6665,7 +6665,7 @@
         <v>12</v>
       </c>
       <c r="E57" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F57" t="s">
         <v>9</v>
@@ -6734,7 +6734,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F60" t="s">
         <v>233</v>
@@ -6780,7 +6780,7 @@
         <v>12</v>
       </c>
       <c r="E62" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F62" t="s">
         <v>9</v>
@@ -7447,7 +7447,7 @@
         <v>16</v>
       </c>
       <c r="E91" t="s">
-        <v>1082</v>
+        <v>1078</v>
       </c>
       <c r="F91" t="s">
         <v>9</v>
@@ -7470,7 +7470,7 @@
         <v>12</v>
       </c>
       <c r="E92" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
       <c r="F92" t="s">
         <v>9</v>
@@ -7493,7 +7493,7 @@
         <v>8</v>
       </c>
       <c r="E93" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F93" t="s">
         <v>9</v>
@@ -7516,7 +7516,7 @@
         <v>8</v>
       </c>
       <c r="E94" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F94" t="s">
         <v>9</v>
@@ -7654,7 +7654,7 @@
         <v>12</v>
       </c>
       <c r="E100" t="s">
-        <v>1058</v>
+        <v>1054</v>
       </c>
       <c r="F100" t="s">
         <v>9</v>
@@ -7677,7 +7677,7 @@
         <v>12</v>
       </c>
       <c r="E101" t="s">
-        <v>1058</v>
+        <v>1054</v>
       </c>
       <c r="F101" t="s">
         <v>9</v>
@@ -7700,7 +7700,7 @@
         <v>12</v>
       </c>
       <c r="E102" t="s">
-        <v>1059</v>
+        <v>1055</v>
       </c>
       <c r="F102" t="s">
         <v>9</v>
@@ -7723,7 +7723,7 @@
         <v>12</v>
       </c>
       <c r="E103" t="s">
-        <v>1059</v>
+        <v>1055</v>
       </c>
       <c r="F103" t="s">
         <v>9</v>
@@ -7746,7 +7746,7 @@
         <v>12</v>
       </c>
       <c r="E104" t="s">
-        <v>1059</v>
+        <v>1055</v>
       </c>
       <c r="F104" t="s">
         <v>9</v>
@@ -7907,7 +7907,7 @@
         <v>12</v>
       </c>
       <c r="E111" t="s">
-        <v>1060</v>
+        <v>1056</v>
       </c>
       <c r="F111" t="s">
         <v>233</v>
@@ -7930,7 +7930,7 @@
         <v>6</v>
       </c>
       <c r="E112" t="s">
-        <v>1061</v>
+        <v>1057</v>
       </c>
       <c r="F112" t="s">
         <v>233</v>
@@ -7953,7 +7953,7 @@
         <v>9</v>
       </c>
       <c r="E113" t="s">
-        <v>1062</v>
+        <v>1058</v>
       </c>
       <c r="F113" t="s">
         <v>233</v>
@@ -7976,7 +7976,7 @@
         <v>18</v>
       </c>
       <c r="E114" t="s">
-        <v>1063</v>
+        <v>1059</v>
       </c>
       <c r="F114" t="s">
         <v>233</v>
@@ -7999,7 +7999,7 @@
         <v>15</v>
       </c>
       <c r="E115" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
       <c r="F115" t="s">
         <v>9</v>
@@ -8022,7 +8022,7 @@
         <v>15</v>
       </c>
       <c r="E116" t="s">
-        <v>1064</v>
+        <v>1060</v>
       </c>
       <c r="F116" t="s">
         <v>9</v>
@@ -8086,7 +8086,7 @@
         <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>1065</v>
+        <v>1061</v>
       </c>
       <c r="F2" t="s">
         <v>233</v>
@@ -8109,7 +8109,7 @@
         <v>6</v>
       </c>
       <c r="E3" t="s">
-        <v>1066</v>
+        <v>1062</v>
       </c>
       <c r="F3" t="s">
         <v>233</v>
@@ -8132,7 +8132,7 @@
         <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>1067</v>
+        <v>1063</v>
       </c>
       <c r="F4" t="s">
         <v>233</v>
@@ -8155,7 +8155,7 @@
         <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>1068</v>
+        <v>1064</v>
       </c>
       <c r="F5" t="s">
         <v>233</v>
@@ -8178,7 +8178,7 @@
         <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>1068</v>
+        <v>1064</v>
       </c>
       <c r="F6" t="s">
         <v>233</v>
@@ -8201,7 +8201,7 @@
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>1069</v>
+        <v>1065</v>
       </c>
       <c r="F7" t="s">
         <v>233</v>
@@ -8224,7 +8224,7 @@
         <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>1065</v>
+        <v>1061</v>
       </c>
       <c r="F8" t="s">
         <v>233</v>
@@ -8247,7 +8247,7 @@
         <v>6</v>
       </c>
       <c r="E9" t="s">
-        <v>1070</v>
+        <v>1066</v>
       </c>
       <c r="F9" t="s">
         <v>233</v>
@@ -8270,7 +8270,7 @@
         <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>1068</v>
+        <v>1064</v>
       </c>
       <c r="F10" t="s">
         <v>233</v>
@@ -8334,7 +8334,7 @@
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>1065</v>
+        <v>1061</v>
       </c>
       <c r="F2" t="s">
         <v>233</v>
@@ -8357,7 +8357,7 @@
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>1059</v>
+        <v>1055</v>
       </c>
       <c r="F3" t="s">
         <v>233</v>
@@ -8380,7 +8380,7 @@
         <v>24</v>
       </c>
       <c r="E4" t="s">
-        <v>1067</v>
+        <v>1063</v>
       </c>
       <c r="F4" t="s">
         <v>233</v>
@@ -8403,7 +8403,7 @@
         <v>6</v>
       </c>
       <c r="E5" t="s">
-        <v>1071</v>
+        <v>1067</v>
       </c>
       <c r="F5" t="s">
         <v>233</v>
@@ -8426,7 +8426,7 @@
         <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>1059</v>
+        <v>1055</v>
       </c>
       <c r="F6" t="s">
         <v>13</v>
@@ -8449,7 +8449,7 @@
         <v>24</v>
       </c>
       <c r="E7" t="s">
-        <v>1067</v>
+        <v>1063</v>
       </c>
       <c r="F7" t="s">
         <v>233</v>
@@ -8472,7 +8472,7 @@
         <v>6</v>
       </c>
       <c r="E8" t="s">
-        <v>1072</v>
+        <v>1068</v>
       </c>
       <c r="F8" t="s">
         <v>233</v>
@@ -8536,7 +8536,7 @@
         <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F2" t="s">
         <v>233</v>
@@ -8559,7 +8559,7 @@
         <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
       <c r="F3" t="s">
         <v>233</v>
@@ -8582,7 +8582,7 @@
         <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F4" t="s">
         <v>9</v>
@@ -8605,7 +8605,7 @@
         <v>20</v>
       </c>
       <c r="E5" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
       <c r="F5" t="s">
         <v>9</v>
@@ -8628,7 +8628,7 @@
         <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F6" t="s">
         <v>233</v>
@@ -8651,7 +8651,7 @@
         <v>20</v>
       </c>
       <c r="E7" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
       <c r="F7" t="s">
         <v>233</v>
@@ -8674,7 +8674,7 @@
         <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -8697,7 +8697,7 @@
         <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
       <c r="F9" t="s">
         <v>9</v>
@@ -9515,7 +9515,7 @@
         <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F10" t="s">
         <v>9</v>
@@ -9998,7 +9998,7 @@
         <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F31" t="s">
         <v>9</v>
@@ -10021,7 +10021,7 @@
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F32" t="s">
         <v>9</v>
@@ -10044,7 +10044,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F33" t="s">
         <v>9</v>
@@ -10055,10 +10055,10 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>890</v>
+        <v>1103</v>
       </c>
       <c r="B34" t="s">
-        <v>891</v>
+        <v>1106</v>
       </c>
       <c r="C34">
         <v>4446</v>
@@ -10067,7 +10067,7 @@
         <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F34" t="s">
         <v>9</v>
@@ -10078,10 +10078,10 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>892</v>
+        <v>1104</v>
       </c>
       <c r="B35" t="s">
-        <v>893</v>
+        <v>1105</v>
       </c>
       <c r="C35">
         <v>4476</v>
@@ -10101,10 +10101,10 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>894</v>
+        <v>890</v>
       </c>
       <c r="B36" t="s">
-        <v>895</v>
+        <v>891</v>
       </c>
       <c r="C36">
         <v>4348</v>
@@ -10113,7 +10113,7 @@
         <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F36" t="s">
         <v>9</v>
@@ -10124,10 +10124,10 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>896</v>
+        <v>892</v>
       </c>
       <c r="B37" t="s">
-        <v>897</v>
+        <v>893</v>
       </c>
       <c r="C37">
         <v>4456</v>
@@ -10136,7 +10136,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
       <c r="F37" t="s">
         <v>233</v>
@@ -10147,10 +10147,10 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>898</v>
+        <v>894</v>
       </c>
       <c r="B38" t="s">
-        <v>899</v>
+        <v>895</v>
       </c>
       <c r="C38">
         <v>4051</v>
@@ -10170,10 +10170,10 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>900</v>
+        <v>896</v>
       </c>
       <c r="B39" t="s">
-        <v>901</v>
+        <v>897</v>
       </c>
       <c r="C39">
         <v>4408</v>
@@ -10193,10 +10193,10 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>902</v>
+        <v>898</v>
       </c>
       <c r="B40" t="s">
-        <v>903</v>
+        <v>899</v>
       </c>
       <c r="C40">
         <v>4341</v>
@@ -10216,10 +10216,10 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>904</v>
+        <v>900</v>
       </c>
       <c r="B41" t="s">
-        <v>905</v>
+        <v>901</v>
       </c>
       <c r="C41">
         <v>4265</v>
@@ -10239,10 +10239,10 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>906</v>
+        <v>902</v>
       </c>
       <c r="B42" t="s">
-        <v>907</v>
+        <v>903</v>
       </c>
       <c r="C42">
         <v>4266</v>
@@ -10262,10 +10262,10 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>908</v>
+        <v>904</v>
       </c>
       <c r="B43" t="s">
-        <v>909</v>
+        <v>905</v>
       </c>
       <c r="C43">
         <v>4269</v>
@@ -10285,10 +10285,10 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>910</v>
+        <v>906</v>
       </c>
       <c r="B44" t="s">
-        <v>911</v>
+        <v>907</v>
       </c>
       <c r="C44">
         <v>4273</v>
@@ -10308,10 +10308,10 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>912</v>
+        <v>908</v>
       </c>
       <c r="B45" t="s">
-        <v>913</v>
+        <v>909</v>
       </c>
       <c r="C45">
         <v>4405</v>
@@ -10331,10 +10331,10 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>914</v>
+        <v>910</v>
       </c>
       <c r="B46" t="s">
-        <v>915</v>
+        <v>911</v>
       </c>
       <c r="C46">
         <v>4406</v>
@@ -10354,10 +10354,10 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>916</v>
+        <v>912</v>
       </c>
       <c r="B47" t="s">
-        <v>917</v>
+        <v>913</v>
       </c>
       <c r="C47">
         <v>4267</v>
@@ -10377,10 +10377,10 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>918</v>
+        <v>914</v>
       </c>
       <c r="B48" t="s">
-        <v>919</v>
+        <v>915</v>
       </c>
       <c r="C48">
         <v>4271</v>
@@ -10400,10 +10400,10 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>920</v>
+        <v>916</v>
       </c>
       <c r="B49" t="s">
-        <v>921</v>
+        <v>917</v>
       </c>
       <c r="C49">
         <v>4276</v>
@@ -10423,10 +10423,10 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>922</v>
+        <v>918</v>
       </c>
       <c r="B50" t="s">
-        <v>923</v>
+        <v>919</v>
       </c>
       <c r="C50">
         <v>4342</v>
@@ -10446,10 +10446,10 @@
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>924</v>
+        <v>920</v>
       </c>
       <c r="B51" t="s">
-        <v>925</v>
+        <v>921</v>
       </c>
       <c r="C51">
         <v>4398</v>
@@ -10469,10 +10469,10 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>926</v>
+        <v>922</v>
       </c>
       <c r="B52" t="s">
-        <v>927</v>
+        <v>923</v>
       </c>
       <c r="C52">
         <v>4270</v>
@@ -10492,10 +10492,10 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>928</v>
+        <v>924</v>
       </c>
       <c r="B53" t="s">
-        <v>929</v>
+        <v>925</v>
       </c>
       <c r="C53">
         <v>4275</v>
@@ -10515,10 +10515,10 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>930</v>
+        <v>926</v>
       </c>
       <c r="B54" t="s">
-        <v>931</v>
+        <v>927</v>
       </c>
       <c r="C54">
         <v>4274</v>
@@ -10538,10 +10538,10 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>932</v>
+        <v>928</v>
       </c>
       <c r="B55" t="s">
-        <v>933</v>
+        <v>929</v>
       </c>
       <c r="C55">
         <v>4399</v>
@@ -10561,10 +10561,10 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>934</v>
+        <v>930</v>
       </c>
       <c r="B56" t="s">
-        <v>935</v>
+        <v>931</v>
       </c>
       <c r="C56">
         <v>4404</v>
@@ -10584,10 +10584,10 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>936</v>
+        <v>932</v>
       </c>
       <c r="B57" t="s">
-        <v>937</v>
+        <v>933</v>
       </c>
       <c r="C57">
         <v>4262</v>
@@ -10607,10 +10607,10 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>938</v>
+        <v>934</v>
       </c>
       <c r="B58" t="s">
-        <v>939</v>
+        <v>935</v>
       </c>
       <c r="C58">
         <v>4263</v>
@@ -10630,10 +10630,10 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>940</v>
+        <v>936</v>
       </c>
       <c r="B59" t="s">
-        <v>941</v>
+        <v>937</v>
       </c>
       <c r="C59">
         <v>4264</v>
@@ -10653,10 +10653,10 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>942</v>
+        <v>938</v>
       </c>
       <c r="B60" t="s">
-        <v>943</v>
+        <v>939</v>
       </c>
       <c r="C60">
         <v>4407</v>
@@ -10676,10 +10676,10 @@
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>944</v>
+        <v>940</v>
       </c>
       <c r="B61" t="s">
-        <v>945</v>
+        <v>941</v>
       </c>
       <c r="C61">
         <v>4397</v>
@@ -10699,10 +10699,10 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>946</v>
+        <v>942</v>
       </c>
       <c r="B62" t="s">
-        <v>947</v>
+        <v>943</v>
       </c>
       <c r="C62">
         <v>4343</v>
@@ -10722,10 +10722,10 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>948</v>
+        <v>944</v>
       </c>
       <c r="B63" t="s">
-        <v>949</v>
+        <v>945</v>
       </c>
       <c r="C63">
         <v>4268</v>
@@ -10745,10 +10745,10 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>950</v>
+        <v>946</v>
       </c>
       <c r="B64" t="s">
-        <v>951</v>
+        <v>947</v>
       </c>
       <c r="C64">
         <v>2833</v>
@@ -10768,10 +10768,10 @@
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>950</v>
+        <v>946</v>
       </c>
       <c r="B65" t="s">
-        <v>951</v>
+        <v>947</v>
       </c>
       <c r="C65">
         <v>3125</v>
@@ -10791,10 +10791,10 @@
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>952</v>
+        <v>948</v>
       </c>
       <c r="B66" t="s">
-        <v>953</v>
+        <v>949</v>
       </c>
       <c r="C66">
         <v>3752</v>
@@ -10814,10 +10814,10 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>952</v>
+        <v>948</v>
       </c>
       <c r="B67" t="s">
-        <v>953</v>
+        <v>949</v>
       </c>
       <c r="C67">
         <v>3753</v>
@@ -10837,10 +10837,10 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>954</v>
+        <v>950</v>
       </c>
       <c r="B68" t="s">
-        <v>955</v>
+        <v>951</v>
       </c>
       <c r="C68">
         <v>2511</v>
@@ -10860,10 +10860,10 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>956</v>
+        <v>952</v>
       </c>
       <c r="B69" t="s">
-        <v>957</v>
+        <v>953</v>
       </c>
       <c r="C69">
         <v>4311</v>
@@ -10883,10 +10883,10 @@
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>958</v>
+        <v>954</v>
       </c>
       <c r="B70" t="s">
-        <v>959</v>
+        <v>955</v>
       </c>
       <c r="C70">
         <v>4046</v>
@@ -10906,10 +10906,10 @@
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>958</v>
+        <v>954</v>
       </c>
       <c r="B71" t="s">
-        <v>959</v>
+        <v>955</v>
       </c>
       <c r="C71">
         <v>4047</v>
@@ -10929,10 +10929,10 @@
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>960</v>
+        <v>956</v>
       </c>
       <c r="B72" t="s">
-        <v>961</v>
+        <v>957</v>
       </c>
       <c r="C72">
         <v>4312</v>
@@ -10952,10 +10952,10 @@
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>962</v>
+        <v>958</v>
       </c>
       <c r="B73" t="s">
-        <v>963</v>
+        <v>959</v>
       </c>
       <c r="C73">
         <v>4310</v>
@@ -10975,10 +10975,10 @@
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>964</v>
+        <v>960</v>
       </c>
       <c r="B74" t="s">
-        <v>965</v>
+        <v>961</v>
       </c>
       <c r="C74">
         <v>4074</v>
@@ -10987,7 +10987,7 @@
         <v>1</v>
       </c>
       <c r="E74" t="s">
-        <v>1074</v>
+        <v>1070</v>
       </c>
       <c r="F74" t="s">
         <v>13</v>
@@ -10998,10 +10998,10 @@
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>966</v>
+        <v>962</v>
       </c>
       <c r="B75" t="s">
-        <v>967</v>
+        <v>963</v>
       </c>
       <c r="C75">
         <v>4076</v>
@@ -11010,10 +11010,10 @@
         <v>1</v>
       </c>
       <c r="E75" t="s">
-        <v>1075</v>
+        <v>1071</v>
       </c>
       <c r="F75" t="s">
-        <v>968</v>
+        <v>964</v>
       </c>
       <c r="G75">
         <v>32.5</v>
@@ -11021,10 +11021,10 @@
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>969</v>
+        <v>965</v>
       </c>
       <c r="B76" t="s">
-        <v>970</v>
+        <v>966</v>
       </c>
       <c r="C76">
         <v>4133</v>
@@ -11033,10 +11033,10 @@
         <v>10</v>
       </c>
       <c r="E76" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
       <c r="F76" t="s">
-        <v>968</v>
+        <v>964</v>
       </c>
       <c r="G76">
         <v>72</v>
@@ -11044,10 +11044,10 @@
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>971</v>
+        <v>967</v>
       </c>
       <c r="B77" t="s">
-        <v>972</v>
+        <v>968</v>
       </c>
       <c r="C77">
         <v>3068</v>
@@ -11067,10 +11067,10 @@
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>971</v>
+        <v>967</v>
       </c>
       <c r="B78" t="s">
-        <v>972</v>
+        <v>968</v>
       </c>
       <c r="C78">
         <v>3087</v>
@@ -11090,10 +11090,10 @@
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>973</v>
+        <v>969</v>
       </c>
       <c r="B79" t="s">
-        <v>974</v>
+        <v>970</v>
       </c>
       <c r="C79">
         <v>4560</v>
@@ -11113,10 +11113,10 @@
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>975</v>
+        <v>971</v>
       </c>
       <c r="B80" t="s">
-        <v>976</v>
+        <v>972</v>
       </c>
       <c r="C80">
         <v>4531</v>
@@ -11125,7 +11125,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F80" t="s">
         <v>32</v>
@@ -11136,10 +11136,10 @@
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>975</v>
+        <v>971</v>
       </c>
       <c r="B81" t="s">
-        <v>976</v>
+        <v>972</v>
       </c>
       <c r="C81">
         <v>4532</v>
@@ -11159,10 +11159,10 @@
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>977</v>
+        <v>973</v>
       </c>
       <c r="B82" t="s">
-        <v>978</v>
+        <v>974</v>
       </c>
       <c r="C82">
         <v>4559</v>
@@ -11171,7 +11171,7 @@
         <v>12</v>
       </c>
       <c r="E82" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
       <c r="F82" t="s">
         <v>13</v>
@@ -11182,10 +11182,10 @@
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>979</v>
+        <v>975</v>
       </c>
       <c r="B83" t="s">
-        <v>980</v>
+        <v>976</v>
       </c>
       <c r="C83">
         <v>4493</v>
@@ -11205,10 +11205,10 @@
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>981</v>
+        <v>977</v>
       </c>
       <c r="B84" t="s">
-        <v>982</v>
+        <v>978</v>
       </c>
       <c r="C84">
         <v>4102</v>
@@ -11217,7 +11217,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="F84" t="s">
         <v>13</v>
@@ -11228,10 +11228,10 @@
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>983</v>
+        <v>979</v>
       </c>
       <c r="B85" t="s">
-        <v>984</v>
+        <v>980</v>
       </c>
       <c r="C85">
         <v>4103</v>
@@ -11240,7 +11240,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="F85" t="s">
         <v>233</v>
@@ -11251,10 +11251,10 @@
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>985</v>
+        <v>981</v>
       </c>
       <c r="B86" t="s">
-        <v>986</v>
+        <v>982</v>
       </c>
       <c r="C86">
         <v>4547</v>
@@ -11263,7 +11263,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="F86" t="s">
         <v>233</v>
@@ -11274,10 +11274,10 @@
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>1089</v>
+        <v>1085</v>
       </c>
       <c r="B87" t="s">
-        <v>1095</v>
+        <v>1091</v>
       </c>
       <c r="C87">
         <v>4624</v>
@@ -11286,7 +11286,7 @@
         <v>21</v>
       </c>
       <c r="E87" t="s">
-        <v>1101</v>
+        <v>1097</v>
       </c>
       <c r="F87" t="s">
         <v>13</v>
@@ -11297,10 +11297,10 @@
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>1105</v>
+        <v>1101</v>
       </c>
       <c r="B88" t="s">
-        <v>1106</v>
+        <v>1102</v>
       </c>
       <c r="C88">
         <v>4627</v>
@@ -11309,7 +11309,7 @@
         <v>25</v>
       </c>
       <c r="E88" t="s">
-        <v>1102</v>
+        <v>1098</v>
       </c>
       <c r="F88" t="s">
         <v>13</v>
@@ -11320,10 +11320,10 @@
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>1090</v>
+        <v>1086</v>
       </c>
       <c r="B89" t="s">
-        <v>1096</v>
+        <v>1092</v>
       </c>
       <c r="C89">
         <v>4628</v>
@@ -11332,7 +11332,7 @@
         <v>15</v>
       </c>
       <c r="E89" t="s">
-        <v>1103</v>
+        <v>1099</v>
       </c>
       <c r="F89" t="s">
         <v>13</v>
@@ -11343,10 +11343,10 @@
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>1091</v>
+        <v>1087</v>
       </c>
       <c r="B90" t="s">
-        <v>1097</v>
+        <v>1093</v>
       </c>
       <c r="C90">
         <v>4625</v>
@@ -11355,7 +11355,7 @@
         <v>21</v>
       </c>
       <c r="E90" t="s">
-        <v>1101</v>
+        <v>1097</v>
       </c>
       <c r="F90" t="s">
         <v>13</v>
@@ -11366,10 +11366,10 @@
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>1092</v>
+        <v>1088</v>
       </c>
       <c r="B91" t="s">
-        <v>1098</v>
+        <v>1094</v>
       </c>
       <c r="C91">
         <v>4626</v>
@@ -11378,7 +11378,7 @@
         <v>21</v>
       </c>
       <c r="E91" t="s">
-        <v>1101</v>
+        <v>1097</v>
       </c>
       <c r="F91" t="s">
         <v>13</v>
@@ -11389,10 +11389,10 @@
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>1093</v>
+        <v>1089</v>
       </c>
       <c r="B92" t="s">
-        <v>1099</v>
+        <v>1095</v>
       </c>
       <c r="C92">
         <v>4629</v>
@@ -11401,7 +11401,7 @@
         <v>12</v>
       </c>
       <c r="E92" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="F92" t="s">
         <v>9</v>
@@ -11412,10 +11412,10 @@
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>1094</v>
+        <v>1090</v>
       </c>
       <c r="B93" t="s">
-        <v>1100</v>
+        <v>1096</v>
       </c>
       <c r="C93">
         <v>4630</v>
@@ -11424,7 +11424,7 @@
         <v>12</v>
       </c>
       <c r="E93" t="s">
-        <v>1104</v>
+        <v>1100</v>
       </c>
       <c r="F93" t="s">
         <v>9</v>
@@ -11435,10 +11435,10 @@
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>987</v>
+        <v>983</v>
       </c>
       <c r="B94" t="s">
-        <v>988</v>
+        <v>984</v>
       </c>
       <c r="C94">
         <v>4104</v>
@@ -11447,7 +11447,7 @@
         <v>10</v>
       </c>
       <c r="E94" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="F94" t="s">
         <v>233</v>
@@ -11458,10 +11458,10 @@
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>989</v>
+        <v>985</v>
       </c>
       <c r="B95" t="s">
-        <v>990</v>
+        <v>986</v>
       </c>
       <c r="C95">
         <v>4101</v>
@@ -11470,7 +11470,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="F95" t="s">
         <v>233</v>
@@ -11481,10 +11481,10 @@
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>991</v>
+        <v>987</v>
       </c>
       <c r="B96" t="s">
-        <v>992</v>
+        <v>988</v>
       </c>
       <c r="C96">
         <v>4105</v>
@@ -11493,7 +11493,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="F96" t="s">
         <v>233</v>
@@ -11504,10 +11504,10 @@
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>993</v>
+        <v>989</v>
       </c>
       <c r="B97" t="s">
-        <v>994</v>
+        <v>990</v>
       </c>
       <c r="C97">
         <v>3705</v>
@@ -11516,7 +11516,7 @@
         <v>12</v>
       </c>
       <c r="E97" t="s">
-        <v>1076</v>
+        <v>1072</v>
       </c>
       <c r="F97" t="s">
         <v>233</v>
@@ -11527,10 +11527,10 @@
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>995</v>
+        <v>991</v>
       </c>
       <c r="B98" t="s">
-        <v>996</v>
+        <v>992</v>
       </c>
       <c r="C98">
         <v>3823</v>
@@ -11539,7 +11539,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="F98" t="s">
         <v>9</v>
@@ -11550,10 +11550,10 @@
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>997</v>
+        <v>993</v>
       </c>
       <c r="B99" t="s">
-        <v>998</v>
+        <v>994</v>
       </c>
       <c r="C99">
         <v>4583</v>
@@ -11562,7 +11562,7 @@
         <v>12</v>
       </c>
       <c r="E99" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="F99" t="s">
         <v>233</v>
@@ -11573,10 +11573,10 @@
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>999</v>
+        <v>995</v>
       </c>
       <c r="B100" t="s">
-        <v>1000</v>
+        <v>996</v>
       </c>
       <c r="C100">
         <v>4308</v>
@@ -11585,7 +11585,7 @@
         <v>10</v>
       </c>
       <c r="E100" t="s">
-        <v>1077</v>
+        <v>1073</v>
       </c>
       <c r="F100" t="s">
         <v>13</v>
@@ -11596,10 +11596,10 @@
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>1001</v>
+        <v>997</v>
       </c>
       <c r="B101" t="s">
-        <v>1002</v>
+        <v>998</v>
       </c>
       <c r="C101">
         <v>4309</v>
@@ -11608,10 +11608,10 @@
         <v>10</v>
       </c>
       <c r="E101" t="s">
-        <v>1077</v>
+        <v>1073</v>
       </c>
       <c r="F101" t="s">
-        <v>968</v>
+        <v>964</v>
       </c>
       <c r="G101">
         <v>68.5</v>
@@ -11619,10 +11619,10 @@
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>1003</v>
+        <v>999</v>
       </c>
       <c r="B102" t="s">
-        <v>1004</v>
+        <v>1000</v>
       </c>
       <c r="C102">
         <v>4412</v>
@@ -11634,7 +11634,7 @@
         <v>8</v>
       </c>
       <c r="F102" t="s">
-        <v>968</v>
+        <v>964</v>
       </c>
       <c r="G102">
         <v>71.5</v>
@@ -11642,10 +11642,10 @@
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>1005</v>
+        <v>1001</v>
       </c>
       <c r="B103" t="s">
-        <v>1006</v>
+        <v>1002</v>
       </c>
       <c r="C103">
         <v>4413</v>
@@ -11665,10 +11665,10 @@
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>1005</v>
+        <v>1001</v>
       </c>
       <c r="B104" t="s">
-        <v>1006</v>
+        <v>1002</v>
       </c>
       <c r="C104">
         <v>4414</v>
@@ -11688,10 +11688,10 @@
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>1007</v>
+        <v>1003</v>
       </c>
       <c r="B105" t="s">
-        <v>1008</v>
+        <v>1004</v>
       </c>
       <c r="C105">
         <v>4415</v>
@@ -11711,10 +11711,10 @@
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>1007</v>
+        <v>1003</v>
       </c>
       <c r="B106" t="s">
-        <v>1008</v>
+        <v>1004</v>
       </c>
       <c r="C106">
         <v>4416</v>
@@ -11734,10 +11734,10 @@
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>1009</v>
+        <v>1005</v>
       </c>
       <c r="B107" t="s">
-        <v>1010</v>
+        <v>1006</v>
       </c>
       <c r="C107">
         <v>4475</v>
@@ -11746,7 +11746,7 @@
         <v>1</v>
       </c>
       <c r="E107" t="s">
-        <v>1083</v>
+        <v>1079</v>
       </c>
       <c r="F107" t="s">
         <v>13</v>
@@ -11757,10 +11757,10 @@
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>1011</v>
+        <v>1007</v>
       </c>
       <c r="B108" t="s">
-        <v>1012</v>
+        <v>1008</v>
       </c>
       <c r="C108">
         <v>4354</v>
@@ -11769,7 +11769,7 @@
         <v>12</v>
       </c>
       <c r="E108" t="s">
-        <v>1083</v>
+        <v>1079</v>
       </c>
       <c r="F108" t="s">
         <v>744</v>
@@ -11780,10 +11780,10 @@
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>1013</v>
+        <v>1009</v>
       </c>
       <c r="B109" t="s">
-        <v>1014</v>
+        <v>1010</v>
       </c>
       <c r="C109">
         <v>4445</v>
@@ -11792,7 +11792,7 @@
         <v>12</v>
       </c>
       <c r="E109" t="s">
-        <v>1083</v>
+        <v>1079</v>
       </c>
       <c r="F109" t="s">
         <v>9</v>
@@ -11803,10 +11803,10 @@
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>1015</v>
+        <v>1011</v>
       </c>
       <c r="B110" t="s">
-        <v>1016</v>
+        <v>1012</v>
       </c>
       <c r="C110">
         <v>4353</v>
@@ -11815,7 +11815,7 @@
         <v>12</v>
       </c>
       <c r="E110" t="s">
-        <v>1083</v>
+        <v>1079</v>
       </c>
       <c r="F110" t="s">
         <v>9</v>
@@ -11826,10 +11826,10 @@
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>1017</v>
+        <v>1013</v>
       </c>
       <c r="B111" t="s">
-        <v>1018</v>
+        <v>1014</v>
       </c>
       <c r="C111">
         <v>4350</v>
@@ -11838,7 +11838,7 @@
         <v>12</v>
       </c>
       <c r="E111" t="s">
-        <v>1083</v>
+        <v>1079</v>
       </c>
       <c r="F111" t="s">
         <v>9</v>
@@ -11849,10 +11849,10 @@
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>1019</v>
+        <v>1015</v>
       </c>
       <c r="B112" t="s">
-        <v>1020</v>
+        <v>1016</v>
       </c>
       <c r="C112">
         <v>4352</v>
@@ -11861,7 +11861,7 @@
         <v>12</v>
       </c>
       <c r="E112" t="s">
-        <v>1083</v>
+        <v>1079</v>
       </c>
       <c r="F112" t="s">
         <v>9</v>
@@ -11872,10 +11872,10 @@
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>1021</v>
+        <v>1017</v>
       </c>
       <c r="B113" t="s">
-        <v>1022</v>
+        <v>1018</v>
       </c>
       <c r="C113">
         <v>4349</v>
@@ -11884,7 +11884,7 @@
         <v>12</v>
       </c>
       <c r="E113" t="s">
-        <v>1083</v>
+        <v>1079</v>
       </c>
       <c r="F113" t="s">
         <v>9</v>
@@ -11895,10 +11895,10 @@
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>1023</v>
+        <v>1019</v>
       </c>
       <c r="B114" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="C114">
         <v>4351</v>
@@ -11907,7 +11907,7 @@
         <v>12</v>
       </c>
       <c r="E114" t="s">
-        <v>1083</v>
+        <v>1079</v>
       </c>
       <c r="F114" t="s">
         <v>9</v>
@@ -11918,10 +11918,10 @@
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>1025</v>
+        <v>1021</v>
       </c>
       <c r="B115" t="s">
-        <v>1026</v>
+        <v>1022</v>
       </c>
       <c r="C115">
         <v>4581</v>
@@ -11930,7 +11930,7 @@
         <v>12</v>
       </c>
       <c r="E115" t="s">
-        <v>1083</v>
+        <v>1079</v>
       </c>
       <c r="F115" t="s">
         <v>9</v>
@@ -11941,10 +11941,10 @@
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>1027</v>
+        <v>1023</v>
       </c>
       <c r="B116" t="s">
-        <v>1028</v>
+        <v>1024</v>
       </c>
       <c r="C116">
         <v>4096</v>
@@ -11964,10 +11964,10 @@
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>1029</v>
+        <v>1025</v>
       </c>
       <c r="B117" t="s">
-        <v>1030</v>
+        <v>1026</v>
       </c>
       <c r="C117">
         <v>4123</v>
@@ -11976,7 +11976,7 @@
         <v>10</v>
       </c>
       <c r="E117" t="s">
-        <v>1076</v>
+        <v>1072</v>
       </c>
       <c r="F117" t="s">
         <v>13</v>
@@ -11987,10 +11987,10 @@
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>1031</v>
+        <v>1027</v>
       </c>
       <c r="B118" t="s">
-        <v>1032</v>
+        <v>1028</v>
       </c>
       <c r="C118">
         <v>4306</v>
@@ -11999,10 +11999,10 @@
         <v>10</v>
       </c>
       <c r="E118" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="F118" t="s">
-        <v>968</v>
+        <v>964</v>
       </c>
       <c r="G118">
         <v>81</v>
@@ -12010,10 +12010,10 @@
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>1033</v>
+        <v>1029</v>
       </c>
       <c r="B119" t="s">
-        <v>1034</v>
+        <v>1030</v>
       </c>
       <c r="C119">
         <v>4307</v>
@@ -12022,10 +12022,10 @@
         <v>10</v>
       </c>
       <c r="E119" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="F119" t="s">
-        <v>968</v>
+        <v>964</v>
       </c>
       <c r="G119">
         <v>81</v>
@@ -12033,10 +12033,10 @@
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>1035</v>
+        <v>1031</v>
       </c>
       <c r="B120" t="s">
-        <v>1036</v>
+        <v>1032</v>
       </c>
       <c r="C120">
         <v>2659</v>
@@ -12045,7 +12045,7 @@
         <v>20</v>
       </c>
       <c r="E120" t="s">
-        <v>1079</v>
+        <v>1075</v>
       </c>
       <c r="F120" t="s">
         <v>233</v>
@@ -12056,10 +12056,10 @@
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>1035</v>
+        <v>1031</v>
       </c>
       <c r="B121" t="s">
-        <v>1036</v>
+        <v>1032</v>
       </c>
       <c r="C121">
         <v>2621</v>
@@ -12068,7 +12068,7 @@
         <v>5</v>
       </c>
       <c r="E121" t="s">
-        <v>1080</v>
+        <v>1076</v>
       </c>
       <c r="F121" t="s">
         <v>233</v>
@@ -12079,10 +12079,10 @@
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>1037</v>
+        <v>1033</v>
       </c>
       <c r="B122" t="s">
-        <v>1038</v>
+        <v>1034</v>
       </c>
       <c r="C122">
         <v>3656</v>
@@ -12091,7 +12091,7 @@
         <v>5</v>
       </c>
       <c r="E122" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="F122" t="s">
         <v>233</v>
@@ -12143,10 +12143,10 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1039</v>
+        <v>1035</v>
       </c>
       <c r="B2" t="s">
-        <v>1040</v>
+        <v>1036</v>
       </c>
       <c r="C2">
         <v>3459</v>
@@ -12166,10 +12166,10 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1041</v>
+        <v>1037</v>
       </c>
       <c r="B3" t="s">
-        <v>1042</v>
+        <v>1038</v>
       </c>
       <c r="C3">
         <v>3803</v>
@@ -12189,10 +12189,10 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1043</v>
+        <v>1039</v>
       </c>
       <c r="B4" t="s">
-        <v>1044</v>
+        <v>1040</v>
       </c>
       <c r="C4">
         <v>3425</v>
@@ -12212,10 +12212,10 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1043</v>
+        <v>1039</v>
       </c>
       <c r="B5" t="s">
-        <v>1044</v>
+        <v>1040</v>
       </c>
       <c r="C5">
         <v>3426</v>
@@ -12235,10 +12235,10 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="B6" t="s">
-        <v>1046</v>
+        <v>1042</v>
       </c>
       <c r="C6">
         <v>3427</v>
@@ -12258,10 +12258,10 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="B7" t="s">
-        <v>1046</v>
+        <v>1042</v>
       </c>
       <c r="C7">
         <v>3428</v>
@@ -12281,10 +12281,10 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>1047</v>
+        <v>1043</v>
       </c>
       <c r="B8" t="s">
-        <v>1048</v>
+        <v>1044</v>
       </c>
       <c r="C8">
         <v>3429</v>
@@ -12304,10 +12304,10 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>1047</v>
+        <v>1043</v>
       </c>
       <c r="B9" t="s">
-        <v>1048</v>
+        <v>1044</v>
       </c>
       <c r="C9">
         <v>3430</v>
@@ -12327,10 +12327,10 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>1049</v>
+        <v>1045</v>
       </c>
       <c r="B10" t="s">
-        <v>1050</v>
+        <v>1046</v>
       </c>
       <c r="C10">
         <v>3913</v>
@@ -12350,10 +12350,10 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>1049</v>
+        <v>1045</v>
       </c>
       <c r="B11" t="s">
-        <v>1050</v>
+        <v>1046</v>
       </c>
       <c r="C11">
         <v>3872</v>
@@ -12373,10 +12373,10 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>1051</v>
+        <v>1047</v>
       </c>
       <c r="B12" t="s">
-        <v>1052</v>
+        <v>1048</v>
       </c>
       <c r="C12">
         <v>3422</v>
@@ -12396,10 +12396,10 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>1051</v>
+        <v>1047</v>
       </c>
       <c r="B13" t="s">
-        <v>1052</v>
+        <v>1048</v>
       </c>
       <c r="C13">
         <v>3423</v>
@@ -12408,7 +12408,7 @@
         <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>1081</v>
+        <v>1077</v>
       </c>
       <c r="F13" t="s">
         <v>9</v>
@@ -12419,10 +12419,10 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
       <c r="B14" t="s">
-        <v>1054</v>
+        <v>1050</v>
       </c>
       <c r="C14">
         <v>3431</v>
@@ -12442,10 +12442,10 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
       <c r="B15" t="s">
-        <v>1054</v>
+        <v>1050</v>
       </c>
       <c r="C15">
         <v>3432</v>
@@ -12509,7 +12509,7 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>1084</v>
+        <v>1080</v>
       </c>
       <c r="C2">
         <v>585</v>
@@ -12532,7 +12532,7 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>1085</v>
+        <v>1081</v>
       </c>
       <c r="C3">
         <v>467</v>
@@ -13541,7 +13541,7 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>1086</v>
+        <v>1082</v>
       </c>
       <c r="B47" t="s">
         <v>59</v>
@@ -16424,10 +16424,10 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>1087</v>
+        <v>1083</v>
       </c>
       <c r="B48" t="s">
-        <v>1088</v>
+        <v>1084</v>
       </c>
       <c r="C48">
         <v>2466</v>
@@ -16447,10 +16447,10 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>1087</v>
+        <v>1083</v>
       </c>
       <c r="B49" t="s">
-        <v>1088</v>
+        <v>1084</v>
       </c>
       <c r="C49">
         <v>2465</v>
@@ -17466,7 +17466,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F17" t="s">
         <v>13</v>
@@ -17535,7 +17535,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F20" t="s">
         <v>233</v>
@@ -18294,7 +18294,7 @@
         <v>4</v>
       </c>
       <c r="E53" t="s">
-        <v>1056</v>
+        <v>1052</v>
       </c>
       <c r="F53" t="s">
         <v>233</v>
@@ -18363,7 +18363,7 @@
         <v>4</v>
       </c>
       <c r="E56" t="s">
-        <v>1056</v>
+        <v>1052</v>
       </c>
       <c r="F56" t="s">
         <v>233</v>
@@ -18570,7 +18570,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F65" t="s">
         <v>233</v>
@@ -21251,7 +21251,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
       <c r="F17" t="s">
         <v>233</v>
@@ -21274,7 +21274,7 @@
         <v>20</v>
       </c>
       <c r="E18" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
       <c r="F18" t="s">
         <v>233</v>
@@ -22465,7 +22465,7 @@
         <v>20</v>
       </c>
       <c r="E32" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F32" t="s">
         <v>9</v>
@@ -22488,7 +22488,7 @@
         <v>20</v>
       </c>
       <c r="E33" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F33" t="s">
         <v>233</v>
@@ -22511,7 +22511,7 @@
         <v>18</v>
       </c>
       <c r="E34" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F34" t="s">
         <v>9</v>
@@ -22534,7 +22534,7 @@
         <v>15</v>
       </c>
       <c r="E35" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F35" t="s">
         <v>9</v>
@@ -22580,7 +22580,7 @@
         <v>30</v>
       </c>
       <c r="E37" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F37" t="s">
         <v>233</v>
@@ -22626,7 +22626,7 @@
         <v>30</v>
       </c>
       <c r="E39" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="F39" t="s">
         <v>233</v>
@@ -23247,7 +23247,7 @@
         <v>6</v>
       </c>
       <c r="E66" t="s">
-        <v>1056</v>
+        <v>1052</v>
       </c>
       <c r="F66" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Atualizando item novo 12/05
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodos.xlsx
+++ b/data/ProdutosFomatodos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\listaDeProdutosB\lista-de-produtos-b\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25E48348-D186-4370-81E1-91703B074A98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87F2E9D9-8B07-40F2-8BE4-9131FB929469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="570" yWindow="780" windowWidth="27300" windowHeight="13920" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="570" yWindow="780" windowWidth="27300" windowHeight="13920" firstSheet="6" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="promoçoes" sheetId="18" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3590" uniqueCount="1107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3594" uniqueCount="1109">
   <si>
     <t>produto_grupo</t>
   </si>
@@ -3358,6 +3358,12 @@
   </si>
   <si>
     <t>BALA GELATINA COBRINHA CITRICA</t>
+  </si>
+  <si>
+    <t>gota-chocolate-branco</t>
+  </si>
+  <si>
+    <t>GOTA CHOCOLATE BRANCO</t>
   </si>
 </sst>
 </file>
@@ -9283,7 +9289,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
-  <dimension ref="A1:G122"/>
+  <dimension ref="A1:G123"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -11619,48 +11625,48 @@
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>999</v>
+        <v>1107</v>
       </c>
       <c r="B102" t="s">
-        <v>1000</v>
+        <v>1108</v>
       </c>
       <c r="C102">
-        <v>4412</v>
+        <v>4635</v>
       </c>
       <c r="D102">
-        <v>2.5</v>
+        <v>10</v>
       </c>
       <c r="E102" t="s">
-        <v>8</v>
+        <v>1069</v>
       </c>
       <c r="F102" t="s">
         <v>964</v>
       </c>
       <c r="G102">
-        <v>71.5</v>
+        <v>167</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>1001</v>
+        <v>999</v>
       </c>
       <c r="B103" t="s">
-        <v>1002</v>
+        <v>1000</v>
       </c>
       <c r="C103">
-        <v>4413</v>
+        <v>4412</v>
       </c>
       <c r="D103">
-        <v>25</v>
+        <v>2.5</v>
       </c>
       <c r="E103" t="s">
         <v>8</v>
       </c>
       <c r="F103" t="s">
-        <v>13</v>
+        <v>964</v>
       </c>
       <c r="G103">
-        <v>496</v>
+        <v>71.5</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
@@ -11671,10 +11677,10 @@
         <v>1002</v>
       </c>
       <c r="C104">
-        <v>4414</v>
+        <v>4413</v>
       </c>
       <c r="D104">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E104" t="s">
         <v>8</v>
@@ -11683,21 +11689,21 @@
         <v>13</v>
       </c>
       <c r="G104">
-        <v>101</v>
+        <v>496</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>1003</v>
+        <v>1001</v>
       </c>
       <c r="B105" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
       <c r="C105">
-        <v>4415</v>
+        <v>4414</v>
       </c>
       <c r="D105">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E105" t="s">
         <v>8</v>
@@ -11706,7 +11712,7 @@
         <v>13</v>
       </c>
       <c r="G105">
-        <v>414</v>
+        <v>101</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
@@ -11717,10 +11723,10 @@
         <v>1004</v>
       </c>
       <c r="C106">
-        <v>4416</v>
+        <v>4415</v>
       </c>
       <c r="D106">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E106" t="s">
         <v>8</v>
@@ -11729,64 +11735,64 @@
         <v>13</v>
       </c>
       <c r="G106">
-        <v>85</v>
+        <v>414</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>1005</v>
+        <v>1003</v>
       </c>
       <c r="B107" t="s">
-        <v>1006</v>
+        <v>1004</v>
       </c>
       <c r="C107">
-        <v>4475</v>
+        <v>4416</v>
       </c>
       <c r="D107">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E107" t="s">
-        <v>1079</v>
+        <v>8</v>
       </c>
       <c r="F107" t="s">
         <v>13</v>
       </c>
       <c r="G107">
-        <v>9</v>
+        <v>85</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>1007</v>
+        <v>1005</v>
       </c>
       <c r="B108" t="s">
-        <v>1008</v>
+        <v>1006</v>
       </c>
       <c r="C108">
-        <v>4354</v>
+        <v>4475</v>
       </c>
       <c r="D108">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E108" t="s">
         <v>1079</v>
       </c>
       <c r="F108" t="s">
-        <v>744</v>
+        <v>13</v>
       </c>
       <c r="G108">
-        <v>79.5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>1009</v>
+        <v>1007</v>
       </c>
       <c r="B109" t="s">
-        <v>1010</v>
+        <v>1008</v>
       </c>
       <c r="C109">
-        <v>4445</v>
+        <v>4354</v>
       </c>
       <c r="D109">
         <v>12</v>
@@ -11795,7 +11801,7 @@
         <v>1079</v>
       </c>
       <c r="F109" t="s">
-        <v>9</v>
+        <v>744</v>
       </c>
       <c r="G109">
         <v>79.5</v>
@@ -11803,13 +11809,13 @@
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>1011</v>
+        <v>1009</v>
       </c>
       <c r="B110" t="s">
-        <v>1012</v>
+        <v>1010</v>
       </c>
       <c r="C110">
-        <v>4353</v>
+        <v>4445</v>
       </c>
       <c r="D110">
         <v>12</v>
@@ -11826,13 +11832,13 @@
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>1013</v>
+        <v>1011</v>
       </c>
       <c r="B111" t="s">
-        <v>1014</v>
+        <v>1012</v>
       </c>
       <c r="C111">
-        <v>4350</v>
+        <v>4353</v>
       </c>
       <c r="D111">
         <v>12</v>
@@ -11849,13 +11855,13 @@
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>1015</v>
+        <v>1013</v>
       </c>
       <c r="B112" t="s">
-        <v>1016</v>
+        <v>1014</v>
       </c>
       <c r="C112">
-        <v>4352</v>
+        <v>4350</v>
       </c>
       <c r="D112">
         <v>12</v>
@@ -11872,13 +11878,13 @@
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>1017</v>
+        <v>1015</v>
       </c>
       <c r="B113" t="s">
-        <v>1018</v>
+        <v>1016</v>
       </c>
       <c r="C113">
-        <v>4349</v>
+        <v>4352</v>
       </c>
       <c r="D113">
         <v>12</v>
@@ -11895,13 +11901,13 @@
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>1019</v>
+        <v>1017</v>
       </c>
       <c r="B114" t="s">
-        <v>1020</v>
+        <v>1018</v>
       </c>
       <c r="C114">
-        <v>4351</v>
+        <v>4349</v>
       </c>
       <c r="D114">
         <v>12</v>
@@ -11918,13 +11924,13 @@
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>1021</v>
+        <v>1019</v>
       </c>
       <c r="B115" t="s">
-        <v>1022</v>
+        <v>1020</v>
       </c>
       <c r="C115">
-        <v>4581</v>
+        <v>4351</v>
       </c>
       <c r="D115">
         <v>12</v>
@@ -11941,82 +11947,82 @@
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>1023</v>
+        <v>1021</v>
       </c>
       <c r="B116" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="C116">
-        <v>4096</v>
+        <v>4581</v>
       </c>
       <c r="D116">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E116" t="s">
-        <v>8</v>
+        <v>1079</v>
       </c>
       <c r="F116" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G116">
-        <v>79</v>
+        <v>79.5</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
       <c r="B117" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
       <c r="C117">
-        <v>4123</v>
+        <v>4096</v>
       </c>
       <c r="D117">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E117" t="s">
-        <v>1072</v>
+        <v>8</v>
       </c>
       <c r="F117" t="s">
         <v>13</v>
       </c>
       <c r="G117">
-        <v>60</v>
+        <v>79</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
       <c r="B118" t="s">
-        <v>1028</v>
+        <v>1026</v>
       </c>
       <c r="C118">
-        <v>4306</v>
+        <v>4123</v>
       </c>
       <c r="D118">
         <v>10</v>
       </c>
       <c r="E118" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
       <c r="F118" t="s">
-        <v>964</v>
+        <v>13</v>
       </c>
       <c r="G118">
-        <v>81</v>
+        <v>60</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>1029</v>
+        <v>1027</v>
       </c>
       <c r="B119" t="s">
-        <v>1030</v>
+        <v>1028</v>
       </c>
       <c r="C119">
-        <v>4307</v>
+        <v>4306</v>
       </c>
       <c r="D119">
         <v>10</v>
@@ -12033,25 +12039,25 @@
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
       <c r="B120" t="s">
-        <v>1032</v>
+        <v>1030</v>
       </c>
       <c r="C120">
-        <v>2659</v>
+        <v>4307</v>
       </c>
       <c r="D120">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E120" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="F120" t="s">
-        <v>233</v>
+        <v>964</v>
       </c>
       <c r="G120">
-        <v>27.5</v>
+        <v>81</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
@@ -12062,41 +12068,64 @@
         <v>1032</v>
       </c>
       <c r="C121">
-        <v>2621</v>
+        <v>2659</v>
       </c>
       <c r="D121">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E121" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="F121" t="s">
         <v>233</v>
       </c>
       <c r="G121">
-        <v>24.5</v>
+        <v>27.5</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>1033</v>
+        <v>1031</v>
       </c>
       <c r="B122" t="s">
-        <v>1034</v>
+        <v>1032</v>
       </c>
       <c r="C122">
-        <v>3656</v>
+        <v>2621</v>
       </c>
       <c r="D122">
         <v>5</v>
       </c>
       <c r="E122" t="s">
-        <v>1074</v>
+        <v>1076</v>
       </c>
       <c r="F122" t="s">
         <v>233</v>
       </c>
       <c r="G122">
+        <v>24.5</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B123" t="s">
+        <v>1034</v>
+      </c>
+      <c r="C123">
+        <v>3656</v>
+      </c>
+      <c r="D123">
+        <v>5</v>
+      </c>
+      <c r="E123" t="s">
+        <v>1074</v>
+      </c>
+      <c r="F123" t="s">
+        <v>233</v>
+      </c>
+      <c r="G123">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizando preços e produtos novos 21/05
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodos.xlsx
+++ b/data/ProdutosFomatodos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\listaDeProdutosB\lista-de-produtos-b\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1F583BD-A60C-4DAD-BC6E-905FC1C3107E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5B73CEB-260B-4B6F-9A2C-3F9C500AFC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="promoçoes" sheetId="18" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3590" uniqueCount="1109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3602" uniqueCount="1113">
   <si>
     <t>produto_grupo</t>
   </si>
@@ -3364,6 +3364,18 @@
   </si>
   <si>
     <t>GOTA CHOCOLATE BRANCO</t>
+  </si>
+  <si>
+    <t>flocos-de-arroz</t>
+  </si>
+  <si>
+    <t>FLOCOS DE ARROZ</t>
+  </si>
+  <si>
+    <t>ameixa-em-po</t>
+  </si>
+  <si>
+    <t>AMEIXA EM PÓ</t>
   </si>
 </sst>
 </file>
@@ -5358,7 +5370,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:G116"/>
+  <dimension ref="A1:G119"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -5550,7 +5562,7 @@
         <v>233</v>
       </c>
       <c r="G8">
-        <v>57.5</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -5573,7 +5585,7 @@
         <v>233</v>
       </c>
       <c r="G9">
-        <v>65</v>
+        <v>69.5</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -5596,7 +5608,7 @@
         <v>233</v>
       </c>
       <c r="G10">
-        <v>141.5</v>
+        <v>153.5</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -5762,25 +5774,25 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>654</v>
+        <v>1111</v>
       </c>
       <c r="B18" t="s">
-        <v>655</v>
+        <v>1112</v>
       </c>
       <c r="C18">
-        <v>2336</v>
+        <v>4639</v>
       </c>
       <c r="D18">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E18" t="s">
         <v>8</v>
       </c>
       <c r="F18" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G18">
-        <v>750</v>
+        <v>295</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -5791,42 +5803,42 @@
         <v>655</v>
       </c>
       <c r="C19">
-        <v>2421</v>
+        <v>2336</v>
       </c>
       <c r="D19">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="E19" t="s">
         <v>8</v>
       </c>
       <c r="F19" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G19">
-        <v>91</v>
+        <v>750</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="B20" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="C20">
-        <v>2568</v>
+        <v>2421</v>
       </c>
       <c r="D20">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E20" t="s">
         <v>8</v>
       </c>
       <c r="F20" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G20">
-        <v>260</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -5837,53 +5849,53 @@
         <v>657</v>
       </c>
       <c r="C21">
-        <v>3009</v>
+        <v>2568</v>
       </c>
       <c r="D21">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E21" t="s">
         <v>8</v>
       </c>
       <c r="F21" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G21">
-        <v>78</v>
+        <v>260</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="B22" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="C22">
-        <v>2778</v>
+        <v>3009</v>
       </c>
       <c r="D22">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E22" t="s">
         <v>8</v>
       </c>
       <c r="F22" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G22">
-        <v>180</v>
+        <v>78</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="B23" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="C23">
-        <v>3106</v>
+        <v>2778</v>
       </c>
       <c r="D23">
         <v>5</v>
@@ -5892,33 +5904,33 @@
         <v>8</v>
       </c>
       <c r="F23" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G23">
-        <v>260</v>
+        <v>180</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="B24" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="C24">
-        <v>3489</v>
+        <v>3106</v>
       </c>
       <c r="D24">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E24" t="s">
         <v>8</v>
       </c>
       <c r="F24" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G24">
-        <v>700</v>
+        <v>260</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -5929,10 +5941,10 @@
         <v>663</v>
       </c>
       <c r="C25">
-        <v>3696</v>
+        <v>3489</v>
       </c>
       <c r="D25">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E25" t="s">
         <v>8</v>
@@ -5941,7 +5953,7 @@
         <v>32</v>
       </c>
       <c r="G25">
-        <v>280</v>
+        <v>700</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -5952,19 +5964,19 @@
         <v>663</v>
       </c>
       <c r="C26">
-        <v>2783</v>
+        <v>3696</v>
       </c>
       <c r="D26">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E26" t="s">
         <v>8</v>
       </c>
       <c r="F26" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G26">
-        <v>142</v>
+        <v>280</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -5975,10 +5987,10 @@
         <v>663</v>
       </c>
       <c r="C27">
-        <v>3755</v>
+        <v>2783</v>
       </c>
       <c r="D27">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E27" t="s">
         <v>8</v>
@@ -5987,30 +5999,30 @@
         <v>13</v>
       </c>
       <c r="G27">
-        <v>85</v>
+        <v>142</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="B28" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="C28">
-        <v>3486</v>
+        <v>3755</v>
       </c>
       <c r="D28">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E28" t="s">
         <v>8</v>
       </c>
       <c r="F28" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G28">
-        <v>595</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -6021,33 +6033,33 @@
         <v>665</v>
       </c>
       <c r="C29">
-        <v>4488</v>
+        <v>3486</v>
       </c>
       <c r="D29">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E29" t="s">
         <v>8</v>
       </c>
       <c r="F29" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G29">
-        <v>299.5</v>
+        <v>595</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="B30" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="C30">
-        <v>4333</v>
+        <v>3487</v>
       </c>
       <c r="D30">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E30" t="s">
         <v>8</v>
@@ -6056,18 +6068,18 @@
         <v>13</v>
       </c>
       <c r="G30">
-        <v>259.5</v>
+        <v>180</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>668</v>
+        <v>664</v>
       </c>
       <c r="B31" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
       <c r="C31">
-        <v>4388</v>
+        <v>4488</v>
       </c>
       <c r="D31">
         <v>5</v>
@@ -6079,18 +6091,18 @@
         <v>13</v>
       </c>
       <c r="G31">
-        <v>145</v>
+        <v>299.5</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
       <c r="B32" t="s">
-        <v>671</v>
+        <v>667</v>
       </c>
       <c r="C32">
-        <v>4389</v>
+        <v>4333</v>
       </c>
       <c r="D32">
         <v>5</v>
@@ -6102,41 +6114,41 @@
         <v>13</v>
       </c>
       <c r="G32">
-        <v>102</v>
+        <v>259.5</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
       <c r="B33" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="C33">
-        <v>3488</v>
+        <v>4388</v>
       </c>
       <c r="D33">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E33" t="s">
         <v>8</v>
       </c>
       <c r="F33" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G33">
-        <v>220</v>
+        <v>145</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="B34" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="C34">
-        <v>3400</v>
+        <v>4389</v>
       </c>
       <c r="D34">
         <v>5</v>
@@ -6148,64 +6160,64 @@
         <v>13</v>
       </c>
       <c r="G34">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="B35" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="C35">
-        <v>2257</v>
+        <v>3488</v>
       </c>
       <c r="D35">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="E35" t="s">
         <v>8</v>
       </c>
       <c r="F35" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G35">
-        <v>16</v>
+        <v>220</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="B36" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="C36">
-        <v>565</v>
+        <v>3400</v>
       </c>
       <c r="D36">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E36" t="s">
         <v>8</v>
       </c>
       <c r="F36" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G36">
-        <v>123</v>
+        <v>57</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="B37" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="C37">
-        <v>4474</v>
+        <v>2257</v>
       </c>
       <c r="D37">
         <v>3</v>
@@ -6217,41 +6229,41 @@
         <v>13</v>
       </c>
       <c r="G37">
-        <v>39</v>
+        <v>16</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>678</v>
+        <v>674</v>
       </c>
       <c r="B38" t="s">
-        <v>679</v>
+        <v>675</v>
       </c>
       <c r="C38">
-        <v>4473</v>
+        <v>565</v>
       </c>
       <c r="D38">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="E38" t="s">
         <v>8</v>
       </c>
       <c r="F38" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G38">
-        <v>39</v>
+        <v>123</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="B39" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
       <c r="C39">
-        <v>2658</v>
+        <v>4474</v>
       </c>
       <c r="D39">
         <v>3</v>
@@ -6268,13 +6280,13 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="B40" t="s">
-        <v>683</v>
+        <v>679</v>
       </c>
       <c r="C40">
-        <v>2657</v>
+        <v>4473</v>
       </c>
       <c r="D40">
         <v>3</v>
@@ -6291,16 +6303,16 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>684</v>
+        <v>680</v>
       </c>
       <c r="B41" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="C41">
-        <v>2657</v>
+        <v>2658</v>
       </c>
       <c r="D41">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E41" t="s">
         <v>8</v>
@@ -6309,21 +6321,21 @@
         <v>13</v>
       </c>
       <c r="G41">
-        <v>65</v>
+        <v>39</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="B42" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="C42">
-        <v>2658</v>
+        <v>2657</v>
       </c>
       <c r="D42">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E42" t="s">
         <v>8</v>
@@ -6332,251 +6344,251 @@
         <v>13</v>
       </c>
       <c r="G42">
-        <v>65</v>
+        <v>39</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="B43" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="C43">
-        <v>3537</v>
+        <v>2657</v>
       </c>
       <c r="D43">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E43" t="s">
-        <v>1051</v>
+        <v>8</v>
       </c>
       <c r="F43" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G43">
-        <v>162</v>
+        <v>65</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>688</v>
+        <v>680</v>
       </c>
       <c r="B44" t="s">
-        <v>689</v>
+        <v>681</v>
       </c>
       <c r="C44">
-        <v>2732</v>
+        <v>2658</v>
       </c>
       <c r="D44">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E44" t="s">
         <v>8</v>
       </c>
       <c r="F44" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G44">
-        <v>189</v>
+        <v>65</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>688</v>
+        <v>1109</v>
       </c>
       <c r="B45" t="s">
-        <v>689</v>
+        <v>1110</v>
       </c>
       <c r="C45">
-        <v>2733</v>
+        <v>4640</v>
       </c>
       <c r="D45">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E45" t="s">
-        <v>8</v>
+        <v>1051</v>
       </c>
       <c r="F45" t="s">
         <v>13</v>
       </c>
       <c r="G45">
-        <v>96.5</v>
+        <v>82.5</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>690</v>
+        <v>686</v>
       </c>
       <c r="B46" t="s">
-        <v>691</v>
+        <v>687</v>
       </c>
       <c r="C46">
-        <v>2584</v>
+        <v>3537</v>
       </c>
       <c r="D46">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>8</v>
+        <v>1051</v>
       </c>
       <c r="F46" t="s">
         <v>9</v>
       </c>
       <c r="G46">
-        <v>223</v>
+        <v>162</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="B47" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="C47">
-        <v>2677</v>
+        <v>2732</v>
       </c>
       <c r="D47">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E47" t="s">
         <v>8</v>
       </c>
       <c r="F47" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G47">
-        <v>113.5</v>
+        <v>189</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>692</v>
+        <v>688</v>
       </c>
       <c r="B48" t="s">
-        <v>693</v>
+        <v>689</v>
       </c>
       <c r="C48">
-        <v>2495</v>
+        <v>2733</v>
       </c>
       <c r="D48">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E48" t="s">
         <v>8</v>
       </c>
       <c r="F48" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G48">
-        <v>220</v>
+        <v>96.5</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="B49" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="C49">
-        <v>2678</v>
+        <v>2584</v>
       </c>
       <c r="D49">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E49" t="s">
         <v>8</v>
       </c>
       <c r="F49" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G49">
-        <v>112</v>
+        <v>223</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>694</v>
+        <v>690</v>
       </c>
       <c r="B50" t="s">
-        <v>695</v>
+        <v>691</v>
       </c>
       <c r="C50">
-        <v>4498</v>
+        <v>2677</v>
       </c>
       <c r="D50">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E50" t="s">
-        <v>1051</v>
+        <v>8</v>
       </c>
       <c r="F50" t="s">
-        <v>233</v>
+        <v>13</v>
       </c>
       <c r="G50">
-        <v>240</v>
+        <v>113.5</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>696</v>
+        <v>692</v>
       </c>
       <c r="B51" t="s">
-        <v>697</v>
+        <v>693</v>
       </c>
       <c r="C51">
-        <v>4253</v>
+        <v>2495</v>
       </c>
       <c r="D51">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E51" t="s">
         <v>8</v>
       </c>
       <c r="F51" t="s">
-        <v>233</v>
+        <v>9</v>
       </c>
       <c r="G51">
-        <v>112</v>
+        <v>220</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>696</v>
+        <v>692</v>
       </c>
       <c r="B52" t="s">
-        <v>697</v>
+        <v>693</v>
       </c>
       <c r="C52">
-        <v>4500</v>
+        <v>2678</v>
       </c>
       <c r="D52">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E52" t="s">
         <v>8</v>
       </c>
       <c r="F52" t="s">
-        <v>233</v>
+        <v>13</v>
       </c>
       <c r="G52">
-        <v>224</v>
+        <v>112</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="B53" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="C53">
-        <v>4249</v>
+        <v>4498</v>
       </c>
       <c r="D53">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E53" t="s">
         <v>1051</v>
@@ -6585,7 +6597,7 @@
         <v>233</v>
       </c>
       <c r="G53">
-        <v>230</v>
+        <v>240</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
@@ -6596,56 +6608,56 @@
         <v>697</v>
       </c>
       <c r="C54">
-        <v>3724</v>
+        <v>4253</v>
       </c>
       <c r="D54">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E54" t="s">
-        <v>1051</v>
+        <v>8</v>
       </c>
       <c r="F54" t="s">
         <v>233</v>
       </c>
       <c r="G54">
-        <v>224</v>
+        <v>112</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="B55" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="C55">
-        <v>3736</v>
+        <v>4500</v>
       </c>
       <c r="D55">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E55" t="s">
-        <v>1051</v>
+        <v>8</v>
       </c>
       <c r="F55" t="s">
-        <v>9</v>
+        <v>233</v>
       </c>
       <c r="G55">
-        <v>162</v>
+        <v>224</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>700</v>
+        <v>696</v>
       </c>
       <c r="B56" t="s">
-        <v>701</v>
+        <v>697</v>
       </c>
       <c r="C56">
-        <v>4499</v>
+        <v>4249</v>
       </c>
       <c r="D56">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E56" t="s">
         <v>1051</v>
@@ -6654,110 +6666,110 @@
         <v>233</v>
       </c>
       <c r="G56">
-        <v>240</v>
+        <v>230</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>702</v>
+        <v>696</v>
       </c>
       <c r="B57" t="s">
-        <v>703</v>
+        <v>697</v>
       </c>
       <c r="C57">
-        <v>3536</v>
+        <v>3724</v>
       </c>
       <c r="D57">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E57" t="s">
         <v>1051</v>
       </c>
       <c r="F57" t="s">
-        <v>9</v>
+        <v>233</v>
       </c>
       <c r="G57">
-        <v>162</v>
+        <v>224</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>704</v>
+        <v>698</v>
       </c>
       <c r="B58" t="s">
-        <v>705</v>
+        <v>699</v>
       </c>
       <c r="C58">
-        <v>2494</v>
+        <v>3736</v>
       </c>
       <c r="D58">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E58" t="s">
-        <v>8</v>
+        <v>1051</v>
       </c>
       <c r="F58" t="s">
         <v>9</v>
       </c>
       <c r="G58">
-        <v>188.5</v>
+        <v>162</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>704</v>
+        <v>700</v>
       </c>
       <c r="B59" t="s">
-        <v>705</v>
+        <v>701</v>
       </c>
       <c r="C59">
-        <v>2679</v>
+        <v>4499</v>
       </c>
       <c r="D59">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E59" t="s">
-        <v>8</v>
+        <v>1051</v>
       </c>
       <c r="F59" t="s">
-        <v>13</v>
+        <v>233</v>
       </c>
       <c r="G59">
-        <v>96</v>
+        <v>240</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>706</v>
+        <v>702</v>
       </c>
       <c r="B60" t="s">
-        <v>707</v>
+        <v>703</v>
       </c>
       <c r="C60">
-        <v>4497</v>
+        <v>3536</v>
       </c>
       <c r="D60">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E60" t="s">
         <v>1051</v>
       </c>
       <c r="F60" t="s">
-        <v>233</v>
+        <v>9</v>
       </c>
       <c r="G60">
-        <v>240</v>
+        <v>162</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>708</v>
+        <v>704</v>
       </c>
       <c r="B61" t="s">
-        <v>709</v>
+        <v>705</v>
       </c>
       <c r="C61">
-        <v>2493</v>
+        <v>2494</v>
       </c>
       <c r="D61">
         <v>10</v>
@@ -6769,205 +6781,205 @@
         <v>9</v>
       </c>
       <c r="G61">
-        <v>180</v>
+        <v>188.5</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>710</v>
+        <v>704</v>
       </c>
       <c r="B62" t="s">
-        <v>711</v>
+        <v>705</v>
       </c>
       <c r="C62">
-        <v>3535</v>
+        <v>2679</v>
       </c>
       <c r="D62">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E62" t="s">
-        <v>1051</v>
+        <v>8</v>
       </c>
       <c r="F62" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G62">
-        <v>162</v>
+        <v>96</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="B63" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="C63">
-        <v>2498</v>
+        <v>4497</v>
       </c>
       <c r="D63">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E63" t="s">
-        <v>8</v>
+        <v>1051</v>
       </c>
       <c r="F63" t="s">
-        <v>13</v>
+        <v>233</v>
       </c>
       <c r="G63">
-        <v>92</v>
+        <v>240</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>712</v>
+        <v>708</v>
       </c>
       <c r="B64" t="s">
-        <v>713</v>
+        <v>709</v>
       </c>
       <c r="C64">
-        <v>2806</v>
+        <v>2493</v>
       </c>
       <c r="D64">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E64" t="s">
         <v>8</v>
       </c>
       <c r="F64" t="s">
-        <v>233</v>
+        <v>9</v>
       </c>
       <c r="G64">
-        <v>472.5</v>
+        <v>180</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="B65" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="C65">
-        <v>2807</v>
+        <v>3535</v>
       </c>
       <c r="D65">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E65" t="s">
-        <v>8</v>
+        <v>1051</v>
       </c>
       <c r="F65" t="s">
         <v>9</v>
       </c>
       <c r="G65">
-        <v>159.5</v>
+        <v>162</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>714</v>
+        <v>708</v>
       </c>
       <c r="B66" t="s">
-        <v>715</v>
+        <v>709</v>
       </c>
       <c r="C66">
-        <v>4556</v>
+        <v>2498</v>
       </c>
       <c r="D66">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E66" t="s">
         <v>8</v>
       </c>
       <c r="F66" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G66">
-        <v>900</v>
+        <v>92</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="B67" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="C67">
-        <v>4557</v>
+        <v>2806</v>
       </c>
       <c r="D67">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E67" t="s">
         <v>8</v>
       </c>
       <c r="F67" t="s">
-        <v>13</v>
+        <v>233</v>
       </c>
       <c r="G67">
-        <v>182</v>
+        <v>472.5</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>716</v>
+        <v>712</v>
       </c>
       <c r="B68" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
       <c r="C68">
-        <v>4018</v>
+        <v>2807</v>
       </c>
       <c r="D68">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E68" t="s">
         <v>8</v>
       </c>
       <c r="F68" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G68">
-        <v>230</v>
+        <v>159.5</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="B69" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="C69">
-        <v>2652</v>
+        <v>4556</v>
       </c>
       <c r="D69">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E69" t="s">
         <v>8</v>
       </c>
       <c r="F69" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G69">
-        <v>117</v>
+        <v>900</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>718</v>
+        <v>714</v>
       </c>
       <c r="B70" t="s">
-        <v>719</v>
+        <v>715</v>
       </c>
       <c r="C70">
-        <v>4049</v>
+        <v>4557</v>
       </c>
       <c r="D70">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E70" t="s">
         <v>8</v>
@@ -6976,21 +6988,21 @@
         <v>13</v>
       </c>
       <c r="G70">
-        <v>210</v>
+        <v>182</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="B71" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="C71">
-        <v>3737</v>
+        <v>4018</v>
       </c>
       <c r="D71">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E71" t="s">
         <v>8</v>
@@ -6999,21 +7011,21 @@
         <v>13</v>
       </c>
       <c r="G71">
-        <v>107</v>
+        <v>230</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>720</v>
+        <v>716</v>
       </c>
       <c r="B72" t="s">
-        <v>721</v>
+        <v>717</v>
       </c>
       <c r="C72">
-        <v>4301</v>
+        <v>2652</v>
       </c>
       <c r="D72">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E72" t="s">
         <v>8</v>
@@ -7022,21 +7034,21 @@
         <v>13</v>
       </c>
       <c r="G72">
-        <v>235</v>
+        <v>117</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>722</v>
+        <v>718</v>
       </c>
       <c r="B73" t="s">
-        <v>723</v>
+        <v>719</v>
       </c>
       <c r="C73">
-        <v>4334</v>
+        <v>4049</v>
       </c>
       <c r="D73">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E73" t="s">
         <v>8</v>
@@ -7045,44 +7057,44 @@
         <v>13</v>
       </c>
       <c r="G73">
-        <v>376.5</v>
+        <v>210</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>724</v>
+        <v>718</v>
       </c>
       <c r="B74" t="s">
-        <v>725</v>
+        <v>719</v>
       </c>
       <c r="C74">
-        <v>195</v>
+        <v>3737</v>
       </c>
       <c r="D74">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E74" t="s">
         <v>8</v>
       </c>
       <c r="F74" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G74">
-        <v>255</v>
+        <v>107</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>724</v>
+        <v>720</v>
       </c>
       <c r="B75" t="s">
-        <v>725</v>
+        <v>721</v>
       </c>
       <c r="C75">
-        <v>54</v>
+        <v>4301</v>
       </c>
       <c r="D75">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E75" t="s">
         <v>8</v>
@@ -7091,113 +7103,113 @@
         <v>13</v>
       </c>
       <c r="G75">
-        <v>53</v>
+        <v>235</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>726</v>
+        <v>722</v>
       </c>
       <c r="B76" t="s">
-        <v>727</v>
+        <v>723</v>
       </c>
       <c r="C76">
-        <v>63</v>
+        <v>4334</v>
       </c>
       <c r="D76">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E76" t="s">
         <v>8</v>
       </c>
       <c r="F76" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G76">
-        <v>255</v>
+        <v>376.5</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="B77" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="C77">
-        <v>2483</v>
+        <v>195</v>
       </c>
       <c r="D77">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E77" t="s">
         <v>8</v>
       </c>
       <c r="F77" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G77">
-        <v>53</v>
+        <v>255</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>728</v>
+        <v>724</v>
       </c>
       <c r="B78" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="C78">
-        <v>2974</v>
+        <v>54</v>
       </c>
       <c r="D78">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E78" t="s">
         <v>8</v>
       </c>
       <c r="F78" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G78">
-        <v>250</v>
+        <v>53</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="B79" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="C79">
-        <v>2831</v>
+        <v>63</v>
       </c>
       <c r="D79">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E79" t="s">
         <v>8</v>
       </c>
       <c r="F79" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G79">
-        <v>127</v>
+        <v>255</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>730</v>
+        <v>726</v>
       </c>
       <c r="B80" t="s">
-        <v>731</v>
+        <v>727</v>
       </c>
       <c r="C80">
-        <v>4137</v>
+        <v>2483</v>
       </c>
       <c r="D80">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E80" t="s">
         <v>8</v>
@@ -7206,41 +7218,41 @@
         <v>13</v>
       </c>
       <c r="G80">
-        <v>270</v>
+        <v>53</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>732</v>
+        <v>728</v>
       </c>
       <c r="B81" t="s">
-        <v>733</v>
+        <v>729</v>
       </c>
       <c r="C81">
-        <v>4380</v>
+        <v>2974</v>
       </c>
       <c r="D81">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E81" t="s">
         <v>8</v>
       </c>
       <c r="F81" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G81">
-        <v>270</v>
+        <v>250</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>734</v>
+        <v>728</v>
       </c>
       <c r="B82" t="s">
-        <v>735</v>
+        <v>729</v>
       </c>
       <c r="C82">
-        <v>4566</v>
+        <v>2831</v>
       </c>
       <c r="D82">
         <v>5</v>
@@ -7252,21 +7264,21 @@
         <v>13</v>
       </c>
       <c r="G82">
-        <v>240</v>
+        <v>127</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>736</v>
+        <v>730</v>
       </c>
       <c r="B83" t="s">
-        <v>737</v>
+        <v>731</v>
       </c>
       <c r="C83">
-        <v>4567</v>
+        <v>4137</v>
       </c>
       <c r="D83">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E83" t="s">
         <v>8</v>
@@ -7275,21 +7287,21 @@
         <v>13</v>
       </c>
       <c r="G83">
-        <v>240</v>
+        <v>270</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>738</v>
+        <v>732</v>
       </c>
       <c r="B84" t="s">
-        <v>739</v>
+        <v>733</v>
       </c>
       <c r="C84">
-        <v>4204</v>
+        <v>4380</v>
       </c>
       <c r="D84">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E84" t="s">
         <v>8</v>
@@ -7298,44 +7310,44 @@
         <v>13</v>
       </c>
       <c r="G84">
-        <v>145.5</v>
+        <v>270</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>738</v>
+        <v>734</v>
       </c>
       <c r="B85" t="s">
-        <v>739</v>
+        <v>735</v>
       </c>
       <c r="C85">
-        <v>4205</v>
+        <v>4566</v>
       </c>
       <c r="D85">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E85" t="s">
         <v>8</v>
       </c>
       <c r="F85" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G85">
-        <v>360</v>
+        <v>240</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="B86" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="C86">
-        <v>4225</v>
+        <v>4567</v>
       </c>
       <c r="D86">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E86" t="s">
         <v>8</v>
@@ -7344,44 +7356,44 @@
         <v>13</v>
       </c>
       <c r="G86">
-        <v>900</v>
+        <v>240</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="B87" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C87">
-        <v>4378</v>
+        <v>4204</v>
       </c>
       <c r="D87">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E87" t="s">
         <v>8</v>
       </c>
       <c r="F87" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G87">
-        <v>430</v>
+        <v>145.5</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="B88" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C88">
-        <v>4379</v>
+        <v>4205</v>
       </c>
       <c r="D88">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E88" t="s">
         <v>8</v>
@@ -7390,228 +7402,228 @@
         <v>32</v>
       </c>
       <c r="G88">
-        <v>43</v>
+        <v>360</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="B89" t="s">
-        <v>743</v>
+        <v>739</v>
       </c>
       <c r="C89">
-        <v>3524</v>
+        <v>4225</v>
       </c>
       <c r="D89">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="E89" t="s">
         <v>8</v>
       </c>
       <c r="F89" t="s">
-        <v>744</v>
+        <v>13</v>
       </c>
       <c r="G89">
-        <v>350</v>
+        <v>900</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="B90" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
       <c r="C90">
-        <v>3523</v>
+        <v>4378</v>
       </c>
       <c r="D90">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E90" t="s">
         <v>8</v>
       </c>
       <c r="F90" t="s">
-        <v>744</v>
+        <v>32</v>
       </c>
       <c r="G90">
-        <v>72</v>
+        <v>430</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>745</v>
+        <v>740</v>
       </c>
       <c r="B91" t="s">
-        <v>746</v>
+        <v>741</v>
       </c>
       <c r="C91">
-        <v>3521</v>
+        <v>4379</v>
       </c>
       <c r="D91">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E91" t="s">
-        <v>1078</v>
+        <v>8</v>
       </c>
       <c r="F91" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="G91">
-        <v>158</v>
+        <v>43</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="B92" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="C92">
-        <v>3522</v>
+        <v>3524</v>
       </c>
       <c r="D92">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E92" t="s">
-        <v>1069</v>
+        <v>8</v>
       </c>
       <c r="F92" t="s">
-        <v>9</v>
+        <v>744</v>
       </c>
       <c r="G92">
-        <v>216.5</v>
+        <v>350</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>747</v>
+        <v>742</v>
       </c>
       <c r="B93" t="s">
-        <v>748</v>
+        <v>743</v>
       </c>
       <c r="C93">
-        <v>64</v>
+        <v>3523</v>
       </c>
       <c r="D93">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E93" t="s">
-        <v>1051</v>
+        <v>8</v>
       </c>
       <c r="F93" t="s">
-        <v>9</v>
+        <v>744</v>
       </c>
       <c r="G93">
-        <v>132</v>
+        <v>72</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="B94" t="s">
-        <v>750</v>
+        <v>746</v>
       </c>
       <c r="C94">
-        <v>90</v>
+        <v>3521</v>
       </c>
       <c r="D94">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E94" t="s">
-        <v>1051</v>
+        <v>1078</v>
       </c>
       <c r="F94" t="s">
         <v>9</v>
       </c>
       <c r="G94">
-        <v>132</v>
+        <v>158</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>751</v>
+        <v>745</v>
       </c>
       <c r="B95" t="s">
-        <v>752</v>
+        <v>746</v>
       </c>
       <c r="C95">
-        <v>3637</v>
+        <v>3522</v>
       </c>
       <c r="D95">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="E95" t="s">
-        <v>8</v>
+        <v>1069</v>
       </c>
       <c r="F95" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="G95">
-        <v>375</v>
+        <v>216.5</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>751</v>
+        <v>747</v>
       </c>
       <c r="B96" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="C96">
-        <v>2805</v>
+        <v>64</v>
       </c>
       <c r="D96">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E96" t="s">
-        <v>8</v>
+        <v>1051</v>
       </c>
       <c r="F96" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="G96">
-        <v>150</v>
+        <v>132</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="B97" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="C97">
-        <v>2427</v>
+        <v>90</v>
       </c>
       <c r="D97">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E97" t="s">
-        <v>8</v>
+        <v>1051</v>
       </c>
       <c r="F97" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G97">
-        <v>46</v>
+        <v>132</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="B98" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="C98">
-        <v>3437</v>
+        <v>3637</v>
       </c>
       <c r="D98">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E98" t="s">
         <v>8</v>
@@ -7620,251 +7632,251 @@
         <v>32</v>
       </c>
       <c r="G98">
-        <v>390</v>
+        <v>375</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="B99" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="C99">
-        <v>3396</v>
+        <v>2805</v>
       </c>
       <c r="D99">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E99" t="s">
         <v>8</v>
       </c>
       <c r="F99" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G99">
-        <v>197</v>
+        <v>150</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="B100" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="C100">
-        <v>3395</v>
+        <v>2427</v>
       </c>
       <c r="D100">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E100" t="s">
-        <v>1054</v>
+        <v>8</v>
       </c>
       <c r="F100" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G100">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="B101" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="C101">
-        <v>3490</v>
+        <v>3437</v>
       </c>
       <c r="D101">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E101" t="s">
-        <v>1054</v>
+        <v>8</v>
       </c>
       <c r="F101" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="G101">
-        <v>169</v>
+        <v>390</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>759</v>
+        <v>753</v>
       </c>
       <c r="B102" t="s">
-        <v>760</v>
+        <v>754</v>
       </c>
       <c r="C102">
-        <v>458</v>
+        <v>3396</v>
       </c>
       <c r="D102">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E102" t="s">
-        <v>1055</v>
+        <v>8</v>
       </c>
       <c r="F102" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G102">
-        <v>269.5</v>
+        <v>197</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>761</v>
+        <v>755</v>
       </c>
       <c r="B103" t="s">
-        <v>762</v>
+        <v>756</v>
       </c>
       <c r="C103">
-        <v>2641</v>
+        <v>3395</v>
       </c>
       <c r="D103">
         <v>12</v>
       </c>
       <c r="E103" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="F103" t="s">
         <v>9</v>
       </c>
       <c r="G103">
-        <v>222</v>
+        <v>54</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>763</v>
+        <v>757</v>
       </c>
       <c r="B104" t="s">
-        <v>764</v>
+        <v>758</v>
       </c>
       <c r="C104">
-        <v>4293</v>
+        <v>3490</v>
       </c>
       <c r="D104">
         <v>12</v>
       </c>
       <c r="E104" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="F104" t="s">
         <v>9</v>
       </c>
       <c r="G104">
-        <v>210</v>
+        <v>169</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>765</v>
+        <v>759</v>
       </c>
       <c r="B105" t="s">
-        <v>766</v>
+        <v>760</v>
       </c>
       <c r="C105">
-        <v>2396</v>
+        <v>458</v>
       </c>
       <c r="D105">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="E105" t="s">
-        <v>8</v>
+        <v>1055</v>
       </c>
       <c r="F105" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="G105">
-        <v>675</v>
+        <v>269.5</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>765</v>
+        <v>761</v>
       </c>
       <c r="B106" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="C106">
-        <v>2426</v>
+        <v>2641</v>
       </c>
       <c r="D106">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E106" t="s">
-        <v>8</v>
+        <v>1055</v>
       </c>
       <c r="F106" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G106">
-        <v>137</v>
+        <v>222</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>767</v>
+        <v>763</v>
       </c>
       <c r="B107" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
       <c r="C107">
-        <v>4335</v>
+        <v>4293</v>
       </c>
       <c r="D107">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E107" t="s">
-        <v>8</v>
+        <v>1055</v>
       </c>
       <c r="F107" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G107">
-        <v>440</v>
+        <v>210</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>769</v>
+        <v>765</v>
       </c>
       <c r="B108" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
       <c r="C108">
-        <v>4477</v>
+        <v>2396</v>
       </c>
       <c r="D108">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="E108" t="s">
         <v>8</v>
       </c>
       <c r="F108" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G108">
-        <v>252</v>
+        <v>675</v>
       </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>771</v>
+        <v>765</v>
       </c>
       <c r="B109" t="s">
-        <v>772</v>
+        <v>766</v>
       </c>
       <c r="C109">
-        <v>4479</v>
+        <v>2426</v>
       </c>
       <c r="D109">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E109" t="s">
         <v>8</v>
@@ -7873,18 +7885,18 @@
         <v>13</v>
       </c>
       <c r="G109">
-        <v>252</v>
+        <v>137</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>773</v>
+        <v>767</v>
       </c>
       <c r="B110" t="s">
-        <v>774</v>
+        <v>768</v>
       </c>
       <c r="C110">
-        <v>4478</v>
+        <v>4335</v>
       </c>
       <c r="D110">
         <v>3</v>
@@ -7896,144 +7908,213 @@
         <v>13</v>
       </c>
       <c r="G110">
-        <v>252</v>
+        <v>440</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>775</v>
+        <v>769</v>
       </c>
       <c r="B111" t="s">
-        <v>776</v>
+        <v>770</v>
       </c>
       <c r="C111">
-        <v>2646</v>
+        <v>4477</v>
       </c>
       <c r="D111">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E111" t="s">
-        <v>1056</v>
+        <v>8</v>
       </c>
       <c r="F111" t="s">
-        <v>233</v>
+        <v>13</v>
       </c>
       <c r="G111">
-        <v>50.5</v>
+        <v>252</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
       <c r="B112" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="C112">
-        <v>2645</v>
+        <v>4479</v>
       </c>
       <c r="D112">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E112" t="s">
-        <v>1057</v>
+        <v>8</v>
       </c>
       <c r="F112" t="s">
-        <v>233</v>
+        <v>13</v>
       </c>
       <c r="G112">
-        <v>78</v>
+        <v>252</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="B113" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="C113">
-        <v>2638</v>
+        <v>4478</v>
       </c>
       <c r="D113">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E113" t="s">
-        <v>1058</v>
+        <v>8</v>
       </c>
       <c r="F113" t="s">
-        <v>233</v>
+        <v>13</v>
       </c>
       <c r="G113">
-        <v>65</v>
+        <v>252</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="B114" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="C114">
-        <v>4294</v>
+        <v>2646</v>
       </c>
       <c r="D114">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E114" t="s">
-        <v>1059</v>
+        <v>1056</v>
       </c>
       <c r="F114" t="s">
         <v>233</v>
       </c>
       <c r="G114">
-        <v>150</v>
+        <v>53</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="B115" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="C115">
-        <v>4314</v>
+        <v>2645</v>
       </c>
       <c r="D115">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E115" t="s">
-        <v>1069</v>
+        <v>1057</v>
       </c>
       <c r="F115" t="s">
-        <v>9</v>
+        <v>233</v>
       </c>
       <c r="G115">
-        <v>252</v>
+        <v>81.5</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
+        <v>775</v>
+      </c>
+      <c r="B116" t="s">
+        <v>776</v>
+      </c>
+      <c r="C116">
+        <v>2638</v>
+      </c>
+      <c r="D116">
+        <v>9</v>
+      </c>
+      <c r="E116" t="s">
+        <v>1058</v>
+      </c>
+      <c r="F116" t="s">
+        <v>233</v>
+      </c>
+      <c r="G116">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>777</v>
+      </c>
+      <c r="B117" t="s">
+        <v>778</v>
+      </c>
+      <c r="C117">
+        <v>4294</v>
+      </c>
+      <c r="D117">
+        <v>18</v>
+      </c>
+      <c r="E117" t="s">
+        <v>1059</v>
+      </c>
+      <c r="F117" t="s">
+        <v>233</v>
+      </c>
+      <c r="G117">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>779</v>
+      </c>
+      <c r="B118" t="s">
+        <v>780</v>
+      </c>
+      <c r="C118">
+        <v>4314</v>
+      </c>
+      <c r="D118">
+        <v>15</v>
+      </c>
+      <c r="E118" t="s">
+        <v>1069</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+      <c r="G118">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
         <v>781</v>
       </c>
-      <c r="B116" t="s">
+      <c r="B119" t="s">
         <v>782</v>
       </c>
-      <c r="C116">
+      <c r="C119">
         <v>4315</v>
       </c>
-      <c r="D116">
+      <c r="D119">
         <v>15</v>
       </c>
-      <c r="E116" t="s">
+      <c r="E119" t="s">
         <v>1060</v>
       </c>
-      <c r="F116" t="s">
+      <c r="F119" t="s">
         <v>9</v>
       </c>
-      <c r="G116">
+      <c r="G119">
         <v>450</v>
       </c>
     </row>
@@ -12080,7 +12161,7 @@
         <v>233</v>
       </c>
       <c r="G121">
-        <v>27.5</v>
+        <v>30</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
@@ -12103,7 +12184,7 @@
         <v>233</v>
       </c>
       <c r="G122">
-        <v>24.5</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Atualizando o preço e mercadoria nova 21/05
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodos.xlsx
+++ b/data/ProdutosFomatodos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\listaDeProdutosB\lista-de-produtos-b\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5B73CEB-260B-4B6F-9A2C-3F9C500AFC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4264EEB-64F0-4D88-AEEA-69FF97D773BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="345" yWindow="945" windowWidth="27300" windowHeight="13920" firstSheet="10" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="promoçoes" sheetId="18" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3602" uniqueCount="1113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3606" uniqueCount="1116">
   <si>
     <t>produto_grupo</t>
   </si>
@@ -3376,6 +3376,15 @@
   </si>
   <si>
     <t>AMEIXA EM PÓ</t>
+  </si>
+  <si>
+    <t>pacoca-de-amendoim-espeto</t>
+  </si>
+  <si>
+    <t>PAÇOCA DE AMENDOIM ESPETO</t>
+  </si>
+  <si>
+    <t>X90G</t>
   </si>
 </sst>
 </file>
@@ -9370,7 +9379,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
-  <dimension ref="A1:G123"/>
+  <dimension ref="A1:G124"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -11747,7 +11756,7 @@
         <v>964</v>
       </c>
       <c r="G103">
-        <v>71.5</v>
+        <v>75.5</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
@@ -12074,59 +12083,59 @@
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>1025</v>
+        <v>1113</v>
       </c>
       <c r="B118" t="s">
-        <v>1026</v>
+        <v>1114</v>
       </c>
       <c r="C118">
-        <v>4123</v>
+        <v>4582</v>
       </c>
       <c r="D118">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E118" t="s">
-        <v>1072</v>
+        <v>1115</v>
       </c>
       <c r="F118" t="s">
         <v>13</v>
       </c>
       <c r="G118">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
       <c r="B119" t="s">
-        <v>1028</v>
+        <v>1026</v>
       </c>
       <c r="C119">
-        <v>4306</v>
+        <v>4123</v>
       </c>
       <c r="D119">
         <v>10</v>
       </c>
       <c r="E119" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
       <c r="F119" t="s">
-        <v>964</v>
+        <v>13</v>
       </c>
       <c r="G119">
-        <v>81</v>
+        <v>60</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>1029</v>
+        <v>1027</v>
       </c>
       <c r="B120" t="s">
-        <v>1030</v>
+        <v>1028</v>
       </c>
       <c r="C120">
-        <v>4307</v>
+        <v>4306</v>
       </c>
       <c r="D120">
         <v>10</v>
@@ -12143,25 +12152,25 @@
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
       <c r="B121" t="s">
-        <v>1032</v>
+        <v>1030</v>
       </c>
       <c r="C121">
-        <v>2659</v>
+        <v>4307</v>
       </c>
       <c r="D121">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E121" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="F121" t="s">
-        <v>233</v>
+        <v>964</v>
       </c>
       <c r="G121">
-        <v>30</v>
+        <v>81</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
@@ -12172,41 +12181,64 @@
         <v>1032</v>
       </c>
       <c r="C122">
-        <v>2621</v>
+        <v>2659</v>
       </c>
       <c r="D122">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E122" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="F122" t="s">
         <v>233</v>
       </c>
       <c r="G122">
-        <v>25.5</v>
+        <v>30</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>1033</v>
+        <v>1031</v>
       </c>
       <c r="B123" t="s">
-        <v>1034</v>
+        <v>1032</v>
       </c>
       <c r="C123">
-        <v>3656</v>
+        <v>2621</v>
       </c>
       <c r="D123">
         <v>5</v>
       </c>
       <c r="E123" t="s">
-        <v>1074</v>
+        <v>1076</v>
       </c>
       <c r="F123" t="s">
         <v>233</v>
       </c>
       <c r="G123">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B124" t="s">
+        <v>1034</v>
+      </c>
+      <c r="C124">
+        <v>3656</v>
+      </c>
+      <c r="D124">
+        <v>5</v>
+      </c>
+      <c r="E124" t="s">
+        <v>1074</v>
+      </c>
+      <c r="F124" t="s">
+        <v>233</v>
+      </c>
+      <c r="G124">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizando preço e cadastro de iten 09/06
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodos.xlsx
+++ b/data/ProdutosFomatodos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\listaDeProdutosB\lista-de-produtos-b\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{324B2951-729C-4623-A9D7-77CA7D5D6774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D2B29DD-7B93-495E-B10B-ED12ADF839DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="promoçoes" sheetId="18" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3646" uniqueCount="1119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3650" uniqueCount="1121">
   <si>
     <t>produto_grupo</t>
   </si>
@@ -3394,6 +3394,12 @@
   </si>
   <si>
     <t>doce-de-leite-c-cacausouvenir</t>
+  </si>
+  <si>
+    <t>canjicao-amarelo</t>
+  </si>
+  <si>
+    <t>CANJICÃO AMARELO</t>
   </si>
 </sst>
 </file>
@@ -19059,7 +19065,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G93"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -19187,16 +19193,16 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>290</v>
+        <v>1119</v>
       </c>
       <c r="B6" t="s">
-        <v>291</v>
+        <v>1120</v>
       </c>
       <c r="C6">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="D6">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E6" t="s">
         <v>8</v>
@@ -19205,7 +19211,7 @@
         <v>32</v>
       </c>
       <c r="G6">
-        <v>63</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -19216,42 +19222,42 @@
         <v>291</v>
       </c>
       <c r="C7">
-        <v>2637</v>
+        <v>127</v>
       </c>
       <c r="D7">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E7" t="s">
         <v>8</v>
       </c>
       <c r="F7" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G7">
-        <v>14.5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B8" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C8">
-        <v>12</v>
+        <v>2637</v>
       </c>
       <c r="D8">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E8" t="s">
         <v>8</v>
       </c>
       <c r="F8" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G8">
-        <v>63</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -19262,33 +19268,33 @@
         <v>293</v>
       </c>
       <c r="C9">
-        <v>2501</v>
+        <v>12</v>
       </c>
       <c r="D9">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E9" t="s">
         <v>8</v>
       </c>
       <c r="F9" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G9">
-        <v>14.5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B10" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C10">
-        <v>24</v>
+        <v>2501</v>
       </c>
       <c r="D10">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E10" t="s">
         <v>8</v>
@@ -19297,7 +19303,7 @@
         <v>13</v>
       </c>
       <c r="G10">
-        <v>63</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -19308,33 +19314,33 @@
         <v>295</v>
       </c>
       <c r="C11">
-        <v>2726</v>
+        <v>24</v>
       </c>
       <c r="D11">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E11" t="s">
         <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G11">
-        <v>14.5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B12" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C12">
-        <v>4221</v>
+        <v>2726</v>
       </c>
       <c r="D12">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E12" t="s">
         <v>8</v>
@@ -19343,7 +19349,7 @@
         <v>32</v>
       </c>
       <c r="G12">
-        <v>142.5</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -19354,30 +19360,30 @@
         <v>297</v>
       </c>
       <c r="C13">
-        <v>4222</v>
+        <v>4221</v>
       </c>
       <c r="D13">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E13" t="s">
         <v>8</v>
       </c>
       <c r="F13" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G13">
-        <v>30.5</v>
+        <v>142.5</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B14" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C14">
-        <v>2580</v>
+        <v>4222</v>
       </c>
       <c r="D14">
         <v>5</v>
@@ -19389,7 +19395,7 @@
         <v>13</v>
       </c>
       <c r="G14">
-        <v>38</v>
+        <v>30.5</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -19400,30 +19406,30 @@
         <v>299</v>
       </c>
       <c r="C15">
-        <v>123</v>
+        <v>2580</v>
       </c>
       <c r="D15">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E15" t="s">
         <v>8</v>
       </c>
       <c r="F15" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G15">
-        <v>180</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B16" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C16">
-        <v>4016</v>
+        <v>123</v>
       </c>
       <c r="D16">
         <v>25</v>
@@ -19435,7 +19441,7 @@
         <v>32</v>
       </c>
       <c r="G16">
-        <v>148</v>
+        <v>180</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -19446,10 +19452,10 @@
         <v>301</v>
       </c>
       <c r="C17">
-        <v>4017</v>
+        <v>4016</v>
       </c>
       <c r="D17">
-        <v>45.36</v>
+        <v>25</v>
       </c>
       <c r="E17" t="s">
         <v>8</v>
@@ -19458,7 +19464,7 @@
         <v>32</v>
       </c>
       <c r="G17">
-        <v>268.5</v>
+        <v>148</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -19469,10 +19475,10 @@
         <v>301</v>
       </c>
       <c r="C18">
-        <v>210</v>
+        <v>4017</v>
       </c>
       <c r="D18">
-        <v>5</v>
+        <v>45.36</v>
       </c>
       <c r="E18" t="s">
         <v>8</v>
@@ -19481,21 +19487,21 @@
         <v>32</v>
       </c>
       <c r="G18">
-        <v>31.5</v>
+        <v>268.5</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B19" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C19">
-        <v>4545</v>
+        <v>210</v>
       </c>
       <c r="D19">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E19" t="s">
         <v>8</v>
@@ -19504,7 +19510,7 @@
         <v>32</v>
       </c>
       <c r="G19">
-        <v>590</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -19515,42 +19521,42 @@
         <v>303</v>
       </c>
       <c r="C20">
-        <v>3363</v>
+        <v>4545</v>
       </c>
       <c r="D20">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E20" t="s">
         <v>8</v>
       </c>
       <c r="F20" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G20">
-        <v>100.5</v>
+        <v>590</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B21" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C21">
-        <v>2482</v>
+        <v>3363</v>
       </c>
       <c r="D21">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E21" t="s">
         <v>8</v>
       </c>
       <c r="F21" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G21">
-        <v>540</v>
+        <v>100.5</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -19561,33 +19567,33 @@
         <v>305</v>
       </c>
       <c r="C22">
-        <v>34</v>
+        <v>2482</v>
       </c>
       <c r="D22">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E22" t="s">
         <v>8</v>
       </c>
       <c r="F22" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G22">
-        <v>92</v>
+        <v>540</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B23" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C23">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="D23">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E23" t="s">
         <v>8</v>
@@ -19596,7 +19602,7 @@
         <v>13</v>
       </c>
       <c r="G23">
-        <v>540</v>
+        <v>92</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -19607,33 +19613,33 @@
         <v>307</v>
       </c>
       <c r="C24">
-        <v>114</v>
+        <v>89</v>
       </c>
       <c r="D24">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E24" t="s">
         <v>8</v>
       </c>
       <c r="F24" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G24">
-        <v>92</v>
+        <v>540</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B25" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C25">
-        <v>2486</v>
+        <v>114</v>
       </c>
       <c r="D25">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E25" t="s">
         <v>8</v>
@@ -19642,7 +19648,7 @@
         <v>32</v>
       </c>
       <c r="G25">
-        <v>540</v>
+        <v>92</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -19653,42 +19659,42 @@
         <v>309</v>
       </c>
       <c r="C26">
-        <v>2241</v>
+        <v>2486</v>
       </c>
       <c r="D26">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E26" t="s">
         <v>8</v>
       </c>
       <c r="F26" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G26">
-        <v>92</v>
+        <v>540</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B27" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C27">
-        <v>2487</v>
+        <v>2241</v>
       </c>
       <c r="D27">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E27" t="s">
         <v>8</v>
       </c>
       <c r="F27" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G27">
-        <v>540</v>
+        <v>92</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -19699,42 +19705,42 @@
         <v>311</v>
       </c>
       <c r="C28">
-        <v>23</v>
+        <v>2487</v>
       </c>
       <c r="D28">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E28" t="s">
         <v>8</v>
       </c>
       <c r="F28" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G28">
-        <v>92</v>
+        <v>540</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B29" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C29">
-        <v>2260</v>
+        <v>23</v>
       </c>
       <c r="D29">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E29" t="s">
         <v>8</v>
       </c>
       <c r="F29" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G29">
-        <v>430</v>
+        <v>92</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -19745,10 +19751,10 @@
         <v>313</v>
       </c>
       <c r="C30">
-        <v>214</v>
+        <v>2260</v>
       </c>
       <c r="D30">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E30" t="s">
         <v>8</v>
@@ -19757,21 +19763,21 @@
         <v>32</v>
       </c>
       <c r="G30">
-        <v>73.5</v>
+        <v>430</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B31" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C31">
-        <v>28</v>
+        <v>214</v>
       </c>
       <c r="D31">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E31" t="s">
         <v>8</v>
@@ -19780,7 +19786,7 @@
         <v>32</v>
       </c>
       <c r="G31">
-        <v>270</v>
+        <v>73.5</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -19791,30 +19797,30 @@
         <v>315</v>
       </c>
       <c r="C32">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="D32">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E32" t="s">
         <v>8</v>
       </c>
       <c r="F32" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G32">
-        <v>47</v>
+        <v>270</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B33" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C33">
-        <v>2302</v>
+        <v>68</v>
       </c>
       <c r="D33">
         <v>5</v>
@@ -19823,10 +19829,10 @@
         <v>8</v>
       </c>
       <c r="F33" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G33">
-        <v>54.5</v>
+        <v>47</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -19837,10 +19843,10 @@
         <v>317</v>
       </c>
       <c r="C34">
-        <v>320</v>
+        <v>2302</v>
       </c>
       <c r="D34">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E34" t="s">
         <v>8</v>
@@ -19849,21 +19855,21 @@
         <v>32</v>
       </c>
       <c r="G34">
-        <v>315</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B35" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C35">
-        <v>3479</v>
+        <v>320</v>
       </c>
       <c r="D35">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="E35" t="s">
         <v>8</v>
@@ -19872,7 +19878,7 @@
         <v>32</v>
       </c>
       <c r="G35">
-        <v>356</v>
+        <v>315</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -19883,10 +19889,10 @@
         <v>319</v>
       </c>
       <c r="C36">
-        <v>130</v>
+        <v>3479</v>
       </c>
       <c r="D36">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="E36" t="s">
         <v>8</v>
@@ -19895,7 +19901,7 @@
         <v>32</v>
       </c>
       <c r="G36">
-        <v>178</v>
+        <v>356</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -19906,42 +19912,42 @@
         <v>319</v>
       </c>
       <c r="C37">
-        <v>2464</v>
+        <v>130</v>
       </c>
       <c r="D37">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E37" t="s">
         <v>8</v>
       </c>
       <c r="F37" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G37">
-        <v>37.5</v>
+        <v>178</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B38" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C38">
-        <v>101</v>
+        <v>2464</v>
       </c>
       <c r="D38">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E38" t="s">
         <v>8</v>
       </c>
       <c r="F38" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G38">
-        <v>360</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -19952,30 +19958,30 @@
         <v>321</v>
       </c>
       <c r="C39">
-        <v>2465</v>
+        <v>101</v>
       </c>
       <c r="D39">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E39" t="s">
         <v>8</v>
       </c>
       <c r="F39" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G39">
-        <v>62</v>
+        <v>360</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B40" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C40">
-        <v>65</v>
+        <v>2465</v>
       </c>
       <c r="D40">
         <v>5</v>
@@ -19987,7 +19993,7 @@
         <v>13</v>
       </c>
       <c r="G40">
-        <v>24.5</v>
+        <v>62</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
@@ -19998,19 +20004,19 @@
         <v>323</v>
       </c>
       <c r="C41">
-        <v>2624</v>
+        <v>65</v>
       </c>
       <c r="D41">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E41" t="s">
         <v>8</v>
       </c>
       <c r="F41" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G41">
-        <v>135</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
@@ -20021,10 +20027,10 @@
         <v>323</v>
       </c>
       <c r="C42">
-        <v>119</v>
+        <v>2624</v>
       </c>
       <c r="D42">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="E42" t="s">
         <v>8</v>
@@ -20033,21 +20039,21 @@
         <v>32</v>
       </c>
       <c r="G42">
-        <v>270</v>
+        <v>135</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B43" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C43">
-        <v>2834</v>
+        <v>119</v>
       </c>
       <c r="D43">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="E43" t="s">
         <v>8</v>
@@ -20056,7 +20062,7 @@
         <v>32</v>
       </c>
       <c r="G43">
-        <v>123</v>
+        <v>270</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
@@ -20067,10 +20073,10 @@
         <v>325</v>
       </c>
       <c r="C44">
-        <v>3621</v>
+        <v>2834</v>
       </c>
       <c r="D44">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E44" t="s">
         <v>8</v>
@@ -20079,7 +20085,7 @@
         <v>32</v>
       </c>
       <c r="G44">
-        <v>102.5</v>
+        <v>123</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
@@ -20090,10 +20096,10 @@
         <v>325</v>
       </c>
       <c r="C45">
-        <v>141</v>
+        <v>3621</v>
       </c>
       <c r="D45">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E45" t="s">
         <v>8</v>
@@ -20102,21 +20108,21 @@
         <v>32</v>
       </c>
       <c r="G45">
-        <v>23</v>
+        <v>102.5</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B46" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C46">
-        <v>3025</v>
+        <v>141</v>
       </c>
       <c r="D46">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E46" t="s">
         <v>8</v>
@@ -20125,7 +20131,7 @@
         <v>32</v>
       </c>
       <c r="G46">
-        <v>200</v>
+        <v>23</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
@@ -20136,42 +20142,42 @@
         <v>327</v>
       </c>
       <c r="C47">
-        <v>2543</v>
+        <v>3025</v>
       </c>
       <c r="D47">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E47" t="s">
         <v>8</v>
       </c>
       <c r="F47" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G47">
-        <v>35.5</v>
+        <v>200</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="B48" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C48">
-        <v>98</v>
+        <v>2543</v>
       </c>
       <c r="D48">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E48" t="s">
         <v>8</v>
       </c>
       <c r="F48" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G48">
-        <v>320</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -20182,10 +20188,10 @@
         <v>329</v>
       </c>
       <c r="C49">
-        <v>35</v>
+        <v>98</v>
       </c>
       <c r="D49">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E49" t="s">
         <v>8</v>
@@ -20194,21 +20200,21 @@
         <v>32</v>
       </c>
       <c r="G49">
-        <v>55.5</v>
+        <v>320</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B50" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C50">
-        <v>2353</v>
+        <v>35</v>
       </c>
       <c r="D50">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E50" t="s">
         <v>8</v>
@@ -20217,7 +20223,7 @@
         <v>32</v>
       </c>
       <c r="G50">
-        <v>362.5</v>
+        <v>55.5</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
@@ -20228,42 +20234,42 @@
         <v>331</v>
       </c>
       <c r="C51">
-        <v>2466</v>
+        <v>2353</v>
       </c>
       <c r="D51">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E51" t="s">
         <v>8</v>
       </c>
       <c r="F51" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G51">
-        <v>74.5</v>
+        <v>362.5</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B52" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C52">
-        <v>3089</v>
+        <v>2466</v>
       </c>
       <c r="D52">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E52" t="s">
         <v>8</v>
       </c>
       <c r="F52" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G52">
-        <v>255</v>
+        <v>74.5</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
@@ -20274,10 +20280,10 @@
         <v>333</v>
       </c>
       <c r="C53">
-        <v>2666</v>
+        <v>3089</v>
       </c>
       <c r="D53">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E53" t="s">
         <v>8</v>
@@ -20286,7 +20292,7 @@
         <v>32</v>
       </c>
       <c r="G53">
-        <v>212.5</v>
+        <v>255</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
@@ -20297,42 +20303,42 @@
         <v>333</v>
       </c>
       <c r="C54">
-        <v>2667</v>
+        <v>2666</v>
       </c>
       <c r="D54">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E54" t="s">
         <v>8</v>
       </c>
       <c r="F54" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G54">
-        <v>44.5</v>
+        <v>212.5</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B55" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C55">
-        <v>3478</v>
+        <v>2667</v>
       </c>
       <c r="D55">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="E55" t="s">
         <v>8</v>
       </c>
       <c r="F55" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G55">
-        <v>350</v>
+        <v>44.5</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
@@ -20343,10 +20349,10 @@
         <v>335</v>
       </c>
       <c r="C56">
-        <v>190</v>
+        <v>3478</v>
       </c>
       <c r="D56">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="E56" t="s">
         <v>8</v>
@@ -20355,7 +20361,7 @@
         <v>32</v>
       </c>
       <c r="G56">
-        <v>175</v>
+        <v>350</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
@@ -20366,42 +20372,42 @@
         <v>335</v>
       </c>
       <c r="C57">
-        <v>2335</v>
+        <v>190</v>
       </c>
       <c r="D57">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E57" t="s">
         <v>8</v>
       </c>
       <c r="F57" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G57">
-        <v>31</v>
+        <v>175</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B58" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C58">
-        <v>3446</v>
+        <v>2335</v>
       </c>
       <c r="D58">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E58" t="s">
         <v>8</v>
       </c>
       <c r="F58" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G58">
-        <v>275</v>
+        <v>31</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
@@ -20412,42 +20418,42 @@
         <v>337</v>
       </c>
       <c r="C59">
-        <v>3447</v>
+        <v>3446</v>
       </c>
       <c r="D59">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E59" t="s">
         <v>8</v>
       </c>
       <c r="F59" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G59">
-        <v>57</v>
+        <v>275</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B60" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C60">
-        <v>100</v>
+        <v>3447</v>
       </c>
       <c r="D60">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E60" t="s">
         <v>8</v>
       </c>
       <c r="F60" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G60">
-        <v>280</v>
+        <v>57</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
@@ -20458,10 +20464,10 @@
         <v>339</v>
       </c>
       <c r="C61">
-        <v>136</v>
+        <v>100</v>
       </c>
       <c r="D61">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E61" t="s">
         <v>8</v>
@@ -20470,21 +20476,21 @@
         <v>32</v>
       </c>
       <c r="G61">
-        <v>48.5</v>
+        <v>280</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B62" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C62">
-        <v>259</v>
+        <v>136</v>
       </c>
       <c r="D62">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E62" t="s">
         <v>8</v>
@@ -20493,7 +20499,7 @@
         <v>32</v>
       </c>
       <c r="G62">
-        <v>375</v>
+        <v>48.5</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
@@ -20504,42 +20510,42 @@
         <v>341</v>
       </c>
       <c r="C63">
-        <v>2319</v>
+        <v>259</v>
       </c>
       <c r="D63">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E63" t="s">
         <v>8</v>
       </c>
       <c r="F63" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G63">
-        <v>64.5</v>
+        <v>375</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B64" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C64">
-        <v>125</v>
+        <v>2319</v>
       </c>
       <c r="D64">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E64" t="s">
         <v>8</v>
       </c>
       <c r="F64" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G64">
-        <v>330</v>
+        <v>64.5</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
@@ -20550,42 +20556,42 @@
         <v>343</v>
       </c>
       <c r="C65">
-        <v>2468</v>
+        <v>125</v>
       </c>
       <c r="D65">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E65" t="s">
         <v>8</v>
       </c>
       <c r="F65" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G65">
-        <v>57</v>
+        <v>330</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B66" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C66">
-        <v>3670</v>
+        <v>2468</v>
       </c>
       <c r="D66">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E66" t="s">
         <v>8</v>
       </c>
       <c r="F66" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G66">
-        <v>285</v>
+        <v>57</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
@@ -20596,10 +20602,10 @@
         <v>345</v>
       </c>
       <c r="C67">
-        <v>3740</v>
+        <v>3670</v>
       </c>
       <c r="D67">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E67" t="s">
         <v>8</v>
@@ -20608,7 +20614,7 @@
         <v>32</v>
       </c>
       <c r="G67">
-        <v>237.5</v>
+        <v>285</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
@@ -20619,42 +20625,42 @@
         <v>345</v>
       </c>
       <c r="C68">
-        <v>2469</v>
+        <v>3740</v>
       </c>
       <c r="D68">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E68" t="s">
         <v>8</v>
       </c>
       <c r="F68" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G68">
-        <v>49.5</v>
+        <v>237.5</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B69" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C69">
-        <v>3006</v>
+        <v>2469</v>
       </c>
       <c r="D69">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E69" t="s">
         <v>8</v>
       </c>
       <c r="F69" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G69">
-        <v>312.5</v>
+        <v>49.5</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
@@ -20665,42 +20671,42 @@
         <v>347</v>
       </c>
       <c r="C70">
-        <v>3007</v>
+        <v>3006</v>
       </c>
       <c r="D70">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E70" t="s">
         <v>8</v>
       </c>
       <c r="F70" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G70">
-        <v>64.5</v>
+        <v>312.5</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B71" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C71">
-        <v>117</v>
+        <v>3007</v>
       </c>
       <c r="D71">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E71" t="s">
         <v>8</v>
       </c>
       <c r="F71" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G71">
-        <v>300</v>
+        <v>64.5</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
@@ -20711,42 +20717,42 @@
         <v>349</v>
       </c>
       <c r="C72">
-        <v>2320</v>
+        <v>117</v>
       </c>
       <c r="D72">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E72" t="s">
         <v>8</v>
       </c>
       <c r="F72" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G72">
-        <v>62</v>
+        <v>300</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="B73" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C73">
-        <v>60</v>
+        <v>2320</v>
       </c>
       <c r="D73">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E73" t="s">
         <v>8</v>
       </c>
       <c r="F73" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G73">
-        <v>180</v>
+        <v>62</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
@@ -20757,42 +20763,42 @@
         <v>351</v>
       </c>
       <c r="C74">
-        <v>2321</v>
+        <v>60</v>
       </c>
       <c r="D74">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E74" t="s">
         <v>8</v>
       </c>
       <c r="F74" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G74">
-        <v>38</v>
+        <v>180</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B75" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C75">
-        <v>211</v>
+        <v>2321</v>
       </c>
       <c r="D75">
-        <v>22.68</v>
+        <v>5</v>
       </c>
       <c r="E75" t="s">
         <v>8</v>
       </c>
       <c r="F75" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G75">
-        <v>187.5</v>
+        <v>38</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
@@ -20803,10 +20809,10 @@
         <v>353</v>
       </c>
       <c r="C76">
-        <v>41</v>
+        <v>211</v>
       </c>
       <c r="D76">
-        <v>45.36</v>
+        <v>22.68</v>
       </c>
       <c r="E76" t="s">
         <v>8</v>
@@ -20815,7 +20821,7 @@
         <v>32</v>
       </c>
       <c r="G76">
-        <v>375</v>
+        <v>187.5</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
@@ -20826,42 +20832,42 @@
         <v>353</v>
       </c>
       <c r="C77">
-        <v>2322</v>
+        <v>41</v>
       </c>
       <c r="D77">
-        <v>5</v>
+        <v>45.36</v>
       </c>
       <c r="E77" t="s">
         <v>8</v>
       </c>
       <c r="F77" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G77">
-        <v>43.5</v>
+        <v>375</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B78" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C78">
-        <v>67</v>
+        <v>2322</v>
       </c>
       <c r="D78">
-        <v>45.36</v>
+        <v>5</v>
       </c>
       <c r="E78" t="s">
         <v>8</v>
       </c>
       <c r="F78" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G78">
-        <v>626</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
@@ -20872,10 +20878,10 @@
         <v>355</v>
       </c>
       <c r="C79">
-        <v>2244</v>
+        <v>67</v>
       </c>
       <c r="D79">
-        <v>22.68</v>
+        <v>45.36</v>
       </c>
       <c r="E79" t="s">
         <v>8</v>
@@ -20884,7 +20890,7 @@
         <v>32</v>
       </c>
       <c r="G79">
-        <v>313</v>
+        <v>626</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
@@ -20895,65 +20901,65 @@
         <v>355</v>
       </c>
       <c r="C80">
-        <v>2488</v>
+        <v>2244</v>
       </c>
       <c r="D80">
-        <v>5</v>
+        <v>22.68</v>
       </c>
       <c r="E80" t="s">
         <v>8</v>
       </c>
       <c r="F80" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G80">
-        <v>71</v>
+        <v>313</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B81" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C81">
-        <v>520</v>
+        <v>2488</v>
       </c>
       <c r="D81">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E81" t="s">
         <v>8</v>
       </c>
       <c r="F81" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G81">
-        <v>52</v>
+        <v>71</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B82" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C82">
-        <v>4546</v>
+        <v>520</v>
       </c>
       <c r="D82">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E82" t="s">
         <v>8</v>
       </c>
       <c r="F82" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G82">
-        <v>182</v>
+        <v>52</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
@@ -20964,19 +20970,19 @@
         <v>359</v>
       </c>
       <c r="C83">
-        <v>3695</v>
+        <v>4546</v>
       </c>
       <c r="D83">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E83" t="s">
         <v>8</v>
       </c>
       <c r="F83" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G83">
-        <v>350</v>
+        <v>182</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
@@ -20987,10 +20993,10 @@
         <v>359</v>
       </c>
       <c r="C84">
-        <v>3097</v>
+        <v>3695</v>
       </c>
       <c r="D84">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E84" t="s">
         <v>8</v>
@@ -20999,7 +21005,7 @@
         <v>32</v>
       </c>
       <c r="G84">
-        <v>700</v>
+        <v>350</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
@@ -21010,56 +21016,56 @@
         <v>359</v>
       </c>
       <c r="C85">
-        <v>2460</v>
+        <v>3097</v>
       </c>
       <c r="D85">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="E85" t="s">
         <v>8</v>
       </c>
       <c r="F85" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G85">
-        <v>106</v>
+        <v>700</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B86" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C86">
-        <v>3110</v>
+        <v>2460</v>
       </c>
       <c r="D86">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="E86" t="s">
         <v>8</v>
       </c>
       <c r="F86" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G86">
-        <v>87</v>
+        <v>106</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B87" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="C87">
-        <v>135</v>
+        <v>3110</v>
       </c>
       <c r="D87">
-        <v>22.68</v>
+        <v>25</v>
       </c>
       <c r="E87" t="s">
         <v>8</v>
@@ -21068,21 +21074,21 @@
         <v>32</v>
       </c>
       <c r="G87">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B88" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C88">
-        <v>2463</v>
+        <v>135</v>
       </c>
       <c r="D88">
-        <v>5</v>
+        <v>22.68</v>
       </c>
       <c r="E88" t="s">
         <v>8</v>
@@ -21091,21 +21097,21 @@
         <v>32</v>
       </c>
       <c r="G88">
-        <v>21</v>
+        <v>85</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B89" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C89">
-        <v>55</v>
+        <v>2463</v>
       </c>
       <c r="D89">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E89" t="s">
         <v>8</v>
@@ -21114,7 +21120,7 @@
         <v>32</v>
       </c>
       <c r="G89">
-        <v>114</v>
+        <v>21</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
@@ -21125,10 +21131,10 @@
         <v>367</v>
       </c>
       <c r="C90">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D90">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E90" t="s">
         <v>8</v>
@@ -21137,7 +21143,7 @@
         <v>32</v>
       </c>
       <c r="G90">
-        <v>27</v>
+        <v>114</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
@@ -21148,10 +21154,10 @@
         <v>367</v>
       </c>
       <c r="C91">
-        <v>201</v>
+        <v>51</v>
       </c>
       <c r="D91">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="E91" t="s">
         <v>8</v>
@@ -21160,21 +21166,21 @@
         <v>32</v>
       </c>
       <c r="G91">
-        <v>228</v>
+        <v>27</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B92" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C92">
-        <v>4223</v>
+        <v>201</v>
       </c>
       <c r="D92">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="E92" t="s">
         <v>8</v>
@@ -21183,7 +21189,7 @@
         <v>32</v>
       </c>
       <c r="G92">
-        <v>125</v>
+        <v>228</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
@@ -21194,18 +21200,41 @@
         <v>369</v>
       </c>
       <c r="C93">
+        <v>4223</v>
+      </c>
+      <c r="D93">
+        <v>25</v>
+      </c>
+      <c r="E93" t="s">
+        <v>8</v>
+      </c>
+      <c r="F93" t="s">
+        <v>32</v>
+      </c>
+      <c r="G93">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>368</v>
+      </c>
+      <c r="B94" t="s">
+        <v>369</v>
+      </c>
+      <c r="C94">
         <v>4224</v>
       </c>
-      <c r="D93">
-        <v>5</v>
-      </c>
-      <c r="E93" t="s">
-        <v>8</v>
-      </c>
-      <c r="F93" t="s">
-        <v>13</v>
-      </c>
-      <c r="G93">
+      <c r="D94">
+        <v>5</v>
+      </c>
+      <c r="E94" t="s">
+        <v>8</v>
+      </c>
+      <c r="F94" t="s">
+        <v>13</v>
+      </c>
+      <c r="G94">
         <v>27</v>
       </c>
     </row>
@@ -24117,7 +24146,7 @@
         <v>13</v>
       </c>
       <c r="G88">
-        <v>200</v>
+        <v>180</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
@@ -24140,7 +24169,7 @@
         <v>13</v>
       </c>
       <c r="G89">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Atualizando itens em destaque
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodos.xlsx
+++ b/data/ProdutosFomatodos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\astra\Documents\lista-bourached\Lista-de-Produtos-Bourached\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D579D5AC-4BA5-42C8-8252-EFAFB2673F47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFF3AF5A-9580-46BE-A06E-AF672E9AEAD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11685" yWindow="0" windowWidth="17220" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4005" yWindow="420" windowWidth="13710" windowHeight="13920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="promoçoes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3698" uniqueCount="1123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3786" uniqueCount="1123">
   <si>
     <t>produto_grupo</t>
   </si>
@@ -3809,7 +3809,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
@@ -4030,16 +4030,16 @@
     </row>
     <row r="10" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>274</v>
+        <v>1060</v>
       </c>
       <c r="B10" t="s">
-        <v>275</v>
+        <v>1061</v>
       </c>
       <c r="C10" s="3">
-        <v>2825</v>
+        <v>2283</v>
       </c>
       <c r="D10" s="3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E10" t="s">
         <v>29</v>
@@ -4048,21 +4048,21 @@
         <v>10</v>
       </c>
       <c r="G10" s="3">
-        <v>25</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>276</v>
+        <v>1062</v>
       </c>
       <c r="B11" t="s">
-        <v>277</v>
+        <v>1063</v>
       </c>
       <c r="C11" s="3">
-        <v>2828</v>
+        <v>4255</v>
       </c>
       <c r="D11" s="3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E11" t="s">
         <v>29</v>
@@ -4071,21 +4071,21 @@
         <v>10</v>
       </c>
       <c r="G11" s="3">
-        <v>25</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>278</v>
+        <v>1090</v>
       </c>
       <c r="B12" t="s">
-        <v>279</v>
+        <v>1091</v>
       </c>
       <c r="C12" s="3">
-        <v>2826</v>
+        <v>3081</v>
       </c>
       <c r="D12" s="3">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E12" t="s">
         <v>29</v>
@@ -4094,21 +4094,21 @@
         <v>10</v>
       </c>
       <c r="G12" s="3">
-        <v>25</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>280</v>
+        <v>1090</v>
       </c>
       <c r="B13" t="s">
-        <v>281</v>
+        <v>1091</v>
       </c>
       <c r="C13" s="3">
-        <v>3058</v>
+        <v>3818</v>
       </c>
       <c r="D13" s="3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E13" t="s">
         <v>29</v>
@@ -4116,22 +4116,22 @@
       <c r="F13" t="s">
         <v>10</v>
       </c>
-      <c r="G13" s="3">
-        <v>25</v>
+      <c r="G13" s="4">
+        <v>72.5</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>282</v>
+        <v>1092</v>
       </c>
       <c r="B14" t="s">
-        <v>283</v>
+        <v>1093</v>
       </c>
       <c r="C14" s="3">
-        <v>3059</v>
+        <v>2534</v>
       </c>
       <c r="D14" s="3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E14" t="s">
         <v>29</v>
@@ -4139,22 +4139,22 @@
       <c r="F14" t="s">
         <v>10</v>
       </c>
-      <c r="G14" s="3">
-        <v>25</v>
+      <c r="G14" s="4">
+        <v>72.5</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>284</v>
+        <v>1092</v>
       </c>
       <c r="B15" t="s">
-        <v>285</v>
+        <v>1093</v>
       </c>
       <c r="C15" s="3">
-        <v>2829</v>
+        <v>2234</v>
       </c>
       <c r="D15" s="3">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E15" t="s">
         <v>29</v>
@@ -4163,21 +4163,21 @@
         <v>10</v>
       </c>
       <c r="G15" s="3">
-        <v>25</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>286</v>
+        <v>1094</v>
       </c>
       <c r="B16" t="s">
-        <v>287</v>
+        <v>1095</v>
       </c>
       <c r="C16" s="3">
-        <v>4126</v>
+        <v>2238</v>
       </c>
       <c r="D16" s="3">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
@@ -4186,21 +4186,21 @@
         <v>10</v>
       </c>
       <c r="G16" s="3">
-        <v>25</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>288</v>
+        <v>1094</v>
       </c>
       <c r="B17" t="s">
-        <v>289</v>
+        <v>1096</v>
       </c>
       <c r="C17" s="3">
-        <v>2827</v>
+        <v>2535</v>
       </c>
       <c r="D17" s="3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E17" t="s">
         <v>29</v>
@@ -4208,45 +4208,45 @@
       <c r="F17" t="s">
         <v>10</v>
       </c>
-      <c r="G17" s="3">
-        <v>25</v>
+      <c r="G17" s="4">
+        <v>72.5</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>290</v>
+        <v>1099</v>
       </c>
       <c r="B18" t="s">
-        <v>291</v>
+        <v>1100</v>
       </c>
       <c r="C18" s="3">
-        <v>3801</v>
+        <v>2236</v>
       </c>
       <c r="D18" s="3">
-        <v>500</v>
+        <v>10</v>
       </c>
       <c r="E18" t="s">
-        <v>253</v>
+        <v>29</v>
       </c>
       <c r="F18" t="s">
         <v>10</v>
       </c>
       <c r="G18" s="3">
-        <v>25</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>296</v>
+        <v>1099</v>
       </c>
       <c r="B19" t="s">
-        <v>297</v>
+        <v>1100</v>
       </c>
       <c r="C19" s="3">
-        <v>3764</v>
+        <v>2546</v>
       </c>
       <c r="D19" s="3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E19" t="s">
         <v>29</v>
@@ -4254,191 +4254,697 @@
       <c r="F19" t="s">
         <v>10</v>
       </c>
-      <c r="G19" s="3">
-        <v>81</v>
+      <c r="G19" s="4">
+        <v>72.5</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>313</v>
+        <v>1101</v>
       </c>
       <c r="B20" t="s">
-        <v>314</v>
+        <v>1102</v>
       </c>
       <c r="C20" s="3">
-        <v>3402</v>
+        <v>2232</v>
       </c>
       <c r="D20" s="3">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E20" t="s">
-        <v>306</v>
+        <v>29</v>
       </c>
       <c r="F20" t="s">
-        <v>49</v>
-      </c>
-      <c r="G20" s="4">
-        <v>46.5</v>
+        <v>10</v>
+      </c>
+      <c r="G20" s="3">
+        <v>139</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>313</v>
+        <v>1101</v>
       </c>
       <c r="B21" t="s">
-        <v>314</v>
+        <v>1102</v>
       </c>
       <c r="C21" s="3">
-        <v>3401</v>
+        <v>2536</v>
       </c>
       <c r="D21" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E21" t="s">
-        <v>315</v>
+        <v>29</v>
       </c>
       <c r="F21" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="G21" s="4">
-        <v>66.5</v>
+        <v>72.5</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>313</v>
+        <v>1066</v>
       </c>
       <c r="B22" t="s">
-        <v>314</v>
+        <v>1067</v>
       </c>
       <c r="C22" s="3">
-        <v>3403</v>
+        <v>2452</v>
       </c>
       <c r="D22" s="3">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E22" t="s">
-        <v>308</v>
+        <v>29</v>
       </c>
       <c r="F22" t="s">
-        <v>49</v>
-      </c>
-      <c r="G22" s="4">
-        <v>38.5</v>
+        <v>10</v>
+      </c>
+      <c r="G22" s="3">
+        <v>76</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>316</v>
+        <v>1066</v>
       </c>
       <c r="B23" t="s">
-        <v>317</v>
+        <v>1067</v>
       </c>
       <c r="C23" s="3">
-        <v>4032</v>
+        <v>150</v>
       </c>
       <c r="D23" s="3">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E23" t="s">
-        <v>318</v>
+        <v>29</v>
       </c>
       <c r="F23" t="s">
-        <v>49</v>
-      </c>
-      <c r="G23" s="4">
-        <v>57.5</v>
+        <v>156</v>
+      </c>
+      <c r="G23" s="3">
+        <v>190</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>319</v>
+        <v>1066</v>
       </c>
       <c r="B24" t="s">
-        <v>320</v>
+        <v>1067</v>
       </c>
       <c r="C24" s="3">
-        <v>4460</v>
+        <v>2453</v>
       </c>
       <c r="D24" s="3">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E24" t="s">
-        <v>318</v>
+        <v>29</v>
       </c>
       <c r="F24" t="s">
-        <v>49</v>
-      </c>
-      <c r="G24" s="4">
-        <v>57.5</v>
+        <v>10</v>
+      </c>
+      <c r="G24" s="3">
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>324</v>
+        <v>1068</v>
       </c>
       <c r="B25" t="s">
-        <v>325</v>
+        <v>1069</v>
       </c>
       <c r="C25" s="3">
-        <v>2551</v>
+        <v>2450</v>
       </c>
       <c r="D25" s="3">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E25" t="s">
-        <v>306</v>
+        <v>29</v>
       </c>
       <c r="F25" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="G25" s="3">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>326</v>
+        <v>1068</v>
       </c>
       <c r="B26" t="s">
-        <v>327</v>
+        <v>1069</v>
       </c>
       <c r="C26" s="3">
-        <v>2550</v>
+        <v>7</v>
       </c>
       <c r="D26" s="3">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="E26" t="s">
-        <v>328</v>
+        <v>29</v>
       </c>
       <c r="F26" t="s">
-        <v>49</v>
-      </c>
-      <c r="G26" s="4">
-        <v>25.5</v>
+        <v>156</v>
+      </c>
+      <c r="G26" s="3">
+        <v>190</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>1068</v>
+      </c>
+      <c r="B27" t="s">
+        <v>1069</v>
+      </c>
+      <c r="C27" s="3">
+        <v>2451</v>
+      </c>
+      <c r="D27" s="3">
+        <v>5</v>
+      </c>
+      <c r="E27" t="s">
+        <v>29</v>
+      </c>
+      <c r="F27" t="s">
+        <v>10</v>
+      </c>
+      <c r="G27" s="3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>1048</v>
+      </c>
+      <c r="B28" t="s">
+        <v>1049</v>
+      </c>
+      <c r="C28" s="3">
+        <v>2643</v>
+      </c>
+      <c r="D28" s="3">
+        <v>5</v>
+      </c>
+      <c r="E28" t="s">
+        <v>29</v>
+      </c>
+      <c r="F28" t="s">
+        <v>10</v>
+      </c>
+      <c r="G28" s="3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B29" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C29" s="3">
+        <v>2644</v>
+      </c>
+      <c r="D29" s="3">
+        <v>5</v>
+      </c>
+      <c r="E29" t="s">
+        <v>29</v>
+      </c>
+      <c r="F29" t="s">
+        <v>10</v>
+      </c>
+      <c r="G29" s="3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>1052</v>
+      </c>
+      <c r="B30" t="s">
+        <v>1053</v>
+      </c>
+      <c r="C30" s="3">
+        <v>2570</v>
+      </c>
+      <c r="D30" s="3">
+        <v>5</v>
+      </c>
+      <c r="E30" t="s">
+        <v>29</v>
+      </c>
+      <c r="F30" t="s">
+        <v>10</v>
+      </c>
+      <c r="G30" s="3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>1054</v>
+      </c>
+      <c r="B31" t="s">
+        <v>1055</v>
+      </c>
+      <c r="C31" s="3">
+        <v>3021</v>
+      </c>
+      <c r="D31" s="3">
+        <v>5</v>
+      </c>
+      <c r="E31" t="s">
+        <v>29</v>
+      </c>
+      <c r="F31" t="s">
+        <v>10</v>
+      </c>
+      <c r="G31" s="3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>274</v>
+      </c>
+      <c r="B32" t="s">
+        <v>275</v>
+      </c>
+      <c r="C32" s="3">
+        <v>2825</v>
+      </c>
+      <c r="D32" s="3">
+        <v>2</v>
+      </c>
+      <c r="E32" t="s">
+        <v>29</v>
+      </c>
+      <c r="F32" t="s">
+        <v>10</v>
+      </c>
+      <c r="G32" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>276</v>
+      </c>
+      <c r="B33" t="s">
+        <v>277</v>
+      </c>
+      <c r="C33" s="3">
+        <v>2828</v>
+      </c>
+      <c r="D33" s="3">
+        <v>2</v>
+      </c>
+      <c r="E33" t="s">
+        <v>29</v>
+      </c>
+      <c r="F33" t="s">
+        <v>10</v>
+      </c>
+      <c r="G33" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>278</v>
+      </c>
+      <c r="B34" t="s">
+        <v>279</v>
+      </c>
+      <c r="C34" s="3">
+        <v>2826</v>
+      </c>
+      <c r="D34" s="3">
+        <v>2</v>
+      </c>
+      <c r="E34" t="s">
+        <v>29</v>
+      </c>
+      <c r="F34" t="s">
+        <v>10</v>
+      </c>
+      <c r="G34" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>280</v>
+      </c>
+      <c r="B35" t="s">
+        <v>281</v>
+      </c>
+      <c r="C35" s="3">
+        <v>3058</v>
+      </c>
+      <c r="D35" s="3">
+        <v>2</v>
+      </c>
+      <c r="E35" t="s">
+        <v>29</v>
+      </c>
+      <c r="F35" t="s">
+        <v>10</v>
+      </c>
+      <c r="G35" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>282</v>
+      </c>
+      <c r="B36" t="s">
+        <v>283</v>
+      </c>
+      <c r="C36" s="3">
+        <v>3059</v>
+      </c>
+      <c r="D36" s="3">
+        <v>2</v>
+      </c>
+      <c r="E36" t="s">
+        <v>29</v>
+      </c>
+      <c r="F36" t="s">
+        <v>10</v>
+      </c>
+      <c r="G36" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>284</v>
+      </c>
+      <c r="B37" t="s">
+        <v>285</v>
+      </c>
+      <c r="C37" s="3">
+        <v>2829</v>
+      </c>
+      <c r="D37" s="3">
+        <v>2</v>
+      </c>
+      <c r="E37" t="s">
+        <v>29</v>
+      </c>
+      <c r="F37" t="s">
+        <v>10</v>
+      </c>
+      <c r="G37" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>286</v>
+      </c>
+      <c r="B38" t="s">
+        <v>287</v>
+      </c>
+      <c r="C38" s="3">
+        <v>4126</v>
+      </c>
+      <c r="D38" s="3">
+        <v>2</v>
+      </c>
+      <c r="E38" t="s">
+        <v>29</v>
+      </c>
+      <c r="F38" t="s">
+        <v>10</v>
+      </c>
+      <c r="G38" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>288</v>
+      </c>
+      <c r="B39" t="s">
+        <v>289</v>
+      </c>
+      <c r="C39" s="3">
+        <v>2827</v>
+      </c>
+      <c r="D39" s="3">
+        <v>2</v>
+      </c>
+      <c r="E39" t="s">
+        <v>29</v>
+      </c>
+      <c r="F39" t="s">
+        <v>10</v>
+      </c>
+      <c r="G39" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>290</v>
+      </c>
+      <c r="B40" t="s">
+        <v>291</v>
+      </c>
+      <c r="C40" s="3">
+        <v>3801</v>
+      </c>
+      <c r="D40" s="3">
+        <v>500</v>
+      </c>
+      <c r="E40" t="s">
+        <v>253</v>
+      </c>
+      <c r="F40" t="s">
+        <v>10</v>
+      </c>
+      <c r="G40" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>296</v>
+      </c>
+      <c r="B41" t="s">
+        <v>297</v>
+      </c>
+      <c r="C41" s="3">
+        <v>3764</v>
+      </c>
+      <c r="D41" s="3">
+        <v>2</v>
+      </c>
+      <c r="E41" t="s">
+        <v>29</v>
+      </c>
+      <c r="F41" t="s">
+        <v>10</v>
+      </c>
+      <c r="G41" s="3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>313</v>
+      </c>
+      <c r="B42" t="s">
+        <v>314</v>
+      </c>
+      <c r="C42" s="3">
+        <v>3402</v>
+      </c>
+      <c r="D42" s="3">
+        <v>6</v>
+      </c>
+      <c r="E42" t="s">
+        <v>306</v>
+      </c>
+      <c r="F42" t="s">
+        <v>49</v>
+      </c>
+      <c r="G42" s="4">
+        <v>46.5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>313</v>
+      </c>
+      <c r="B43" t="s">
+        <v>314</v>
+      </c>
+      <c r="C43" s="3">
+        <v>3401</v>
+      </c>
+      <c r="D43" s="3">
+        <v>6</v>
+      </c>
+      <c r="E43" t="s">
+        <v>315</v>
+      </c>
+      <c r="F43" t="s">
+        <v>49</v>
+      </c>
+      <c r="G43" s="4">
+        <v>66.5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>313</v>
+      </c>
+      <c r="B44" t="s">
+        <v>314</v>
+      </c>
+      <c r="C44" s="3">
+        <v>3403</v>
+      </c>
+      <c r="D44" s="3">
+        <v>12</v>
+      </c>
+      <c r="E44" t="s">
+        <v>308</v>
+      </c>
+      <c r="F44" t="s">
+        <v>49</v>
+      </c>
+      <c r="G44" s="4">
+        <v>38.5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>316</v>
+      </c>
+      <c r="B45" t="s">
+        <v>317</v>
+      </c>
+      <c r="C45" s="3">
+        <v>4032</v>
+      </c>
+      <c r="D45" s="3">
+        <v>12</v>
+      </c>
+      <c r="E45" t="s">
+        <v>318</v>
+      </c>
+      <c r="F45" t="s">
+        <v>49</v>
+      </c>
+      <c r="G45" s="4">
+        <v>57.5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>319</v>
+      </c>
+      <c r="B46" t="s">
+        <v>320</v>
+      </c>
+      <c r="C46" s="3">
+        <v>4460</v>
+      </c>
+      <c r="D46" s="3">
+        <v>12</v>
+      </c>
+      <c r="E46" t="s">
+        <v>318</v>
+      </c>
+      <c r="F46" t="s">
+        <v>49</v>
+      </c>
+      <c r="G46" s="4">
+        <v>57.5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>324</v>
+      </c>
+      <c r="B47" t="s">
+        <v>325</v>
+      </c>
+      <c r="C47" s="3">
+        <v>2551</v>
+      </c>
+      <c r="D47" s="3">
+        <v>12</v>
+      </c>
+      <c r="E47" t="s">
+        <v>306</v>
+      </c>
+      <c r="F47" t="s">
+        <v>49</v>
+      </c>
+      <c r="G47" s="3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>326</v>
+      </c>
+      <c r="B48" t="s">
+        <v>327</v>
+      </c>
+      <c r="C48" s="3">
+        <v>2550</v>
+      </c>
+      <c r="D48" s="3">
+        <v>6</v>
+      </c>
+      <c r="E48" t="s">
+        <v>328</v>
+      </c>
+      <c r="F48" t="s">
+        <v>49</v>
+      </c>
+      <c r="G48" s="4">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
         <v>329</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B49" t="s">
         <v>330</v>
       </c>
-      <c r="C27" s="3">
+      <c r="C49" s="3">
         <v>4383</v>
       </c>
-      <c r="D27" s="3">
+      <c r="D49" s="3">
         <v>12</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E49" t="s">
         <v>318</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F49" t="s">
         <v>49</v>
       </c>
-      <c r="G27" s="3">
+      <c r="G49" s="3">
         <v>53</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizando o design 20/07
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodos.xlsx
+++ b/data/ProdutosFomatodos.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="10"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="promoçoes"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3782" uniqueCount="1127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3718" uniqueCount="1128">
   <si>
     <t>produto_grupo</t>
   </si>
@@ -3412,6 +3412,9 @@
   </si>
   <si>
     <t>XEREM DE AMENDOIM</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -3488,7 +3491,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -3516,6 +3519,12 @@
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3819,7 +3828,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="6" width="15.290714285714287" customWidth="1" bestFit="1"/>
@@ -3877,30 +3886,30 @@
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="3" t="s">
-        <v>1068</v>
+        <v>1060</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1069</v>
+        <v>1061</v>
       </c>
       <c r="C3" s="4">
-        <v>103</v>
+        <v>2419</v>
       </c>
       <c r="D3" s="4">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="G3" s="4">
-        <v>215</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
+        <v>10</v>
+      </c>
+      <c r="G3" s="5">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="3" t="s">
         <v>838</v>
       </c>
@@ -3923,363 +3932,363 @@
         <v>87</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="3" t="s">
-        <v>266</v>
+        <v>1048</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>267</v>
+        <v>1049</v>
       </c>
       <c r="C5" s="4">
-        <v>3870</v>
+        <v>3821</v>
       </c>
       <c r="D5" s="4">
-        <v>500</v>
+        <v>25</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>255</v>
+        <v>29</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G5" s="4">
-        <v>22</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
+        <v>140</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="3" t="s">
-        <v>268</v>
+        <v>1048</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>269</v>
+        <v>1049</v>
       </c>
       <c r="C6" s="4">
-        <v>3701</v>
-      </c>
-      <c r="D6" s="4">
-        <v>500</v>
+        <v>2263</v>
+      </c>
+      <c r="D6" s="5">
+        <v>12.5</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>255</v>
+        <v>29</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G6" s="4">
-        <v>22</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+        <v>70</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="3" t="s">
-        <v>270</v>
+        <v>894</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>271</v>
+        <v>895</v>
       </c>
       <c r="C7" s="4">
-        <v>3800</v>
+        <v>92</v>
       </c>
       <c r="D7" s="4">
-        <v>500</v>
+        <v>20</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>255</v>
+        <v>29</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G7" s="4">
-        <v>22</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
+        <v>67</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="3" t="s">
-        <v>272</v>
+        <v>894</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>273</v>
+        <v>895</v>
       </c>
       <c r="C8" s="4">
-        <v>3725</v>
+        <v>2476</v>
       </c>
       <c r="D8" s="4">
-        <v>500</v>
+        <v>3</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>255</v>
+        <v>29</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="4">
-        <v>22</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
+      <c r="G8" s="5">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="3" t="s">
-        <v>274</v>
+        <v>892</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>275</v>
+        <v>893</v>
       </c>
       <c r="C9" s="4">
-        <v>3871</v>
+        <v>261</v>
       </c>
       <c r="D9" s="4">
-        <v>500</v>
+        <v>25</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>255</v>
+        <v>29</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G9" s="4">
+        <v>83</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+      <c r="A10" s="3" t="s">
+        <v>892</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>893</v>
+      </c>
+      <c r="C10" s="4">
+        <v>2475</v>
+      </c>
+      <c r="D10" s="4">
+        <v>5</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="5">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="A11" s="3" t="s">
+        <v>868</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>869</v>
+      </c>
+      <c r="C11" s="4">
+        <v>564</v>
+      </c>
+      <c r="D11" s="4">
+        <v>25</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="G11" s="4">
+        <v>118</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="A12" s="3" t="s">
+        <v>868</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>869</v>
+      </c>
+      <c r="C12" s="4">
+        <v>2256</v>
+      </c>
+      <c r="D12" s="4">
+        <v>3</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="5">
+        <v>16</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+      <c r="A13" s="3" t="s">
+        <v>714</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>715</v>
+      </c>
+      <c r="C13" s="4">
         <v>27</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
-      <c r="A10" s="3" t="s">
-        <v>1064</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>1065</v>
-      </c>
-      <c r="C10" s="4">
-        <v>2283</v>
-      </c>
-      <c r="D10" s="4">
-        <v>5</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G10" s="4">
-        <v>61</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
-      <c r="A11" s="3" t="s">
-        <v>1066</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>1067</v>
-      </c>
-      <c r="C11" s="4">
-        <v>4255</v>
-      </c>
-      <c r="D11" s="4">
-        <v>5</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G11" s="4">
-        <v>64</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
-      <c r="A12" s="3" t="s">
-        <v>1094</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>1095</v>
-      </c>
-      <c r="C12" s="4">
-        <v>3081</v>
-      </c>
-      <c r="D12" s="4">
-        <v>10</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G12" s="4">
-        <v>139</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
-      <c r="A13" s="3" t="s">
-        <v>1094</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>1095</v>
-      </c>
-      <c r="C13" s="4">
-        <v>3818</v>
-      </c>
       <c r="D13" s="4">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G13" s="5">
-        <v>72.5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
+        <v>158</v>
+      </c>
+      <c r="G13" s="4">
+        <v>110</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="3" t="s">
-        <v>1096</v>
+        <v>716</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1097</v>
+        <v>717</v>
       </c>
       <c r="C14" s="4">
-        <v>2534</v>
+        <v>2255</v>
       </c>
       <c r="D14" s="4">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G14" s="5">
-        <v>72.5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
+        <v>158</v>
+      </c>
+      <c r="G14" s="4">
+        <v>99</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="3" t="s">
-        <v>1096</v>
+        <v>544</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1097</v>
+        <v>545</v>
       </c>
       <c r="C15" s="4">
-        <v>2234</v>
+        <v>2350</v>
       </c>
       <c r="D15" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G15" s="4">
-        <v>139</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
+        <v>250</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="3" t="s">
-        <v>1098</v>
+        <v>552</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>1099</v>
-      </c>
-      <c r="C16" s="4">
-        <v>2238</v>
-      </c>
-      <c r="D16" s="4">
+        <v>553</v>
+      </c>
+      <c r="C16" s="10">
+        <v>2229</v>
+      </c>
+      <c r="D16" s="10">
         <v>10</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G16" s="4">
-        <v>139</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
+        <v>15</v>
+      </c>
+      <c r="G16" s="10">
+        <v>140</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="3" t="s">
-        <v>1098</v>
+        <v>518</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1100</v>
+        <v>519</v>
       </c>
       <c r="C17" s="4">
-        <v>2535</v>
+        <v>4400</v>
       </c>
       <c r="D17" s="4">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G17" s="5">
-        <v>72.5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
+        <v>158</v>
+      </c>
+      <c r="G17" s="4">
+        <v>1875</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="3" t="s">
-        <v>1103</v>
+        <v>518</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>1104</v>
+        <v>519</v>
       </c>
       <c r="C18" s="4">
-        <v>2236</v>
+        <v>2676</v>
       </c>
       <c r="D18" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G18" s="4">
-        <v>139</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
+        <v>378.5</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="3" t="s">
-        <v>1103</v>
+        <v>520</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1104</v>
+        <v>521</v>
       </c>
       <c r="C19" s="4">
-        <v>2546</v>
+        <v>571</v>
       </c>
       <c r="D19" s="4">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G19" s="5">
-        <v>72.5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
+        <v>158</v>
+      </c>
+      <c r="G19" s="4">
+        <v>287.5</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="3" t="s">
-        <v>1105</v>
+        <v>520</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>1106</v>
+        <v>521</v>
       </c>
       <c r="C20" s="4">
-        <v>2232</v>
+        <v>2245</v>
       </c>
       <c r="D20" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>29</v>
@@ -4288,21 +4297,21 @@
         <v>10</v>
       </c>
       <c r="G20" s="4">
-        <v>139</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
+        <v>60.5</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="3" t="s">
-        <v>1105</v>
+        <v>344</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>1106</v>
+        <v>345</v>
       </c>
       <c r="C21" s="4">
-        <v>2536</v>
+        <v>2259</v>
       </c>
       <c r="D21" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>29</v>
@@ -4311,21 +4320,21 @@
         <v>10</v>
       </c>
       <c r="G21" s="5">
-        <v>72.5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
+        <v>16</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="3" t="s">
-        <v>1070</v>
+        <v>348</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>1071</v>
+        <v>349</v>
       </c>
       <c r="C22" s="4">
-        <v>2452</v>
+        <v>2422</v>
       </c>
       <c r="D22" s="4">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>29</v>
@@ -4333,19 +4342,19 @@
       <c r="F22" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G22" s="4">
-        <v>76</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
+      <c r="G22" s="5">
+        <v>16</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="3" t="s">
-        <v>1070</v>
+        <v>348</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>1071</v>
+        <v>349</v>
       </c>
       <c r="C23" s="4">
-        <v>150</v>
+        <v>569</v>
       </c>
       <c r="D23" s="4">
         <v>25</v>
@@ -4357,41 +4366,41 @@
         <v>158</v>
       </c>
       <c r="G23" s="4">
-        <v>190</v>
+        <v>118</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="3" t="s">
-        <v>1070</v>
+        <v>344</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>1071</v>
+        <v>345</v>
       </c>
       <c r="C24" s="4">
-        <v>2453</v>
+        <v>282</v>
       </c>
       <c r="D24" s="4">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G24" s="4">
-        <v>41</v>
+        <v>118</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="3" t="s">
-        <v>1072</v>
+        <v>39</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>1073</v>
+        <v>40</v>
       </c>
       <c r="C25" s="4">
-        <v>2450</v>
+        <v>3123</v>
       </c>
       <c r="D25" s="4">
         <v>10</v>
@@ -4400,67 +4409,67 @@
         <v>29</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G25" s="4">
-        <v>76</v>
+        <v>121</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="3" t="s">
-        <v>1072</v>
+        <v>39</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>1073</v>
+        <v>40</v>
       </c>
       <c r="C26" s="4">
-        <v>7</v>
+        <v>2674</v>
       </c>
       <c r="D26" s="4">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="G26" s="4">
-        <v>190</v>
+        <v>10</v>
+      </c>
+      <c r="G26" s="5">
+        <v>60.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="3" t="s">
-        <v>1072</v>
+        <v>56</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>1073</v>
+        <v>57</v>
       </c>
       <c r="C27" s="4">
-        <v>2451</v>
+        <v>3124</v>
       </c>
       <c r="D27" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G27" s="4">
-        <v>41</v>
+        <v>161</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
       <c r="A28" s="3" t="s">
-        <v>1052</v>
+        <v>56</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>1053</v>
+        <v>57</v>
       </c>
       <c r="C28" s="4">
-        <v>2643</v>
+        <v>2824</v>
       </c>
       <c r="D28" s="4">
         <v>5</v>
@@ -4471,42 +4480,42 @@
       <c r="F28" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G28" s="4">
-        <v>68</v>
+      <c r="G28" s="5">
+        <v>80.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
       <c r="A29" s="3" t="s">
-        <v>1054</v>
+        <v>58</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>1055</v>
+        <v>59</v>
       </c>
       <c r="C29" s="4">
-        <v>2644</v>
+        <v>3130</v>
       </c>
       <c r="D29" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G29" s="4">
-        <v>70</v>
+        <v>138</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
       <c r="A30" s="3" t="s">
-        <v>1056</v>
+        <v>58</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>1057</v>
+        <v>59</v>
       </c>
       <c r="C30" s="4">
-        <v>2570</v>
+        <v>3131</v>
       </c>
       <c r="D30" s="4">
         <v>5</v>
@@ -4518,44 +4527,44 @@
         <v>10</v>
       </c>
       <c r="G30" s="4">
-        <v>57</v>
+        <v>69</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
       <c r="A31" s="3" t="s">
-        <v>1058</v>
+        <v>27</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>1059</v>
+        <v>28</v>
       </c>
       <c r="C31" s="4">
-        <v>3021</v>
+        <v>3438</v>
       </c>
       <c r="D31" s="4">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G31" s="4">
-        <v>63</v>
+        <v>228</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="3" t="s">
-        <v>276</v>
+        <v>27</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>277</v>
+        <v>28</v>
       </c>
       <c r="C32" s="4">
-        <v>2825</v>
+        <v>3434</v>
       </c>
       <c r="D32" s="4">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>29</v>
@@ -4564,399 +4573,34 @@
         <v>10</v>
       </c>
       <c r="G32" s="4">
-        <v>25</v>
+        <v>76</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
-      <c r="A33" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="C33" s="4">
-        <v>2828</v>
-      </c>
-      <c r="D33" s="4">
-        <v>2</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G33" s="4">
-        <v>25</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
-      <c r="A34" s="3" t="s">
-        <v>280</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="C34" s="4">
-        <v>2826</v>
-      </c>
-      <c r="D34" s="4">
-        <v>2</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G34" s="4">
-        <v>25</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
-      <c r="A35" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="C35" s="4">
-        <v>3058</v>
-      </c>
-      <c r="D35" s="4">
-        <v>2</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G35" s="4">
-        <v>25</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
-      <c r="A36" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="C36" s="4">
-        <v>3059</v>
-      </c>
-      <c r="D36" s="4">
-        <v>2</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G36" s="4">
-        <v>25</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
-      <c r="A37" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="C37" s="4">
-        <v>2829</v>
-      </c>
-      <c r="D37" s="4">
-        <v>2</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G37" s="4">
-        <v>25</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
-      <c r="A38" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C38" s="4">
-        <v>4126</v>
-      </c>
-      <c r="D38" s="4">
-        <v>2</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F38" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G38" s="4">
-        <v>25</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
-      <c r="A39" s="3" t="s">
-        <v>290</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="C39" s="4">
-        <v>2827</v>
-      </c>
-      <c r="D39" s="4">
-        <v>2</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G39" s="4">
-        <v>25</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
-      <c r="A40" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="C40" s="4">
-        <v>3801</v>
-      </c>
-      <c r="D40" s="4">
-        <v>500</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G40" s="4">
-        <v>25</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
-      <c r="A41" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="C41" s="4">
-        <v>3764</v>
-      </c>
-      <c r="D41" s="4">
-        <v>2</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G41" s="4">
-        <v>81</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
-      <c r="A42" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="C42" s="4">
-        <v>3402</v>
-      </c>
-      <c r="D42" s="4">
-        <v>6</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>308</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G42" s="5">
-        <v>46.5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
-      <c r="A43" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="C43" s="4">
-        <v>3401</v>
-      </c>
-      <c r="D43" s="4">
-        <v>6</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>317</v>
-      </c>
-      <c r="F43" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G43" s="5">
-        <v>66.5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
-      <c r="A44" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="C44" s="4">
-        <v>3403</v>
-      </c>
-      <c r="D44" s="4">
-        <v>12</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>310</v>
-      </c>
-      <c r="F44" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G44" s="5">
-        <v>38.5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
-      <c r="A45" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="C45" s="4">
-        <v>4032</v>
-      </c>
-      <c r="D45" s="4">
-        <v>12</v>
-      </c>
-      <c r="E45" s="3" t="s">
-        <v>320</v>
-      </c>
-      <c r="F45" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G45" s="5">
-        <v>57.5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
-      <c r="A46" s="3" t="s">
-        <v>321</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="C46" s="4">
-        <v>4460</v>
-      </c>
-      <c r="D46" s="4">
-        <v>12</v>
-      </c>
-      <c r="E46" s="3" t="s">
-        <v>320</v>
-      </c>
-      <c r="F46" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G46" s="5">
-        <v>57.5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
-      <c r="A47" s="3" t="s">
-        <v>326</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>327</v>
-      </c>
-      <c r="C47" s="4">
-        <v>2551</v>
-      </c>
-      <c r="D47" s="4">
-        <v>12</v>
-      </c>
-      <c r="E47" s="3" t="s">
-        <v>308</v>
-      </c>
-      <c r="F47" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G47" s="4">
-        <v>82</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
-      <c r="A48" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="C48" s="4">
-        <v>2550</v>
-      </c>
-      <c r="D48" s="4">
-        <v>6</v>
-      </c>
-      <c r="E48" s="3" t="s">
-        <v>330</v>
-      </c>
-      <c r="F48" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G48" s="5">
-        <v>25.5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
-      <c r="A49" s="3" t="s">
-        <v>331</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>332</v>
-      </c>
-      <c r="C49" s="4">
-        <v>4383</v>
-      </c>
-      <c r="D49" s="4">
-        <v>12</v>
-      </c>
-      <c r="E49" s="3" t="s">
-        <v>320</v>
-      </c>
-      <c r="F49" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G49" s="4">
-        <v>53</v>
-      </c>
+      <c r="A33" s="3"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="19.5">
+      <c r="A34" s="11" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>1127</v>
+      </c>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="11" t="s">
+        <v>1127</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>1127</v>
+      </c>
+      <c r="G34" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5968,7 +5612,7 @@
         <v>197.5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="3" t="s">
         <v>507</v>
       </c>
@@ -5991,7 +5635,7 @@
         <v>395</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="3" t="s">
         <v>510</v>
       </c>

</xml_diff>